<commit_message>
7/7 & 7/8 Sales and purchases
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{833467AF-3ECC-3047-86E9-0728060032EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C71B2464-DA28-2646-AE19-007737AB0544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="20" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2897" uniqueCount="1153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2912" uniqueCount="1158">
   <si>
     <t>Notes:</t>
   </si>
@@ -3471,18 +3471,12 @@
     <t>Bahuleyan</t>
   </si>
   <si>
-    <t>Shykaja Bank</t>
-  </si>
-  <si>
     <t>Indukala - XL, Shylaja - XXL</t>
   </si>
   <si>
     <t>Indukala - L, Shylaja - XXL</t>
   </si>
   <si>
-    <t>CHR-153 (XXL), CHR-155 (XXL), CHR-51(XXL)</t>
-  </si>
-  <si>
     <t>CHR-76 (XXL Plus white salwar) - 600 advance</t>
   </si>
   <si>
@@ -3501,29 +3495,50 @@
     <t>CHR-92 Jute Kurti &amp; CHR-157 2 piece cotton salwar</t>
   </si>
   <si>
-    <t>Shykaja Bank c/o</t>
-  </si>
-  <si>
     <t>CHR-87 Red Salwar with Elephant print, CHR-58 Wine Red Salwar</t>
   </si>
   <si>
+    <t>light green/maroon</t>
+  </si>
+  <si>
+    <t>Nishitha Friend - brown/maroon (1100), JIJI - Blue/maroon (1100)</t>
+  </si>
+  <si>
+    <t>JIJI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHR-203 kalyani Blue/maroon </t>
+  </si>
+  <si>
+    <t>Bank of baroda customer 2</t>
+  </si>
+  <si>
+    <t>Shylaja Bank</t>
+  </si>
+  <si>
+    <t>CHR-153 (XXL), CHR-155 (XXL), CHR-51(XXL) - 1000 advance</t>
+  </si>
+  <si>
+    <t>Sruthi (1300) - L, Bank of baroda customer - M</t>
+  </si>
+  <si>
     <t>Susmi (1200) - L
-Sreelakshmi (1000) - XL, Prema (1000) - XXL, Shylaja C/O - M</t>
-  </si>
-  <si>
-    <t>Sruthi (1300) - L, Shylaja c/o - size?</t>
-  </si>
-  <si>
-    <t>light green/maroon</t>
-  </si>
-  <si>
-    <t>Nishitha Friend - brown/maroon (1100), JIJI - Blue/maroon (1100)</t>
-  </si>
-  <si>
-    <t>JIJI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CHR-203 kalyani Blue/maroon </t>
+Sreelakshmi (1000) - XL, Prema (1000) - XXL, bank of baroda customer 2- M</t>
+  </si>
+  <si>
+    <t>Asha Sharath (Bulk Order)</t>
+  </si>
+  <si>
+    <t>Parrot Green Banarasi bulk order advance</t>
+  </si>
+  <si>
+    <t>Renju R S</t>
+  </si>
+  <si>
+    <t>CHR-187 - Banarasi Silk (Golden Yellow Blue)</t>
+  </si>
+  <si>
+    <t>Renju</t>
   </si>
 </sst>
 </file>
@@ -4403,7 +4418,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>267</c:v>
+                  <c:v>268</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>93</c:v>
@@ -4506,7 +4521,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>154</c:v>
+                  <c:v>153</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>55</c:v>
@@ -4839,7 +4854,7 @@
                   <c:v>58332</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>120406.43</c:v>
+                  <c:v>119515.43</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>590</c:v>
@@ -5172,7 +5187,7 @@
                   <c:v>99043</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>28882</c:v>
+                  <c:v>28944</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5332,7 +5347,7 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>19339</c:v>
+                  <c:v>23969</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5772,7 +5787,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-9543</c:v>
+                  <c:v>-4975</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6236,10 +6251,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>365</c:v>
+                  <c:v>366</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-272</c:v>
+                  <c:v>-273</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7396,7 +7411,7 @@
     <col min="4" max="4" width="30.1640625" style="6" customWidth="1"/>
     <col min="5" max="5" width="22.1640625" style="6" customWidth="1"/>
     <col min="6" max="6" width="31.1640625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="18.6640625" style="6" customWidth="1"/>
+    <col min="7" max="7" width="14.6640625" style="6" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="8.83203125" style="6"/>
   </cols>
   <sheetData>
@@ -7411,7 +7426,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>483029</v>
+        <v>483091</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7426,7 +7441,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>436807</v>
+        <v>442587</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7443,7 +7458,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>447837</v>
+        <v>452467</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7460,7 +7475,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-46222</v>
+        <v>-40504</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7495,7 +7510,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>62778.993333333347</v>
+        <v>62820.32666666666</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7505,7 +7520,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>5688.0033333333413</v>
+        <v>5667.3366666666552</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7515,7 +7530,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-68466.996666666659</v>
+        <v>-68487.663333333345</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7554,15 +7569,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>242092</v>
+        <v>242154</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>161009.66666666666</v>
+        <v>161030.33333333334</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>81082.333333333343</v>
+        <v>81123.666666666657</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7570,11 +7585,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>62778.993333333347</v>
+        <v>62820.32666666666</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹62,779</v>
+        <v>Receive ₹62,820</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7588,11 +7603,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>161009.66666666666</v>
+        <v>161030.33333333334</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>47327.333333333343</v>
+        <v>47306.666666666657</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7600,11 +7615,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>5688.0033333333413</v>
+        <v>5667.3366666666552</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹5,688</v>
+        <v>Receive ₹5,667</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7618,11 +7633,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>161009.66666666666</v>
+        <v>161030.33333333334</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-128409.66666666666</v>
+        <v>-128430.33333333334</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7630,11 +7645,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-68466.996666666659</v>
+        <v>-68487.663333333345</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹68,467</v>
+        <v>Pay ₹68,488</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7672,15 +7687,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>369653</v>
+        <v>375433</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>145631.45379999999</v>
+        <v>147558.50579999998</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>224021.54620000001</v>
+        <v>227874.49420000002</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7688,11 +7703,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>86711.520199999999</v>
+        <v>90564.468200000003</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹86,712</v>
+        <v>Pay ₹90,564</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7706,11 +7721,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>145544.09239999999</v>
+        <v>147469.9884</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-90920.092399999994</v>
+        <v>-92845.988400000002</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7718,11 +7733,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-19333.050399999993</v>
+        <v>-21258.946400000001</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹19,333</v>
+        <v>Receive ₹21,259</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7736,11 +7751,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>145631.45379999999</v>
+        <v>147558.50579999998</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-133101.45379999999</v>
+        <v>-135028.50579999998</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7748,11 +7763,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-67378.469799999977</v>
+        <v>-69305.521799999973</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹67,378</v>
+        <v>Receive ₹69,306</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7864,7 +7879,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46208</v>
+        <v>46211</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7873,14 +7888,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>483029</v>
+        <v>483091</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>436807</v>
+        <v>442587</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7889,14 +7904,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-46222</v>
+        <v>-40504</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>169707.63</v>
+        <v>168816.63</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7948,7 +7963,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>365</v>
+        <v>366</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7972,7 +7987,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>-272</v>
+        <v>-273</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8049,15 +8064,15 @@
       </c>
       <c r="B16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A16)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>28882</v>
+        <v>28944</v>
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$995,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$995)=$B$7)*Sales!$C$2:$C$995),0)</f>
-        <v>19339</v>
+        <v>23969</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-9543</v>
+        <v>-4975</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8168,11 +8183,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8199,7 +8214,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>120406.43</v>
+        <v>119515.43</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9590,10 +9605,18 @@
       </c>
     </row>
     <row r="93" spans="1:4" ht="15" customHeight="1">
-      <c r="A93" s="38"/>
-      <c r="B93" s="39"/>
-      <c r="C93" s="40"/>
-      <c r="D93" s="39"/>
+      <c r="A93" s="38">
+        <v>46210</v>
+      </c>
+      <c r="B93" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C93" s="40">
+        <v>62</v>
+      </c>
+      <c r="D93" s="39" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="94" spans="1:4" ht="15" customHeight="1">
       <c r="A94" s="35"/>
@@ -17877,15 +17900,19 @@
       <c r="C249" s="54">
         <v>1200</v>
       </c>
-      <c r="D249" s="53"/>
-      <c r="E249" s="53"/>
+      <c r="D249" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E249" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F249" s="56"/>
       <c r="G249" s="56"/>
       <c r="H249" s="57" t="s">
         <v>1086</v>
       </c>
       <c r="I249" s="53" t="s">
-        <v>356</v>
+        <v>148</v>
       </c>
     </row>
     <row r="250" spans="1:9" ht="14">
@@ -18174,7 +18201,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>356</v>
@@ -18235,7 +18262,7 @@
         <v>46206</v>
       </c>
       <c r="B264" s="49" t="s">
-        <v>1135</v>
+        <v>1149</v>
       </c>
       <c r="C264" s="50">
         <v>2500</v>
@@ -18249,7 +18276,7 @@
       <c r="F264" s="49"/>
       <c r="G264" s="49"/>
       <c r="H264" s="51" t="s">
-        <v>1138</v>
+        <v>1150</v>
       </c>
       <c r="I264" s="49" t="s">
         <v>356</v>
@@ -18260,7 +18287,7 @@
         <v>46206</v>
       </c>
       <c r="B265" s="53" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="C265" s="54">
         <v>1300</v>
@@ -18274,7 +18301,7 @@
       <c r="F265" s="56"/>
       <c r="G265" s="56"/>
       <c r="H265" s="57" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="I265" s="53" t="s">
         <v>356</v>
@@ -18299,7 +18326,7 @@
       <c r="F266" s="49"/>
       <c r="G266" s="49"/>
       <c r="H266" s="51" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="I266" s="49" t="s">
         <v>148</v>
@@ -18324,7 +18351,7 @@
       <c r="F267" s="56"/>
       <c r="G267" s="56"/>
       <c r="H267" s="57" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="I267" s="53" t="s">
         <v>148</v>
@@ -18335,17 +18362,17 @@
         <v>46208</v>
       </c>
       <c r="B268" s="49" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
       <c r="C268" s="50">
-        <v>2250</v>
+        <v>2300</v>
       </c>
       <c r="D268" s="49"/>
       <c r="E268" s="49"/>
       <c r="F268" s="49"/>
       <c r="G268" s="49"/>
       <c r="H268" s="51" t="s">
-        <v>1146</v>
+        <v>1143</v>
       </c>
       <c r="I268" s="49" t="s">
         <v>356</v>
@@ -18356,7 +18383,7 @@
         <v>46209</v>
       </c>
       <c r="B269" s="53" t="s">
-        <v>1151</v>
+        <v>1146</v>
       </c>
       <c r="C269" s="54">
         <v>1100</v>
@@ -18370,33 +18397,61 @@
       <c r="F269" s="56"/>
       <c r="G269" s="56"/>
       <c r="H269" s="57" t="s">
-        <v>1152</v>
+        <v>1147</v>
       </c>
       <c r="I269" s="53" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="270" spans="1:9">
-      <c r="A270" s="48"/>
-      <c r="B270" s="49"/>
-      <c r="C270" s="50"/>
-      <c r="D270" s="49"/>
-      <c r="E270" s="49"/>
+    <row r="270" spans="1:9" ht="14">
+      <c r="A270" s="48">
+        <v>46210</v>
+      </c>
+      <c r="B270" s="49" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C270" s="50">
+        <v>3200</v>
+      </c>
+      <c r="D270" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E270" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F270" s="49"/>
       <c r="G270" s="49"/>
-      <c r="H270" s="51"/>
-      <c r="I270" s="49"/>
-    </row>
-    <row r="271" spans="1:9">
-      <c r="A271" s="52"/>
-      <c r="B271" s="53"/>
-      <c r="C271" s="54"/>
-      <c r="D271" s="53"/>
-      <c r="E271" s="53"/>
+      <c r="H270" s="51" t="s">
+        <v>1154</v>
+      </c>
+      <c r="I270" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="271" spans="1:9" ht="14">
+      <c r="A271" s="52">
+        <v>46211</v>
+      </c>
+      <c r="B271" s="53" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C271" s="54">
+        <v>1380</v>
+      </c>
+      <c r="D271" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E271" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F271" s="56"/>
       <c r="G271" s="56"/>
-      <c r="H271" s="57"/>
-      <c r="I271" s="53"/>
+      <c r="H271" s="57" t="s">
+        <v>1156</v>
+      </c>
+      <c r="I271" s="53" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="272" spans="1:9">
       <c r="A272" s="48"/>
@@ -25251,14 +25306,14 @@
         <v>1145</v>
       </c>
       <c r="L59" s="66" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="M59" s="66"/>
       <c r="N59" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O59" s="66" t="s">
-        <v>621</v>
+        <v>229</v>
       </c>
       <c r="P59" s="66" t="s">
         <v>622</v>
@@ -26797,7 +26852,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="63" t="s">
-        <v>1147</v>
+        <v>1152</v>
       </c>
       <c r="M88" s="63"/>
       <c r="N88" s="63" t="s">
@@ -30955,7 +31010,7 @@
         <v>949</v>
       </c>
       <c r="L154" s="63" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="M154" s="63"/>
       <c r="N154" s="63" t="s">
@@ -31061,7 +31116,7 @@
         <v>1900</v>
       </c>
       <c r="L156" s="63" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="M156" s="63"/>
       <c r="N156" s="63" t="s">
@@ -32728,10 +32783,10 @@
         <v>1380</v>
       </c>
       <c r="F188" s="78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G188" s="78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H188" s="77">
         <f t="shared" si="12"/>
@@ -32743,16 +32798,18 @@
       </c>
       <c r="J188" s="77">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>891</v>
       </c>
       <c r="K188" s="77">
         <f t="shared" si="10"/>
-        <v>1782</v>
-      </c>
-      <c r="L188" s="63"/>
+        <v>891</v>
+      </c>
+      <c r="L188" s="63" t="s">
+        <v>1157</v>
+      </c>
       <c r="M188" s="63"/>
       <c r="N188" s="63" t="s">
-        <v>678</v>
+        <v>589</v>
       </c>
       <c r="O188" s="63"/>
       <c r="P188" s="63"/>
@@ -32800,7 +32857,7 @@
         <v>2673</v>
       </c>
       <c r="L189" s="66" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="M189" s="66"/>
       <c r="N189" s="66" t="s">
@@ -33554,14 +33611,14 @@
         <v>880</v>
       </c>
       <c r="L204" s="63" t="s">
-        <v>1150</v>
+        <v>1145</v>
       </c>
       <c r="M204" s="63"/>
       <c r="N204" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P204" s="58" t="s">
-        <v>1149</v>
+        <v>1144</v>
       </c>
       <c r="S204" s="58"/>
       <c r="T204" s="58"/>
@@ -38401,15 +38458,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>242092</v>
+        <v>242154</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>161009.66666666666</v>
+        <v>161030.33333333334</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>81082.333333333343</v>
+        <v>81123.666666666657</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38417,7 +38474,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>81082.333333333343</v>
+        <v>81123.666666666657</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -38425,7 +38482,7 @@
       </c>
       <c r="H8" s="85">
         <f>F8-G8</f>
-        <v>62778.993333333347</v>
+        <v>62820.32666666666</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -38438,11 +38495,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>161009.66666666666</v>
+        <v>161030.33333333334</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>47327.333333333343</v>
+        <v>47306.666666666657</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38450,7 +38507,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>47327.333333333343</v>
+        <v>47306.666666666657</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -38458,7 +38515,7 @@
       </c>
       <c r="H9" s="86">
         <f>F9-G9</f>
-        <v>5688.0033333333413</v>
+        <v>5667.3366666666552</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -38471,11 +38528,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>161009.66666666666</v>
+        <v>161030.33333333334</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-128409.66666666666</v>
+        <v>-128430.33333333334</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38483,7 +38540,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-128409.66666666666</v>
+        <v>-128430.33333333334</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -38491,7 +38548,7 @@
       </c>
       <c r="H10" s="85">
         <f>F10-G10</f>
-        <v>-68466.996666666659</v>
+        <v>-68487.663333333345</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">
@@ -38908,7 +38965,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>369653</v>
+        <v>375433</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -38916,11 +38973,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>145631.45379999999</v>
+        <v>147558.50579999998</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>224021.54620000001</v>
+        <v>227874.49420000002</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -38928,7 +38985,7 @@
       </c>
       <c r="G4" s="85">
         <f>E4+F4</f>
-        <v>86711.520199999999</v>
+        <v>90564.468200000003</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -38945,11 +39002,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>145544.09239999999</v>
+        <v>147469.9884</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-90920.092399999994</v>
+        <v>-92845.988400000002</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -38957,7 +39014,7 @@
       </c>
       <c r="G5" s="86">
         <f>E5+F5</f>
-        <v>-19333.050399999993</v>
+        <v>-21258.946400000001</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -38974,11 +39031,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>145631.45379999999</v>
+        <v>147558.50579999998</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-133101.45379999999</v>
+        <v>-135028.50579999998</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -38986,7 +39043,7 @@
       </c>
       <c r="G6" s="85">
         <f>E6+F6</f>
-        <v>-67378.469799999977</v>
+        <v>-69305.521799999973</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
7/9 komappas purchase 28130
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C71B2464-DA28-2646-AE19-007737AB0544}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3B6BE6-CBD6-3240-84CD-8630F131FFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2912" uniqueCount="1158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2914" uniqueCount="1158">
   <si>
     <t>Notes:</t>
   </si>
@@ -3385,9 +3385,6 @@
     <t>Cotton 2-piece set with blue floral prints-M (CHR-156), Short Kurti(CHR-151)-L, Dusty Rose Salwar(CHR-77)-L, Chanderis Silk Saree(Yellow-CHR-119), Matka - Lavender/Violet(CHR-174), Chikku Maroon new design(CHR-188)</t>
   </si>
   <si>
-    <t>peacock blue/navy, red/green, mustard/blue, golden yellow &amp; green triangle</t>
-  </si>
-  <si>
     <t>Dison Jose</t>
   </si>
   <si>
@@ -3483,9 +3480,6 @@
     <t>Bank of baroda customer</t>
   </si>
   <si>
-    <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim, Rust Orange/Coffee Brown - Nishida, Chikku Maroon(1200) - Nishida, Komalavalli - Red/green</t>
-  </si>
-  <si>
     <t>CHR-188 Red/green new banarasi</t>
   </si>
   <si>
@@ -3539,6 +3533,12 @@
   </si>
   <si>
     <t>Renju</t>
+  </si>
+  <si>
+    <t>mustard/blue, golden yellow &amp; green triangle</t>
+  </si>
+  <si>
+    <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim, Rust Orange/Coffee Brown - Nishida, Chikku Maroon(1200) - Nishida, Komalavalli - Red/green, peacock blue/navy - returned</t>
   </si>
 </sst>
 </file>
@@ -4521,7 +4521,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>153</c:v>
+                  <c:v>152</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>55</c:v>
@@ -4854,7 +4854,7 @@
                   <c:v>58332</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>119515.43</c:v>
+                  <c:v>118624.43</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>590</c:v>
@@ -5187,7 +5187,7 @@
                   <c:v>99043</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>28944</c:v>
+                  <c:v>57074</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5787,7 +5787,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-4975</c:v>
+                  <c:v>-33105</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6254,7 +6254,7 @@
                   <c:v>366</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-273</c:v>
+                  <c:v>-274</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7426,7 +7426,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>483091</v>
+        <v>511221</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7475,7 +7475,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-40504</v>
+        <v>-68634</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7510,7 +7510,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>62820.32666666666</v>
+        <v>53443.66</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7520,7 +7520,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>5667.3366666666552</v>
+        <v>24420.67</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7530,7 +7530,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-68487.663333333345</v>
+        <v>-77864.33</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7573,11 +7573,11 @@
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>161030.33333333334</v>
+        <v>170407</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>81123.666666666657</v>
+        <v>71747</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7585,11 +7585,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>62820.32666666666</v>
+        <v>53443.66</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹62,820</v>
+        <v>Receive ₹53,444</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7599,15 +7599,15 @@
       </c>
       <c r="B19" s="12">
         <f>PartnerShares!B9</f>
-        <v>208337</v>
+        <v>236467</v>
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>161030.33333333334</v>
+        <v>170407</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>47306.666666666657</v>
+        <v>66060</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7615,11 +7615,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>5667.3366666666552</v>
+        <v>24420.67</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹5,667</v>
+        <v>Receive ₹24,421</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>161030.33333333334</v>
+        <v>170407</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-128430.33333333334</v>
+        <v>-137807</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7645,11 +7645,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-68487.663333333345</v>
+        <v>-77864.33</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹68,488</v>
+        <v>Pay ₹77,864</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7879,7 +7879,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46211</v>
+        <v>46212</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7888,7 +7888,7 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>483091</v>
+        <v>511221</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
@@ -7904,14 +7904,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-40504</v>
+        <v>-68634</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>168816.63</v>
+        <v>167925.63</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7987,7 +7987,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>-273</v>
+        <v>-274</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8064,7 +8064,7 @@
       </c>
       <c r="B16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A16)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>28944</v>
+        <v>57074</v>
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$995,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$995)=$B$7)*Sales!$C$2:$C$995),0)</f>
@@ -8072,7 +8072,7 @@
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-4975</v>
+        <v>-33105</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8187,7 +8187,7 @@
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8214,7 +8214,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>119515.43</v>
+        <v>118624.43</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9587,7 +9587,7 @@
         <v>28526</v>
       </c>
       <c r="D91" s="39" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" customHeight="1">
@@ -9619,10 +9619,18 @@
       </c>
     </row>
     <row r="94" spans="1:4" ht="15" customHeight="1">
-      <c r="A94" s="35"/>
-      <c r="B94" s="36"/>
-      <c r="C94" s="37"/>
-      <c r="D94" s="36"/>
+      <c r="A94" s="35">
+        <v>46212</v>
+      </c>
+      <c r="B94" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C94" s="37">
+        <v>28130</v>
+      </c>
+      <c r="D94" s="36" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="95" spans="1:4" ht="15" customHeight="1">
       <c r="A95" s="38"/>
@@ -17941,7 +17949,7 @@
         <v>46201</v>
       </c>
       <c r="B251" s="53" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="C251" s="54">
         <v>1380</v>
@@ -18066,7 +18074,7 @@
         <v>46203</v>
       </c>
       <c r="B256" s="49" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="C256" s="50">
         <v>950</v>
@@ -18080,7 +18088,7 @@
       <c r="F256" s="49"/>
       <c r="G256" s="49"/>
       <c r="H256" s="51" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="I256" s="49" t="s">
         <v>148</v>
@@ -18091,7 +18099,7 @@
         <v>46204</v>
       </c>
       <c r="B257" s="53" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="C257" s="54">
         <v>699</v>
@@ -18105,7 +18113,7 @@
       <c r="F257" s="56"/>
       <c r="G257" s="56"/>
       <c r="H257" s="57" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="I257" s="53" t="s">
         <v>148</v>
@@ -18116,7 +18124,7 @@
         <v>46205</v>
       </c>
       <c r="B258" s="49" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="C258" s="50">
         <v>1500</v>
@@ -18130,7 +18138,7 @@
       <c r="F258" s="49"/>
       <c r="G258" s="49"/>
       <c r="H258" s="51" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="I258" s="49" t="s">
         <v>148</v>
@@ -18141,7 +18149,7 @@
         <v>46205</v>
       </c>
       <c r="B259" s="53" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="C259" s="54">
         <v>1200</v>
@@ -18155,7 +18163,7 @@
       <c r="F259" s="56"/>
       <c r="G259" s="56"/>
       <c r="H259" s="57" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="I259" s="53" t="s">
         <v>148</v>
@@ -18166,7 +18174,7 @@
         <v>46205</v>
       </c>
       <c r="B260" s="49" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C260" s="50">
         <v>1500</v>
@@ -18180,7 +18188,7 @@
       <c r="F260" s="49"/>
       <c r="G260" s="49"/>
       <c r="H260" s="51" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="I260" s="49" t="s">
         <v>148</v>
@@ -18191,7 +18199,7 @@
         <v>46205</v>
       </c>
       <c r="B261" s="53" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="C261" s="54">
         <v>1900</v>
@@ -18201,7 +18209,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>356</v>
@@ -18212,7 +18220,7 @@
         <v>46206</v>
       </c>
       <c r="B262" s="49" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="C262" s="50">
         <v>1380</v>
@@ -18237,7 +18245,7 @@
         <v>46206</v>
       </c>
       <c r="B263" s="53" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="C263" s="54">
         <v>1380</v>
@@ -18262,7 +18270,7 @@
         <v>46206</v>
       </c>
       <c r="B264" s="49" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="C264" s="50">
         <v>2500</v>
@@ -18276,7 +18284,7 @@
       <c r="F264" s="49"/>
       <c r="G264" s="49"/>
       <c r="H264" s="51" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="I264" s="49" t="s">
         <v>356</v>
@@ -18287,7 +18295,7 @@
         <v>46206</v>
       </c>
       <c r="B265" s="53" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="C265" s="54">
         <v>1300</v>
@@ -18301,7 +18309,7 @@
       <c r="F265" s="56"/>
       <c r="G265" s="56"/>
       <c r="H265" s="57" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="I265" s="53" t="s">
         <v>356</v>
@@ -18312,7 +18320,7 @@
         <v>46206</v>
       </c>
       <c r="B266" s="49" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C266" s="50">
         <v>1380</v>
@@ -18326,7 +18334,7 @@
       <c r="F266" s="49"/>
       <c r="G266" s="49"/>
       <c r="H266" s="51" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="I266" s="49" t="s">
         <v>148</v>
@@ -18351,7 +18359,7 @@
       <c r="F267" s="56"/>
       <c r="G267" s="56"/>
       <c r="H267" s="57" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="I267" s="53" t="s">
         <v>148</v>
@@ -18362,7 +18370,7 @@
         <v>46208</v>
       </c>
       <c r="B268" s="49" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="C268" s="50">
         <v>2300</v>
@@ -18372,7 +18380,7 @@
       <c r="F268" s="49"/>
       <c r="G268" s="49"/>
       <c r="H268" s="51" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="I268" s="49" t="s">
         <v>356</v>
@@ -18383,7 +18391,7 @@
         <v>46209</v>
       </c>
       <c r="B269" s="53" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="C269" s="54">
         <v>1100</v>
@@ -18397,7 +18405,7 @@
       <c r="F269" s="56"/>
       <c r="G269" s="56"/>
       <c r="H269" s="57" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="I269" s="53" t="s">
         <v>148</v>
@@ -18408,7 +18416,7 @@
         <v>46210</v>
       </c>
       <c r="B270" s="49" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="C270" s="50">
         <v>3200</v>
@@ -18422,7 +18430,7 @@
       <c r="F270" s="49"/>
       <c r="G270" s="49"/>
       <c r="H270" s="51" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="I270" s="49" t="s">
         <v>148</v>
@@ -18433,7 +18441,7 @@
         <v>46211</v>
       </c>
       <c r="B271" s="53" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="C271" s="54">
         <v>1380</v>
@@ -18447,7 +18455,7 @@
       <c r="F271" s="56"/>
       <c r="G271" s="56"/>
       <c r="H271" s="57" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="I271" s="53" t="s">
         <v>148</v>
@@ -25306,7 +25314,7 @@
         <v>1145</v>
       </c>
       <c r="L59" s="66" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="M59" s="66"/>
       <c r="N59" s="66" t="s">
@@ -26852,7 +26860,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="63" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="M88" s="63"/>
       <c r="N88" s="63" t="s">
@@ -27112,7 +27120,7 @@
         <v>0</v>
       </c>
       <c r="L93" s="66" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="M93" s="66"/>
       <c r="N93" s="63" t="s">
@@ -31010,14 +31018,14 @@
         <v>949</v>
       </c>
       <c r="L154" s="63" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="M154" s="63"/>
       <c r="N154" s="63" t="s">
         <v>589</v>
       </c>
       <c r="O154" s="63" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="P154" s="63"/>
       <c r="Q154" s="63"/>
@@ -31116,7 +31124,7 @@
         <v>1900</v>
       </c>
       <c r="L156" s="63" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="M156" s="63"/>
       <c r="N156" s="63" t="s">
@@ -31646,7 +31654,7 @@
         <v>1212</v>
       </c>
       <c r="L166" s="63" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="M166" s="63"/>
       <c r="N166" s="63" t="s">
@@ -31654,7 +31662,7 @@
       </c>
       <c r="O166" s="63"/>
       <c r="P166" s="63" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="Q166" s="63"/>
       <c r="R166" s="63"/>
@@ -32122,7 +32130,7 @@
         <v>3491.25</v>
       </c>
       <c r="L175" s="66" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="M175" s="66"/>
       <c r="N175" s="66" t="s">
@@ -32130,7 +32138,7 @@
       </c>
       <c r="O175" s="66"/>
       <c r="P175" s="66" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="Q175" s="66"/>
       <c r="R175" s="66"/>
@@ -32442,14 +32450,14 @@
         <v>3057</v>
       </c>
       <c r="L181" s="66" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="M181" s="66"/>
       <c r="N181" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O181" s="66" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="P181" s="66" t="s">
         <v>960</v>
@@ -32549,7 +32557,7 @@
         <v>2933</v>
       </c>
       <c r="L183" s="66" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="M183" s="66"/>
       <c r="N183" s="66" t="s">
@@ -32601,7 +32609,7 @@
         <v>3564</v>
       </c>
       <c r="L184" s="63" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="M184" s="63"/>
       <c r="N184" s="63" t="s">
@@ -32805,7 +32813,7 @@
         <v>891</v>
       </c>
       <c r="L188" s="63" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="M188" s="63"/>
       <c r="N188" s="63" t="s">
@@ -32818,7 +32826,7 @@
       <c r="S188" s="63"/>
       <c r="T188" s="63"/>
     </row>
-    <row r="189" spans="1:20" ht="30" customHeight="1">
+    <row r="189" spans="1:20" ht="52" customHeight="1">
       <c r="A189" s="66" t="s">
         <v>976</v>
       </c>
@@ -32838,11 +32846,11 @@
         <v>5</v>
       </c>
       <c r="G189" s="76">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H189" s="75">
         <f t="shared" si="12"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I189" s="75">
         <f>IF(D189&lt;&gt;"",D189,IFERROR(E189/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -32854,10 +32862,10 @@
       </c>
       <c r="K189" s="75">
         <f t="shared" si="10"/>
-        <v>2673</v>
+        <v>1782</v>
       </c>
       <c r="L189" s="66" t="s">
-        <v>1139</v>
+        <v>1157</v>
       </c>
       <c r="M189" s="66"/>
       <c r="N189" s="66" t="s">
@@ -32865,7 +32873,7 @@
       </c>
       <c r="O189" s="66"/>
       <c r="P189" s="66" t="s">
-        <v>1107</v>
+        <v>1156</v>
       </c>
       <c r="Q189" s="66"/>
       <c r="R189" s="66"/>
@@ -33509,14 +33517,14 @@
         <v>3760</v>
       </c>
       <c r="L202" s="63" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="M202" s="63"/>
       <c r="N202" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="58" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="S202" s="58"/>
       <c r="T202" s="58"/>
@@ -33611,14 +33619,14 @@
         <v>880</v>
       </c>
       <c r="L204" s="63" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="M204" s="63"/>
       <c r="N204" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P204" s="58" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="S204" s="58"/>
       <c r="T204" s="58"/>
@@ -33977,7 +33985,7 @@
         <v>1043</v>
       </c>
       <c r="B212" s="66" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="C212" s="66" t="s">
         <v>95</v>
@@ -38462,11 +38470,11 @@
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>161030.33333333334</v>
+        <v>170407</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>81123.666666666657</v>
+        <v>71747</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38474,7 +38482,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>81123.666666666657</v>
+        <v>71747</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -38482,7 +38490,7 @@
       </c>
       <c r="H8" s="85">
         <f>F8-G8</f>
-        <v>62820.32666666666</v>
+        <v>53443.66</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -38491,15 +38499,15 @@
       </c>
       <c r="B9" s="11">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A9,Purchases!$C:$C),0)</f>
-        <v>208337</v>
+        <v>236467</v>
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>161030.33333333334</v>
+        <v>170407</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>47306.666666666657</v>
+        <v>66060</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38507,7 +38515,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>47306.666666666657</v>
+        <v>66060</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -38515,7 +38523,7 @@
       </c>
       <c r="H9" s="86">
         <f>F9-G9</f>
-        <v>5667.3366666666552</v>
+        <v>24420.67</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -38528,11 +38536,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>161030.33333333334</v>
+        <v>170407</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-128430.33333333334</v>
+        <v>-137807</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38540,7 +38548,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-128430.33333333334</v>
+        <v>-137807</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -38548,7 +38556,7 @@
       </c>
       <c r="H10" s="85">
         <f>F10-G10</f>
-        <v>-68487.663333333345</v>
+        <v>-77864.33</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
7/11 & 7/12 Sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3B6BE6-CBD6-3240-84CD-8630F131FFB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C95EFE2-6570-164C-897F-14767FEE7873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2914" uniqueCount="1158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2930" uniqueCount="1161">
   <si>
     <t>Notes:</t>
   </si>
@@ -2704,9 +2704,6 @@
     <t>Dark brown embroidered cotton 3-piece salwar set</t>
   </si>
   <si>
-    <t>M, XL, XXL</t>
-  </si>
-  <si>
     <t>CHR-155</t>
   </si>
   <si>
@@ -3404,9 +3401,6 @@
   </si>
   <si>
     <t>CHR-182 (Yellow Linen Saree with Lotus)</t>
-  </si>
-  <si>
-    <t>Irene</t>
   </si>
   <si>
     <t>Shinoob School</t>
@@ -3459,9 +3453,6 @@
     <t>Sourabhya (XL - 580), Lakshmi - L, Jisha bank (XXL)</t>
   </si>
   <si>
-    <t>Sheeba George, Soji Thomas, Jessy Joseph, Jeeja Anil ,Sanam, Geetha, Sushama Bhaskar, Divya Jacob, Baby Johny, Jayasree, Navya, Bindu Saji, Vanajakshi, Dison Jose, Akshitha, Bahuleyan</t>
-  </si>
-  <si>
     <t>Akshitha</t>
   </si>
   <si>
@@ -3474,9 +3465,6 @@
     <t>Indukala - L, Shylaja - XXL</t>
   </si>
   <si>
-    <t>CHR-76 (XXL Plus white salwar) - 600 advance</t>
-  </si>
-  <si>
     <t>Bank of baroda customer</t>
   </si>
   <si>
@@ -3484,12 +3472,6 @@
   </si>
   <si>
     <t>CHR-195 Purple Cotton Saree</t>
-  </si>
-  <si>
-    <t>CHR-92 Jute Kurti &amp; CHR-157 2 piece cotton salwar</t>
-  </si>
-  <si>
-    <t>CHR-87 Red Salwar with Elephant print, CHR-58 Wine Red Salwar</t>
   </si>
   <si>
     <t>light green/maroon</t>
@@ -3532,13 +3514,40 @@
     <t>CHR-187 - Banarasi Silk (Golden Yellow Blue)</t>
   </si>
   <si>
-    <t>Renju</t>
-  </si>
-  <si>
     <t>mustard/blue, golden yellow &amp; green triangle</t>
   </si>
   <si>
     <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim, Rust Orange/Coffee Brown - Nishida, Chikku Maroon(1200) - Nishida, Komalavalli - Red/green, peacock blue/navy - returned</t>
+  </si>
+  <si>
+    <t>CHR-76 (XXL Plus white salwar) - 1100 advance, 200 balance</t>
+  </si>
+  <si>
+    <t>CHR-87 Red Salwar with Elephant print, CHR-58 Wine Red Salwar (1000 advance, 1350 balance)</t>
+  </si>
+  <si>
+    <t>CHR-92 Jute Kurti &amp; CHR-157 2 piece cotton salwar, Banarasi golden yellow blue</t>
+  </si>
+  <si>
+    <t>Renju, Jisha bank</t>
+  </si>
+  <si>
+    <t>Urmila</t>
+  </si>
+  <si>
+    <t>Sheeba George, Soji Thomas, Jessy Joseph, Jeeja Anil ,Sanam, Geetha, Sushama Bhaskar, Divya Jacob, Baby Johny, Jayasree, Navya, Bindu Saji, Vanajakshi, Dison Jose, Akshitha, Bahuleyan, Urmila</t>
+  </si>
+  <si>
+    <t>Preeha Rajeevan</t>
+  </si>
+  <si>
+    <t>Irene, Preetha Rajeevan</t>
+  </si>
+  <si>
+    <t>Chithra - XL, Shanu - XXL (1350)</t>
+  </si>
+  <si>
+    <t>CHR-154 Dark Brown Salwar with mirrion work - XL</t>
   </si>
 </sst>
 </file>
@@ -4418,10 +4427,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>268</c:v>
+                  <c:v>271</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>93</c:v>
+                  <c:v>95</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -4521,10 +4530,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>152</c:v>
+                  <c:v>149</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>55</c:v>
+                  <c:v>53</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>2</c:v>
@@ -4851,10 +4860,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>58332</c:v>
+                  <c:v>56434</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>118624.43</c:v>
+                  <c:v>116423.43</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>590</c:v>
@@ -5347,7 +5356,7 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>23969</c:v>
+                  <c:v>27448</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5787,7 +5796,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-33105</c:v>
+                  <c:v>-29626</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6251,10 +6260,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>366</c:v>
+                  <c:v>371</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-274</c:v>
+                  <c:v>-279</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7441,7 +7450,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>442587</v>
+        <v>446016</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7458,7 +7467,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>452467</v>
+        <v>455946</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7475,7 +7484,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-68634</v>
+        <v>-65205</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7687,15 +7696,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>375433</v>
+        <v>378862</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>147558.50579999998</v>
+        <v>148701.73439999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>227874.49420000002</v>
+        <v>230160.26560000001</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7703,11 +7712,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>90564.468200000003</v>
+        <v>92850.239600000001</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹90,564</v>
+        <v>Pay ₹92,850</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7721,11 +7730,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>147469.9884</v>
+        <v>148612.5312</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-92845.988400000002</v>
+        <v>-93988.531199999998</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7733,11 +7742,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-21258.946400000001</v>
+        <v>-22401.489199999996</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹21,259</v>
+        <v>Receive ₹22,401</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7751,11 +7760,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>147558.50579999998</v>
+        <v>148701.73439999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-135028.50579999998</v>
+        <v>-136171.73439999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7763,11 +7772,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-69305.521799999973</v>
+        <v>-70448.750399999975</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹69,306</v>
+        <v>Receive ₹70,449</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7879,7 +7888,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46212</v>
+        <v>46215</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7895,7 +7904,7 @@
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>442587</v>
+        <v>446016</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7904,14 +7913,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-68634</v>
+        <v>-65205</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>167925.63</v>
+        <v>163826.63</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7963,7 +7972,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>366</v>
+        <v>371</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7987,7 +7996,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>-274</v>
+        <v>-279</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8068,11 +8077,11 @@
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$995,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$995)=$B$7)*Sales!$C$2:$C$995),0)</f>
-        <v>23969</v>
+        <v>27448</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-33105</v>
+        <v>-29626</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8183,18 +8192,18 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
       </c>
       <c r="K47" s="31">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$477=J47)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>58332</v>
+        <v>56434</v>
       </c>
     </row>
     <row r="48" spans="6:11" ht="15" customHeight="1">
@@ -8203,18 +8212,18 @@
       </c>
       <c r="G48" s="30">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!F:F)</f>
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H48" s="30">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="J48" s="30" t="s">
         <v>95</v>
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>118624.43</v>
+        <v>116423.43</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9587,7 +9596,7 @@
         <v>28526</v>
       </c>
       <c r="D91" s="39" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" customHeight="1">
@@ -17092,7 +17101,7 @@
       <c r="F216" s="56"/>
       <c r="G216" s="56"/>
       <c r="H216" s="57" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="I216" s="53" t="s">
         <v>148</v>
@@ -17917,7 +17926,7 @@
       <c r="F249" s="56"/>
       <c r="G249" s="56"/>
       <c r="H249" s="57" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="I249" s="53" t="s">
         <v>148</v>
@@ -17938,7 +17947,7 @@
       <c r="F250" s="49"/>
       <c r="G250" s="49"/>
       <c r="H250" s="51" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="I250" s="49" t="s">
         <v>356</v>
@@ -17949,7 +17958,7 @@
         <v>46201</v>
       </c>
       <c r="B251" s="53" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="C251" s="54">
         <v>1380</v>
@@ -17974,7 +17983,7 @@
         <v>46201</v>
       </c>
       <c r="B252" s="49" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="C252" s="50">
         <v>699</v>
@@ -17988,7 +17997,7 @@
       <c r="F252" s="49"/>
       <c r="G252" s="49"/>
       <c r="H252" s="51" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="I252" s="49" t="s">
         <v>148</v>
@@ -17999,7 +18008,7 @@
         <v>46201</v>
       </c>
       <c r="B253" s="53" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="C253" s="54">
         <v>699</v>
@@ -18013,7 +18022,7 @@
       <c r="F253" s="56"/>
       <c r="G253" s="56"/>
       <c r="H253" s="57" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="I253" s="53" t="s">
         <v>148</v>
@@ -18024,7 +18033,7 @@
         <v>46201</v>
       </c>
       <c r="B254" s="49" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="C254" s="50">
         <v>699</v>
@@ -18038,7 +18047,7 @@
       <c r="F254" s="49"/>
       <c r="G254" s="49"/>
       <c r="H254" s="51" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="I254" s="49" t="s">
         <v>148</v>
@@ -18063,7 +18072,7 @@
       <c r="F255" s="56"/>
       <c r="G255" s="56"/>
       <c r="H255" s="57" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="I255" s="53" t="s">
         <v>148</v>
@@ -18074,7 +18083,7 @@
         <v>46203</v>
       </c>
       <c r="B256" s="49" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="C256" s="50">
         <v>950</v>
@@ -18088,7 +18097,7 @@
       <c r="F256" s="49"/>
       <c r="G256" s="49"/>
       <c r="H256" s="51" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="I256" s="49" t="s">
         <v>148</v>
@@ -18099,7 +18108,7 @@
         <v>46204</v>
       </c>
       <c r="B257" s="53" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="C257" s="54">
         <v>699</v>
@@ -18113,7 +18122,7 @@
       <c r="F257" s="56"/>
       <c r="G257" s="56"/>
       <c r="H257" s="57" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="I257" s="53" t="s">
         <v>148</v>
@@ -18124,7 +18133,7 @@
         <v>46205</v>
       </c>
       <c r="B258" s="49" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="C258" s="50">
         <v>1500</v>
@@ -18138,7 +18147,7 @@
       <c r="F258" s="49"/>
       <c r="G258" s="49"/>
       <c r="H258" s="51" t="s">
-        <v>1116</v>
+        <v>1114</v>
       </c>
       <c r="I258" s="49" t="s">
         <v>148</v>
@@ -18149,7 +18158,7 @@
         <v>46205</v>
       </c>
       <c r="B259" s="53" t="s">
-        <v>1115</v>
+        <v>1113</v>
       </c>
       <c r="C259" s="54">
         <v>1200</v>
@@ -18163,7 +18172,7 @@
       <c r="F259" s="56"/>
       <c r="G259" s="56"/>
       <c r="H259" s="57" t="s">
-        <v>1119</v>
+        <v>1117</v>
       </c>
       <c r="I259" s="53" t="s">
         <v>148</v>
@@ -18174,7 +18183,7 @@
         <v>46205</v>
       </c>
       <c r="B260" s="49" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="C260" s="50">
         <v>1500</v>
@@ -18188,18 +18197,18 @@
       <c r="F260" s="49"/>
       <c r="G260" s="49"/>
       <c r="H260" s="51" t="s">
-        <v>1120</v>
+        <v>1118</v>
       </c>
       <c r="I260" s="49" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="14">
+    <row r="261" spans="1:9" ht="28">
       <c r="A261" s="52">
         <v>46205</v>
       </c>
       <c r="B261" s="53" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="C261" s="54">
         <v>1900</v>
@@ -18209,7 +18218,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1140</v>
+        <v>1153</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>356</v>
@@ -18220,7 +18229,7 @@
         <v>46206</v>
       </c>
       <c r="B262" s="49" t="s">
-        <v>1132</v>
+        <v>1129</v>
       </c>
       <c r="C262" s="50">
         <v>1380</v>
@@ -18245,7 +18254,7 @@
         <v>46206</v>
       </c>
       <c r="B263" s="53" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="C263" s="54">
         <v>1380</v>
@@ -18270,7 +18279,7 @@
         <v>46206</v>
       </c>
       <c r="B264" s="49" t="s">
-        <v>1147</v>
+        <v>1141</v>
       </c>
       <c r="C264" s="50">
         <v>2500</v>
@@ -18284,7 +18293,7 @@
       <c r="F264" s="49"/>
       <c r="G264" s="49"/>
       <c r="H264" s="51" t="s">
-        <v>1148</v>
+        <v>1142</v>
       </c>
       <c r="I264" s="49" t="s">
         <v>356</v>
@@ -18295,7 +18304,7 @@
         <v>46206</v>
       </c>
       <c r="B265" s="53" t="s">
-        <v>1137</v>
+        <v>1133</v>
       </c>
       <c r="C265" s="54">
         <v>1300</v>
@@ -18309,7 +18318,7 @@
       <c r="F265" s="56"/>
       <c r="G265" s="56"/>
       <c r="H265" s="57" t="s">
-        <v>1136</v>
+        <v>1151</v>
       </c>
       <c r="I265" s="53" t="s">
         <v>356</v>
@@ -18320,7 +18329,7 @@
         <v>46206</v>
       </c>
       <c r="B266" s="49" t="s">
-        <v>1121</v>
+        <v>1119</v>
       </c>
       <c r="C266" s="50">
         <v>1380</v>
@@ -18334,7 +18343,7 @@
       <c r="F266" s="49"/>
       <c r="G266" s="49"/>
       <c r="H266" s="51" t="s">
-        <v>1138</v>
+        <v>1134</v>
       </c>
       <c r="I266" s="49" t="s">
         <v>148</v>
@@ -18359,7 +18368,7 @@
       <c r="F267" s="56"/>
       <c r="G267" s="56"/>
       <c r="H267" s="57" t="s">
-        <v>1139</v>
+        <v>1135</v>
       </c>
       <c r="I267" s="53" t="s">
         <v>148</v>
@@ -18370,17 +18379,17 @@
         <v>46208</v>
       </c>
       <c r="B268" s="49" t="s">
-        <v>1146</v>
+        <v>1140</v>
       </c>
       <c r="C268" s="50">
-        <v>2300</v>
+        <v>2350</v>
       </c>
       <c r="D268" s="49"/>
       <c r="E268" s="49"/>
       <c r="F268" s="49"/>
       <c r="G268" s="49"/>
       <c r="H268" s="51" t="s">
-        <v>1141</v>
+        <v>1152</v>
       </c>
       <c r="I268" s="49" t="s">
         <v>356</v>
@@ -18391,7 +18400,7 @@
         <v>46209</v>
       </c>
       <c r="B269" s="53" t="s">
-        <v>1144</v>
+        <v>1138</v>
       </c>
       <c r="C269" s="54">
         <v>1100</v>
@@ -18405,7 +18414,7 @@
       <c r="F269" s="56"/>
       <c r="G269" s="56"/>
       <c r="H269" s="57" t="s">
-        <v>1145</v>
+        <v>1139</v>
       </c>
       <c r="I269" s="53" t="s">
         <v>148</v>
@@ -18416,7 +18425,7 @@
         <v>46210</v>
       </c>
       <c r="B270" s="49" t="s">
-        <v>1151</v>
+        <v>1145</v>
       </c>
       <c r="C270" s="50">
         <v>3200</v>
@@ -18430,7 +18439,7 @@
       <c r="F270" s="49"/>
       <c r="G270" s="49"/>
       <c r="H270" s="51" t="s">
-        <v>1152</v>
+        <v>1146</v>
       </c>
       <c r="I270" s="49" t="s">
         <v>148</v>
@@ -18441,7 +18450,7 @@
         <v>46211</v>
       </c>
       <c r="B271" s="53" t="s">
-        <v>1153</v>
+        <v>1147</v>
       </c>
       <c r="C271" s="54">
         <v>1380</v>
@@ -18455,44 +18464,86 @@
       <c r="F271" s="56"/>
       <c r="G271" s="56"/>
       <c r="H271" s="57" t="s">
-        <v>1154</v>
+        <v>1148</v>
       </c>
       <c r="I271" s="53" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="272" spans="1:9">
-      <c r="A272" s="48"/>
-      <c r="B272" s="49"/>
-      <c r="C272" s="50"/>
-      <c r="D272" s="49"/>
-      <c r="E272" s="49"/>
+    <row r="272" spans="1:9" ht="14">
+      <c r="A272" s="48">
+        <v>46215</v>
+      </c>
+      <c r="B272" s="49" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C272" s="50">
+        <v>1380</v>
+      </c>
+      <c r="D272" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E272" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F272" s="49"/>
       <c r="G272" s="49"/>
-      <c r="H272" s="51"/>
-      <c r="I272" s="49"/>
-    </row>
-    <row r="273" spans="1:9">
-      <c r="A273" s="52"/>
-      <c r="B273" s="53"/>
-      <c r="C273" s="54"/>
-      <c r="D273" s="53"/>
-      <c r="E273" s="53"/>
+      <c r="H272" s="51" t="s">
+        <v>366</v>
+      </c>
+      <c r="I272" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="273" spans="1:9" ht="14">
+      <c r="A273" s="52">
+        <v>46215</v>
+      </c>
+      <c r="B273" s="53" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C273" s="54">
+        <v>699</v>
+      </c>
+      <c r="D273" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E273" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F273" s="56"/>
       <c r="G273" s="56"/>
-      <c r="H273" s="57"/>
-      <c r="I273" s="53"/>
-    </row>
-    <row r="274" spans="1:9">
-      <c r="A274" s="48"/>
-      <c r="B274" s="49"/>
-      <c r="C274" s="50"/>
-      <c r="D274" s="49"/>
-      <c r="E274" s="49"/>
+      <c r="H273" s="57" t="s">
+        <v>1112</v>
+      </c>
+      <c r="I273" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="274" spans="1:9" ht="14">
+      <c r="A274" s="48">
+        <v>46215</v>
+      </c>
+      <c r="B274" s="49" t="s">
+        <v>197</v>
+      </c>
+      <c r="C274" s="50">
+        <v>1350</v>
+      </c>
+      <c r="D274" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E274" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F274" s="49"/>
       <c r="G274" s="49"/>
-      <c r="H274" s="51"/>
-      <c r="I274" s="49"/>
+      <c r="H274" s="51" t="s">
+        <v>1160</v>
+      </c>
+      <c r="I274" s="49" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="275" spans="1:9">
       <c r="A275" s="52"/>
@@ -25314,7 +25365,7 @@
         <v>1145</v>
       </c>
       <c r="L59" s="66" t="s">
-        <v>1149</v>
+        <v>1143</v>
       </c>
       <c r="M59" s="66"/>
       <c r="N59" s="66" t="s">
@@ -26860,7 +26911,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="63" t="s">
-        <v>1150</v>
+        <v>1144</v>
       </c>
       <c r="M88" s="63"/>
       <c r="N88" s="63" t="s">
@@ -27120,7 +27171,7 @@
         <v>0</v>
       </c>
       <c r="L93" s="66" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="M93" s="66"/>
       <c r="N93" s="63" t="s">
@@ -28554,7 +28605,7 @@
         <v>1256.859999999999</v>
       </c>
       <c r="L120" s="63" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="M120" s="63" t="s">
         <v>49</v>
@@ -28564,7 +28615,7 @@
       </c>
       <c r="O120" s="63"/>
       <c r="P120" s="63" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="Q120" s="63"/>
       <c r="R120" s="63"/>
@@ -29662,7 +29713,7 @@
         <v>0</v>
       </c>
       <c r="L128" s="63" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="M128" s="63"/>
       <c r="N128" s="63" t="s">
@@ -30644,7 +30695,7 @@
         <v>1438</v>
       </c>
       <c r="L147" s="66" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="M147" s="66"/>
       <c r="N147" s="66" t="s">
@@ -30652,7 +30703,7 @@
       </c>
       <c r="O147" s="66"/>
       <c r="P147" s="66" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="Q147" s="66"/>
       <c r="R147" s="66"/>
@@ -31018,14 +31069,14 @@
         <v>949</v>
       </c>
       <c r="L154" s="63" t="s">
-        <v>1134</v>
+        <v>1131</v>
       </c>
       <c r="M154" s="63"/>
       <c r="N154" s="63" t="s">
         <v>589</v>
       </c>
       <c r="O154" s="63" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="P154" s="63"/>
       <c r="Q154" s="63"/>
@@ -31050,10 +31101,10 @@
         <v>1450</v>
       </c>
       <c r="F155" s="76">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G155" s="76">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H155" s="75">
         <f t="shared" si="8"/>
@@ -31065,19 +31116,21 @@
       </c>
       <c r="J155" s="75">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>1898</v>
       </c>
       <c r="K155" s="75">
         <f t="shared" si="10"/>
-        <v>2847</v>
-      </c>
-      <c r="L155" s="66"/>
+        <v>949</v>
+      </c>
+      <c r="L155" s="66" t="s">
+        <v>1159</v>
+      </c>
       <c r="M155" s="66"/>
       <c r="N155" s="66" t="s">
-        <v>678</v>
+        <v>589</v>
       </c>
       <c r="O155" s="66" t="s">
-        <v>881</v>
+        <v>1127</v>
       </c>
       <c r="P155" s="66"/>
       <c r="Q155" s="66"/>
@@ -31087,10 +31140,10 @@
     </row>
     <row r="156" spans="1:20" ht="15" customHeight="1">
       <c r="A156" s="63" t="s">
+        <v>881</v>
+      </c>
+      <c r="B156" s="63" t="s">
         <v>882</v>
-      </c>
-      <c r="B156" s="63" t="s">
-        <v>883</v>
       </c>
       <c r="C156" s="63" t="s">
         <v>96</v>
@@ -31124,7 +31177,7 @@
         <v>1900</v>
       </c>
       <c r="L156" s="63" t="s">
-        <v>1135</v>
+        <v>1132</v>
       </c>
       <c r="M156" s="63"/>
       <c r="N156" s="63" t="s">
@@ -31141,10 +31194,10 @@
     </row>
     <row r="157" spans="1:20" ht="15" customHeight="1">
       <c r="A157" s="66" t="s">
+        <v>883</v>
+      </c>
+      <c r="B157" s="66" t="s">
         <v>884</v>
-      </c>
-      <c r="B157" s="66" t="s">
-        <v>885</v>
       </c>
       <c r="C157" s="66" t="s">
         <v>96</v>
@@ -31178,7 +31231,7 @@
         <v>1050</v>
       </c>
       <c r="L157" s="66" t="s">
-        <v>886</v>
+        <v>885</v>
       </c>
       <c r="M157" s="66"/>
       <c r="N157" s="66" t="s">
@@ -31195,10 +31248,10 @@
     </row>
     <row r="158" spans="1:20" ht="15" customHeight="1">
       <c r="A158" s="63" t="s">
+        <v>886</v>
+      </c>
+      <c r="B158" s="63" t="s">
         <v>887</v>
-      </c>
-      <c r="B158" s="63" t="s">
-        <v>888</v>
       </c>
       <c r="C158" s="63" t="s">
         <v>96</v>
@@ -31232,14 +31285,14 @@
         <v>3356</v>
       </c>
       <c r="L158" s="63" t="s">
-        <v>889</v>
+        <v>888</v>
       </c>
       <c r="M158" s="63"/>
       <c r="N158" s="63" t="s">
         <v>678</v>
       </c>
       <c r="O158" s="63" t="s">
-        <v>890</v>
+        <v>889</v>
       </c>
       <c r="P158" s="63"/>
       <c r="Q158" s="63"/>
@@ -31249,10 +31302,10 @@
     </row>
     <row r="159" spans="1:20" ht="15" customHeight="1">
       <c r="A159" s="66" t="s">
+        <v>890</v>
+      </c>
+      <c r="B159" s="66" t="s">
         <v>891</v>
-      </c>
-      <c r="B159" s="66" t="s">
-        <v>892</v>
       </c>
       <c r="C159" s="66" t="s">
         <v>96</v>
@@ -31286,14 +31339,14 @@
         <v>2517</v>
       </c>
       <c r="L159" s="66" t="s">
-        <v>893</v>
+        <v>892</v>
       </c>
       <c r="M159" s="66"/>
       <c r="N159" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O159" s="66" t="s">
-        <v>894</v>
+        <v>893</v>
       </c>
       <c r="P159" s="66"/>
       <c r="Q159" s="66"/>
@@ -31303,10 +31356,10 @@
     </row>
     <row r="160" spans="1:20" ht="15" customHeight="1">
       <c r="A160" s="63" t="s">
+        <v>894</v>
+      </c>
+      <c r="B160" s="63" t="s">
         <v>895</v>
-      </c>
-      <c r="B160" s="63" t="s">
-        <v>896</v>
       </c>
       <c r="C160" s="63" t="s">
         <v>95</v>
@@ -31355,10 +31408,10 @@
     </row>
     <row r="161" spans="1:20" ht="15" customHeight="1">
       <c r="A161" s="66" t="s">
+        <v>896</v>
+      </c>
+      <c r="B161" s="66" t="s">
         <v>897</v>
-      </c>
-      <c r="B161" s="66" t="s">
-        <v>898</v>
       </c>
       <c r="C161" s="66" t="s">
         <v>95</v>
@@ -31407,10 +31460,10 @@
     </row>
     <row r="162" spans="1:20" ht="15" customHeight="1">
       <c r="A162" s="63" t="s">
+        <v>898</v>
+      </c>
+      <c r="B162" s="63" t="s">
         <v>899</v>
-      </c>
-      <c r="B162" s="63" t="s">
-        <v>900</v>
       </c>
       <c r="C162" s="63" t="s">
         <v>95</v>
@@ -31459,10 +31512,10 @@
     </row>
     <row r="163" spans="1:20" ht="15" customHeight="1">
       <c r="A163" s="66" t="s">
+        <v>900</v>
+      </c>
+      <c r="B163" s="66" t="s">
         <v>901</v>
-      </c>
-      <c r="B163" s="66" t="s">
-        <v>902</v>
       </c>
       <c r="C163" s="66" t="s">
         <v>95</v>
@@ -31509,10 +31562,10 @@
     </row>
     <row r="164" spans="1:20" ht="60" customHeight="1">
       <c r="A164" s="63" t="s">
+        <v>902</v>
+      </c>
+      <c r="B164" s="63" t="s">
         <v>903</v>
-      </c>
-      <c r="B164" s="63" t="s">
-        <v>904</v>
       </c>
       <c r="C164" s="63" t="s">
         <v>95</v>
@@ -31546,7 +31599,7 @@
         <v>1013</v>
       </c>
       <c r="L164" s="63" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
       <c r="M164" s="63"/>
       <c r="N164" s="63" t="s">
@@ -31554,7 +31607,7 @@
       </c>
       <c r="O164" s="63"/>
       <c r="P164" s="63" t="s">
-        <v>906</v>
+        <v>905</v>
       </c>
       <c r="Q164" s="63"/>
       <c r="R164" s="63"/>
@@ -31563,10 +31616,10 @@
     </row>
     <row r="165" spans="1:20" ht="15" customHeight="1">
       <c r="A165" s="66" t="s">
+        <v>906</v>
+      </c>
+      <c r="B165" s="66" t="s">
         <v>907</v>
-      </c>
-      <c r="B165" s="66" t="s">
-        <v>908</v>
       </c>
       <c r="C165" s="66" t="s">
         <v>95</v>
@@ -31608,7 +31661,7 @@
       </c>
       <c r="O165" s="66"/>
       <c r="P165" s="66" t="s">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="Q165" s="66"/>
       <c r="R165" s="66"/>
@@ -31617,10 +31670,10 @@
     </row>
     <row r="166" spans="1:20" ht="15" customHeight="1">
       <c r="A166" s="63" t="s">
+        <v>909</v>
+      </c>
+      <c r="B166" s="63" t="s">
         <v>910</v>
-      </c>
-      <c r="B166" s="63" t="s">
-        <v>911</v>
       </c>
       <c r="C166" s="63" t="s">
         <v>95</v>
@@ -31654,7 +31707,7 @@
         <v>1212</v>
       </c>
       <c r="L166" s="63" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="M166" s="63"/>
       <c r="N166" s="63" t="s">
@@ -31662,7 +31715,7 @@
       </c>
       <c r="O166" s="63"/>
       <c r="P166" s="63" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="Q166" s="63"/>
       <c r="R166" s="63"/>
@@ -31671,10 +31724,10 @@
     </row>
     <row r="167" spans="1:20" ht="15" customHeight="1">
       <c r="A167" s="66" t="s">
+        <v>911</v>
+      </c>
+      <c r="B167" s="66" t="s">
         <v>912</v>
-      </c>
-      <c r="B167" s="66" t="s">
-        <v>913</v>
       </c>
       <c r="C167" s="66" t="s">
         <v>95</v>
@@ -31708,7 +31761,7 @@
         <v>2220</v>
       </c>
       <c r="L167" s="66" t="s">
-        <v>914</v>
+        <v>913</v>
       </c>
       <c r="M167" s="66"/>
       <c r="N167" s="66" t="s">
@@ -31716,7 +31769,7 @@
       </c>
       <c r="O167" s="66"/>
       <c r="P167" s="66" t="s">
-        <v>915</v>
+        <v>914</v>
       </c>
       <c r="Q167" s="66"/>
       <c r="R167" s="66"/>
@@ -31725,10 +31778,10 @@
     </row>
     <row r="168" spans="1:20" ht="15" customHeight="1">
       <c r="A168" s="63" t="s">
+        <v>915</v>
+      </c>
+      <c r="B168" s="63" t="s">
         <v>916</v>
-      </c>
-      <c r="B168" s="63" t="s">
-        <v>917</v>
       </c>
       <c r="C168" s="63" t="s">
         <v>95</v>
@@ -31762,7 +31815,7 @@
         <v>1216</v>
       </c>
       <c r="L168" s="63" t="s">
-        <v>918</v>
+        <v>917</v>
       </c>
       <c r="M168" s="63"/>
       <c r="N168" s="63" t="s">
@@ -31770,7 +31823,7 @@
       </c>
       <c r="O168" s="63"/>
       <c r="P168" s="63" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="Q168" s="63"/>
       <c r="R168" s="63"/>
@@ -31779,10 +31832,10 @@
     </row>
     <row r="169" spans="1:20" ht="15" customHeight="1">
       <c r="A169" s="66" t="s">
+        <v>919</v>
+      </c>
+      <c r="B169" s="66" t="s">
         <v>920</v>
-      </c>
-      <c r="B169" s="66" t="s">
-        <v>921</v>
       </c>
       <c r="C169" s="66" t="s">
         <v>95</v>
@@ -31822,7 +31875,7 @@
       </c>
       <c r="O169" s="66"/>
       <c r="P169" s="66" t="s">
-        <v>922</v>
+        <v>921</v>
       </c>
       <c r="Q169" s="66"/>
       <c r="R169" s="66"/>
@@ -31831,10 +31884,10 @@
     </row>
     <row r="170" spans="1:20" ht="30" customHeight="1">
       <c r="A170" s="63" t="s">
+        <v>922</v>
+      </c>
+      <c r="B170" s="63" t="s">
         <v>923</v>
-      </c>
-      <c r="B170" s="63" t="s">
-        <v>924</v>
       </c>
       <c r="C170" s="63" t="s">
         <v>95</v>
@@ -31868,7 +31921,7 @@
         <v>0</v>
       </c>
       <c r="L170" s="63" t="s">
-        <v>925</v>
+        <v>924</v>
       </c>
       <c r="M170" s="63"/>
       <c r="N170" s="63" t="s">
@@ -31876,7 +31929,7 @@
       </c>
       <c r="O170" s="63"/>
       <c r="P170" s="63" t="s">
-        <v>926</v>
+        <v>925</v>
       </c>
       <c r="Q170" s="63"/>
       <c r="R170" s="63"/>
@@ -31885,10 +31938,10 @@
     </row>
     <row r="171" spans="1:20" ht="31.5" customHeight="1">
       <c r="A171" s="66" t="s">
+        <v>926</v>
+      </c>
+      <c r="B171" s="63" t="s">
         <v>927</v>
-      </c>
-      <c r="B171" s="63" t="s">
-        <v>928</v>
       </c>
       <c r="C171" s="66" t="s">
         <v>95</v>
@@ -31922,7 +31975,7 @@
         <v>0</v>
       </c>
       <c r="L171" s="66" t="s">
-        <v>929</v>
+        <v>928</v>
       </c>
       <c r="M171" s="66"/>
       <c r="N171" s="66" t="s">
@@ -31937,10 +31990,10 @@
     </row>
     <row r="172" spans="1:20" ht="15" customHeight="1">
       <c r="A172" s="63" t="s">
+        <v>929</v>
+      </c>
+      <c r="B172" s="63" t="s">
         <v>930</v>
-      </c>
-      <c r="B172" s="63" t="s">
-        <v>931</v>
       </c>
       <c r="C172" s="63" t="s">
         <v>95</v>
@@ -31974,7 +32027,7 @@
         <v>0</v>
       </c>
       <c r="L172" s="63" t="s">
-        <v>932</v>
+        <v>931</v>
       </c>
       <c r="M172" s="63"/>
       <c r="N172" s="63" t="s">
@@ -31989,10 +32042,10 @@
     </row>
     <row r="173" spans="1:20" ht="15" customHeight="1">
       <c r="A173" s="66" t="s">
+        <v>932</v>
+      </c>
+      <c r="B173" s="66" t="s">
         <v>933</v>
-      </c>
-      <c r="B173" s="66" t="s">
-        <v>934</v>
       </c>
       <c r="C173" s="66" t="s">
         <v>95</v>
@@ -32041,10 +32094,10 @@
     </row>
     <row r="174" spans="1:20" ht="15" customHeight="1">
       <c r="A174" s="63" t="s">
+        <v>934</v>
+      </c>
+      <c r="B174" s="63" t="s">
         <v>935</v>
-      </c>
-      <c r="B174" s="63" t="s">
-        <v>936</v>
       </c>
       <c r="C174" s="63" t="s">
         <v>95</v>
@@ -32078,7 +32131,7 @@
         <v>0</v>
       </c>
       <c r="L174" s="63" t="s">
-        <v>937</v>
+        <v>936</v>
       </c>
       <c r="M174" s="63"/>
       <c r="N174" s="63" t="s">
@@ -32093,10 +32146,10 @@
     </row>
     <row r="175" spans="1:20" ht="90" customHeight="1">
       <c r="A175" s="66" t="s">
+        <v>937</v>
+      </c>
+      <c r="B175" s="66" t="s">
         <v>938</v>
-      </c>
-      <c r="B175" s="66" t="s">
-        <v>939</v>
       </c>
       <c r="C175" s="66" t="s">
         <v>95</v>
@@ -32130,7 +32183,7 @@
         <v>3491.25</v>
       </c>
       <c r="L175" s="66" t="s">
-        <v>1118</v>
+        <v>1116</v>
       </c>
       <c r="M175" s="66"/>
       <c r="N175" s="66" t="s">
@@ -32138,7 +32191,7 @@
       </c>
       <c r="O175" s="66"/>
       <c r="P175" s="66" t="s">
-        <v>1117</v>
+        <v>1115</v>
       </c>
       <c r="Q175" s="66"/>
       <c r="R175" s="66"/>
@@ -32147,10 +32200,10 @@
     </row>
     <row r="176" spans="1:20" ht="24" customHeight="1">
       <c r="A176" s="63" t="s">
+        <v>939</v>
+      </c>
+      <c r="B176" s="63" t="s">
         <v>940</v>
-      </c>
-      <c r="B176" s="63" t="s">
-        <v>941</v>
       </c>
       <c r="C176" s="63" t="s">
         <v>95</v>
@@ -32184,7 +32237,7 @@
         <v>0</v>
       </c>
       <c r="L176" s="63" t="s">
-        <v>942</v>
+        <v>941</v>
       </c>
       <c r="M176" s="63"/>
       <c r="N176" s="63" t="s">
@@ -32199,10 +32252,10 @@
     </row>
     <row r="177" spans="1:20" ht="33.75" customHeight="1">
       <c r="A177" s="66" t="s">
+        <v>942</v>
+      </c>
+      <c r="B177" s="66" t="s">
         <v>943</v>
-      </c>
-      <c r="B177" s="66" t="s">
-        <v>944</v>
       </c>
       <c r="C177" s="66" t="s">
         <v>95</v>
@@ -32236,7 +32289,7 @@
         <v>0</v>
       </c>
       <c r="L177" s="66" t="s">
-        <v>945</v>
+        <v>944</v>
       </c>
       <c r="M177" s="66"/>
       <c r="N177" s="66" t="s">
@@ -32244,7 +32297,7 @@
       </c>
       <c r="O177" s="66"/>
       <c r="P177" s="66" t="s">
-        <v>946</v>
+        <v>945</v>
       </c>
       <c r="Q177" s="66"/>
       <c r="R177" s="66"/>
@@ -32253,10 +32306,10 @@
     </row>
     <row r="178" spans="1:20" ht="15" customHeight="1">
       <c r="A178" s="63" t="s">
+        <v>946</v>
+      </c>
+      <c r="B178" s="63" t="s">
         <v>947</v>
-      </c>
-      <c r="B178" s="63" t="s">
-        <v>948</v>
       </c>
       <c r="C178" s="63" t="s">
         <v>95</v>
@@ -32290,7 +32343,7 @@
         <v>0</v>
       </c>
       <c r="L178" s="63" t="s">
-        <v>949</v>
+        <v>948</v>
       </c>
       <c r="M178" s="63"/>
       <c r="N178" s="63" t="s">
@@ -32298,7 +32351,7 @@
       </c>
       <c r="O178" s="63"/>
       <c r="P178" s="63" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="Q178" s="63"/>
       <c r="R178" s="63"/>
@@ -32307,10 +32360,10 @@
     </row>
     <row r="179" spans="1:20" ht="30" customHeight="1">
       <c r="A179" s="66" t="s">
+        <v>950</v>
+      </c>
+      <c r="B179" s="66" t="s">
         <v>951</v>
-      </c>
-      <c r="B179" s="66" t="s">
-        <v>952</v>
       </c>
       <c r="C179" s="66" t="s">
         <v>95</v>
@@ -32344,7 +32397,7 @@
         <v>0</v>
       </c>
       <c r="L179" s="66" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="M179" s="66"/>
       <c r="N179" s="66" t="s">
@@ -32352,7 +32405,7 @@
       </c>
       <c r="O179" s="66"/>
       <c r="P179" s="66" t="s">
-        <v>954</v>
+        <v>953</v>
       </c>
       <c r="Q179" s="66"/>
       <c r="R179" s="66"/>
@@ -32361,10 +32414,10 @@
     </row>
     <row r="180" spans="1:20" ht="33.75" customHeight="1">
       <c r="A180" s="63" t="s">
+        <v>954</v>
+      </c>
+      <c r="B180" s="63" t="s">
         <v>955</v>
-      </c>
-      <c r="B180" s="63" t="s">
-        <v>956</v>
       </c>
       <c r="C180" s="63" t="s">
         <v>95</v>
@@ -32398,7 +32451,7 @@
         <v>0</v>
       </c>
       <c r="L180" s="63" t="s">
-        <v>957</v>
+        <v>956</v>
       </c>
       <c r="M180" s="63"/>
       <c r="N180" s="63" t="s">
@@ -32413,10 +32466,10 @@
     </row>
     <row r="181" spans="1:20" ht="15" customHeight="1">
       <c r="A181" s="66" t="s">
+        <v>957</v>
+      </c>
+      <c r="B181" s="66" t="s">
         <v>958</v>
-      </c>
-      <c r="B181" s="66" t="s">
-        <v>959</v>
       </c>
       <c r="C181" s="66" t="s">
         <v>96</v>
@@ -32450,17 +32503,17 @@
         <v>3057</v>
       </c>
       <c r="L181" s="66" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="M181" s="66"/>
       <c r="N181" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O181" s="66" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="P181" s="66" t="s">
-        <v>960</v>
+        <v>959</v>
       </c>
       <c r="Q181" s="66"/>
       <c r="R181" s="66"/>
@@ -32469,10 +32522,10 @@
     </row>
     <row r="182" spans="1:20" ht="15" customHeight="1">
       <c r="A182" s="63" t="s">
+        <v>960</v>
+      </c>
+      <c r="B182" s="63" t="s">
         <v>961</v>
-      </c>
-      <c r="B182" s="63" t="s">
-        <v>962</v>
       </c>
       <c r="C182" s="63" t="s">
         <v>95</v>
@@ -32512,7 +32565,7 @@
       </c>
       <c r="O182" s="63"/>
       <c r="P182" s="63" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="Q182" s="63"/>
       <c r="R182" s="63"/>
@@ -32521,10 +32574,10 @@
     </row>
     <row r="183" spans="1:20" ht="15" customHeight="1">
       <c r="A183" s="66" t="s">
+        <v>963</v>
+      </c>
+      <c r="B183" s="66" t="s">
         <v>964</v>
-      </c>
-      <c r="B183" s="66" t="s">
-        <v>965</v>
       </c>
       <c r="C183" s="66" t="s">
         <v>95</v>
@@ -32536,10 +32589,10 @@
         <v>699</v>
       </c>
       <c r="F183" s="76">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G183" s="76">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H183" s="75">
         <v>0</v>
@@ -32550,14 +32603,14 @@
       </c>
       <c r="J183" s="75">
         <f t="shared" si="9"/>
-        <v>419</v>
+        <v>838</v>
       </c>
       <c r="K183" s="75">
         <f t="shared" si="10"/>
-        <v>2933</v>
+        <v>2514</v>
       </c>
       <c r="L183" s="66" t="s">
-        <v>1114</v>
+        <v>1158</v>
       </c>
       <c r="M183" s="66"/>
       <c r="N183" s="66" t="s">
@@ -32572,10 +32625,10 @@
     </row>
     <row r="184" spans="1:20" ht="52" customHeight="1">
       <c r="A184" s="63" t="s">
+        <v>965</v>
+      </c>
+      <c r="B184" s="63" t="s">
         <v>966</v>
-      </c>
-      <c r="B184" s="63" t="s">
-        <v>967</v>
       </c>
       <c r="C184" s="63" t="s">
         <v>95</v>
@@ -32587,10 +32640,10 @@
         <v>1380</v>
       </c>
       <c r="F184" s="78">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G184" s="78">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H184" s="77">
         <f t="shared" ref="H184:H226" si="12">F184+IF(LEN(G184)=0,0,G184)</f>
@@ -32602,14 +32655,14 @@
       </c>
       <c r="J184" s="77">
         <f t="shared" si="9"/>
-        <v>14256</v>
+        <v>15147</v>
       </c>
       <c r="K184" s="77">
         <f t="shared" si="10"/>
-        <v>3564</v>
+        <v>2673</v>
       </c>
       <c r="L184" s="63" t="s">
-        <v>1131</v>
+        <v>1156</v>
       </c>
       <c r="M184" s="63"/>
       <c r="N184" s="63" t="s">
@@ -32624,10 +32677,10 @@
     </row>
     <row r="185" spans="1:20" ht="15" customHeight="1">
       <c r="A185" s="66" t="s">
+        <v>967</v>
+      </c>
+      <c r="B185" s="66" t="s">
         <v>968</v>
-      </c>
-      <c r="B185" s="66" t="s">
-        <v>969</v>
       </c>
       <c r="C185" s="66" t="s">
         <v>95</v>
@@ -32661,7 +32714,7 @@
         <v>0</v>
       </c>
       <c r="L185" s="66" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="M185" s="66"/>
       <c r="N185" s="66" t="s">
@@ -32676,7 +32729,7 @@
     </row>
     <row r="186" spans="1:20" ht="15" customHeight="1">
       <c r="A186" s="63" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="B186" s="63" t="s">
         <v>790</v>
@@ -32726,10 +32779,10 @@
     </row>
     <row r="187" spans="1:20" ht="15" customHeight="1">
       <c r="A187" s="66" t="s">
+        <v>971</v>
+      </c>
+      <c r="B187" s="66" t="s">
         <v>972</v>
-      </c>
-      <c r="B187" s="66" t="s">
-        <v>973</v>
       </c>
       <c r="C187" s="66" t="s">
         <v>95</v>
@@ -32776,10 +32829,10 @@
     </row>
     <row r="188" spans="1:20" ht="15" customHeight="1">
       <c r="A188" s="63" t="s">
+        <v>973</v>
+      </c>
+      <c r="B188" s="63" t="s">
         <v>974</v>
-      </c>
-      <c r="B188" s="63" t="s">
-        <v>975</v>
       </c>
       <c r="C188" s="63" t="s">
         <v>95</v>
@@ -32791,10 +32844,10 @@
         <v>1380</v>
       </c>
       <c r="F188" s="78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G188" s="78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H188" s="77">
         <f t="shared" si="12"/>
@@ -32806,18 +32859,18 @@
       </c>
       <c r="J188" s="77">
         <f t="shared" si="9"/>
-        <v>891</v>
+        <v>1782</v>
       </c>
       <c r="K188" s="77">
         <f t="shared" si="10"/>
-        <v>891</v>
+        <v>0</v>
       </c>
       <c r="L188" s="63" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="M188" s="63"/>
       <c r="N188" s="63" t="s">
-        <v>589</v>
+        <v>504</v>
       </c>
       <c r="O188" s="63"/>
       <c r="P188" s="63"/>
@@ -32828,10 +32881,10 @@
     </row>
     <row r="189" spans="1:20" ht="52" customHeight="1">
       <c r="A189" s="66" t="s">
+        <v>975</v>
+      </c>
+      <c r="B189" s="63" t="s">
         <v>976</v>
-      </c>
-      <c r="B189" s="63" t="s">
-        <v>977</v>
       </c>
       <c r="C189" s="63" t="s">
         <v>95</v>
@@ -32865,7 +32918,7 @@
         <v>1782</v>
       </c>
       <c r="L189" s="66" t="s">
-        <v>1157</v>
+        <v>1150</v>
       </c>
       <c r="M189" s="66"/>
       <c r="N189" s="66" t="s">
@@ -32873,7 +32926,7 @@
       </c>
       <c r="O189" s="66"/>
       <c r="P189" s="66" t="s">
-        <v>1156</v>
+        <v>1149</v>
       </c>
       <c r="Q189" s="66"/>
       <c r="R189" s="66"/>
@@ -32882,10 +32935,10 @@
     </row>
     <row r="190" spans="1:20" ht="15" customHeight="1">
       <c r="A190" s="63" t="s">
+        <v>977</v>
+      </c>
+      <c r="B190" s="66" t="s">
         <v>978</v>
-      </c>
-      <c r="B190" s="66" t="s">
-        <v>979</v>
       </c>
       <c r="C190" s="66" t="s">
         <v>95</v>
@@ -32921,20 +32974,20 @@
       <c r="L190" s="63"/>
       <c r="M190" s="63"/>
       <c r="N190" s="58" t="s">
+        <v>979</v>
+      </c>
+      <c r="P190" s="58" t="s">
         <v>980</v>
-      </c>
-      <c r="P190" s="58" t="s">
-        <v>981</v>
       </c>
       <c r="S190" s="58"/>
       <c r="T190" s="58"/>
     </row>
     <row r="191" spans="1:20" ht="30" customHeight="1">
       <c r="A191" s="66" t="s">
+        <v>981</v>
+      </c>
+      <c r="B191" s="63" t="s">
         <v>982</v>
-      </c>
-      <c r="B191" s="63" t="s">
-        <v>983</v>
       </c>
       <c r="C191" s="63" t="s">
         <v>95</v>
@@ -32973,17 +33026,17 @@
         <v>678</v>
       </c>
       <c r="P191" s="58" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="S191" s="58"/>
       <c r="T191" s="58"/>
     </row>
     <row r="192" spans="1:20" ht="15" customHeight="1">
       <c r="A192" s="63" t="s">
+        <v>984</v>
+      </c>
+      <c r="B192" s="66" t="s">
         <v>985</v>
-      </c>
-      <c r="B192" s="66" t="s">
-        <v>986</v>
       </c>
       <c r="C192" s="66" t="s">
         <v>95</v>
@@ -33017,24 +33070,24 @@
         <v>1616</v>
       </c>
       <c r="L192" s="63" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="M192" s="63"/>
       <c r="N192" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P192" s="58" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="S192" s="58"/>
       <c r="T192" s="58"/>
     </row>
     <row r="193" spans="1:20" ht="15" customHeight="1">
       <c r="A193" s="66" t="s">
+        <v>986</v>
+      </c>
+      <c r="B193" s="63" t="s">
         <v>987</v>
-      </c>
-      <c r="B193" s="63" t="s">
-        <v>988</v>
       </c>
       <c r="C193" s="63" t="s">
         <v>95</v>
@@ -33073,17 +33126,17 @@
         <v>678</v>
       </c>
       <c r="P193" s="58" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="S193" s="58"/>
       <c r="T193" s="58"/>
     </row>
     <row r="194" spans="1:20" ht="15" customHeight="1">
       <c r="A194" s="63" t="s">
+        <v>989</v>
+      </c>
+      <c r="B194" s="63" t="s">
         <v>990</v>
-      </c>
-      <c r="B194" s="63" t="s">
-        <v>991</v>
       </c>
       <c r="C194" s="63" t="s">
         <v>95</v>
@@ -33122,17 +33175,17 @@
         <v>678</v>
       </c>
       <c r="P194" s="58" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="S194" s="58"/>
       <c r="T194" s="58"/>
     </row>
     <row r="195" spans="1:20" ht="15" customHeight="1">
       <c r="A195" s="66" t="s">
+        <v>992</v>
+      </c>
+      <c r="B195" s="66" t="s">
         <v>993</v>
-      </c>
-      <c r="B195" s="66" t="s">
-        <v>994</v>
       </c>
       <c r="C195" s="66" t="s">
         <v>95</v>
@@ -33166,24 +33219,24 @@
         <v>5467</v>
       </c>
       <c r="L195" s="66" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="M195" s="66"/>
       <c r="N195" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P195" s="58" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="S195" s="58"/>
       <c r="T195" s="58"/>
     </row>
     <row r="196" spans="1:20" ht="15" customHeight="1">
       <c r="A196" s="63" t="s">
+        <v>996</v>
+      </c>
+      <c r="B196" s="63" t="s">
         <v>997</v>
-      </c>
-      <c r="B196" s="63" t="s">
-        <v>998</v>
       </c>
       <c r="C196" s="63" t="s">
         <v>95</v>
@@ -33217,24 +33270,24 @@
         <v>3985</v>
       </c>
       <c r="L196" s="63" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="M196" s="63"/>
       <c r="N196" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P196" s="58" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="S196" s="58"/>
       <c r="T196" s="58"/>
     </row>
     <row r="197" spans="1:20" ht="15" customHeight="1">
       <c r="A197" s="66" t="s">
+        <v>998</v>
+      </c>
+      <c r="B197" s="66" t="s">
         <v>999</v>
-      </c>
-      <c r="B197" s="66" t="s">
-        <v>1000</v>
       </c>
       <c r="C197" s="66" t="s">
         <v>95</v>
@@ -33273,17 +33326,17 @@
         <v>678</v>
       </c>
       <c r="P197" s="58" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="S197" s="58"/>
       <c r="T197" s="58"/>
     </row>
     <row r="198" spans="1:20" ht="15" customHeight="1">
       <c r="A198" s="63" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B198" s="63" t="s">
         <v>1002</v>
-      </c>
-      <c r="B198" s="63" t="s">
-        <v>1003</v>
       </c>
       <c r="C198" s="63" t="s">
         <v>95</v>
@@ -33322,17 +33375,17 @@
         <v>678</v>
       </c>
       <c r="P198" s="58" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="S198" s="58"/>
       <c r="T198" s="58"/>
     </row>
     <row r="199" spans="1:20" ht="15" customHeight="1">
       <c r="A199" s="66" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B199" s="63" t="s">
         <v>1005</v>
-      </c>
-      <c r="B199" s="63" t="s">
-        <v>1006</v>
       </c>
       <c r="C199" s="63" t="s">
         <v>95</v>
@@ -33371,17 +33424,17 @@
         <v>678</v>
       </c>
       <c r="P199" s="58" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="S199" s="58"/>
       <c r="T199" s="58"/>
     </row>
     <row r="200" spans="1:20" ht="30" customHeight="1">
       <c r="A200" s="63" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B200" s="66" t="s">
         <v>1008</v>
-      </c>
-      <c r="B200" s="66" t="s">
-        <v>1009</v>
       </c>
       <c r="C200" s="66" t="s">
         <v>95</v>
@@ -33415,24 +33468,24 @@
         <v>2598</v>
       </c>
       <c r="L200" s="63" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="M200" s="63"/>
       <c r="N200" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P200" s="58" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="S200" s="58"/>
       <c r="T200" s="58"/>
     </row>
     <row r="201" spans="1:20" ht="15" customHeight="1">
       <c r="A201" s="66" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B201" s="63" t="s">
         <v>1010</v>
-      </c>
-      <c r="B201" s="63" t="s">
-        <v>1011</v>
       </c>
       <c r="C201" s="63" t="s">
         <v>95</v>
@@ -33466,24 +33519,24 @@
         <v>724</v>
       </c>
       <c r="L201" s="66" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="M201" s="66"/>
       <c r="N201" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P201" s="58" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="S201" s="58"/>
       <c r="T201" s="58"/>
     </row>
     <row r="202" spans="1:20" ht="15" customHeight="1">
       <c r="A202" s="63" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B202" s="66" t="s">
         <v>1014</v>
-      </c>
-      <c r="B202" s="66" t="s">
-        <v>1015</v>
       </c>
       <c r="C202" s="66" t="s">
         <v>95</v>
@@ -33517,24 +33570,24 @@
         <v>3760</v>
       </c>
       <c r="L202" s="63" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
       <c r="M202" s="63"/>
       <c r="N202" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="58" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="S202" s="58"/>
       <c r="T202" s="58"/>
     </row>
     <row r="203" spans="1:20" ht="15" customHeight="1">
       <c r="A203" s="66" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B203" s="63" t="s">
         <v>1016</v>
-      </c>
-      <c r="B203" s="63" t="s">
-        <v>1017</v>
       </c>
       <c r="C203" s="63" t="s">
         <v>95</v>
@@ -33568,24 +33621,24 @@
         <v>0</v>
       </c>
       <c r="L203" s="66" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="M203" s="66"/>
       <c r="N203" s="58" t="s">
         <v>504</v>
       </c>
       <c r="P203" s="58" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="S203" s="58"/>
       <c r="T203" s="58"/>
     </row>
     <row r="204" spans="1:20" ht="15" customHeight="1">
       <c r="A204" s="63" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B204" s="63" t="s">
         <v>1020</v>
-      </c>
-      <c r="B204" s="63" t="s">
-        <v>1021</v>
       </c>
       <c r="C204" s="63" t="s">
         <v>95</v>
@@ -33619,24 +33672,24 @@
         <v>880</v>
       </c>
       <c r="L204" s="63" t="s">
-        <v>1143</v>
+        <v>1137</v>
       </c>
       <c r="M204" s="63"/>
       <c r="N204" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P204" s="58" t="s">
-        <v>1142</v>
+        <v>1136</v>
       </c>
       <c r="S204" s="58"/>
       <c r="T204" s="58"/>
     </row>
     <row r="205" spans="1:20" ht="15" customHeight="1">
       <c r="A205" s="66" t="s">
+        <v>1021</v>
+      </c>
+      <c r="B205" s="66" t="s">
         <v>1022</v>
-      </c>
-      <c r="B205" s="66" t="s">
-        <v>1023</v>
       </c>
       <c r="C205" s="66" t="s">
         <v>95</v>
@@ -33670,24 +33723,24 @@
         <v>1522</v>
       </c>
       <c r="L205" s="66" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="M205" s="66"/>
       <c r="N205" s="58" t="s">
         <v>678</v>
       </c>
       <c r="P205" s="58" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="S205" s="58"/>
       <c r="T205" s="58"/>
     </row>
     <row r="206" spans="1:20" ht="15" customHeight="1">
       <c r="A206" s="63" t="s">
+        <v>1025</v>
+      </c>
+      <c r="B206" s="63" t="s">
         <v>1026</v>
-      </c>
-      <c r="B206" s="63" t="s">
-        <v>1027</v>
       </c>
       <c r="C206" s="63" t="s">
         <v>95</v>
@@ -33726,17 +33779,17 @@
         <v>678</v>
       </c>
       <c r="P206" s="58" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="S206" s="58"/>
       <c r="T206" s="58"/>
     </row>
     <row r="207" spans="1:20" ht="15" customHeight="1">
       <c r="A207" s="66" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B207" s="66" t="s">
         <v>1029</v>
-      </c>
-      <c r="B207" s="66" t="s">
-        <v>1030</v>
       </c>
       <c r="C207" s="66" t="s">
         <v>95</v>
@@ -33770,24 +33823,24 @@
         <v>3312</v>
       </c>
       <c r="L207" s="66" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="M207" s="66"/>
       <c r="N207" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P207" s="58" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="S207" s="58"/>
       <c r="T207" s="58"/>
     </row>
     <row r="208" spans="1:20" ht="30" customHeight="1">
       <c r="A208" s="63" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B208" s="63" t="s">
         <v>1033</v>
-      </c>
-      <c r="B208" s="63" t="s">
-        <v>1034</v>
       </c>
       <c r="C208" s="63" t="s">
         <v>95</v>
@@ -33826,17 +33879,17 @@
         <v>678</v>
       </c>
       <c r="P208" s="58" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="S208" s="58"/>
       <c r="T208" s="58"/>
     </row>
     <row r="209" spans="1:20" ht="15" customHeight="1">
       <c r="A209" s="66" t="s">
+        <v>1035</v>
+      </c>
+      <c r="B209" s="63" t="s">
         <v>1036</v>
-      </c>
-      <c r="B209" s="63" t="s">
-        <v>1037</v>
       </c>
       <c r="C209" s="63" t="s">
         <v>95</v>
@@ -33870,24 +33923,24 @@
         <v>982</v>
       </c>
       <c r="L209" s="66" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="M209" s="66"/>
       <c r="N209" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P209" s="58" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="S209" s="58"/>
       <c r="T209" s="58"/>
     </row>
     <row r="210" spans="1:20" ht="15" customHeight="1">
       <c r="A210" s="63" t="s">
+        <v>1037</v>
+      </c>
+      <c r="B210" s="66" t="s">
         <v>1038</v>
-      </c>
-      <c r="B210" s="66" t="s">
-        <v>1039</v>
       </c>
       <c r="C210" s="66" t="s">
         <v>95</v>
@@ -33926,17 +33979,17 @@
         <v>678</v>
       </c>
       <c r="P210" s="58" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="S210" s="58"/>
       <c r="T210" s="58"/>
     </row>
     <row r="211" spans="1:20" ht="15" customHeight="1">
       <c r="A211" s="66" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="B211" s="63" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
       <c r="C211" s="63" t="s">
         <v>95</v>
@@ -33975,17 +34028,17 @@
         <v>678</v>
       </c>
       <c r="P211" s="58" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="S211" s="58"/>
       <c r="T211" s="58"/>
     </row>
     <row r="212" spans="1:20" ht="15" customHeight="1">
       <c r="A212" s="63" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="B212" s="66" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="C212" s="66" t="s">
         <v>95</v>
@@ -34028,7 +34081,7 @@
     </row>
     <row r="213" spans="1:20" ht="15" customHeight="1">
       <c r="A213" s="66" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B213" s="63"/>
       <c r="C213" s="63"/>
@@ -34063,7 +34116,7 @@
     </row>
     <row r="214" spans="1:20" ht="15" customHeight="1">
       <c r="A214" s="63" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B214" s="63"/>
       <c r="C214" s="63"/>
@@ -34098,7 +34151,7 @@
     </row>
     <row r="215" spans="1:20" ht="15" customHeight="1">
       <c r="A215" s="66" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B215" s="66"/>
       <c r="C215" s="66"/>
@@ -34133,7 +34186,7 @@
     </row>
     <row r="216" spans="1:20" ht="15" customHeight="1">
       <c r="A216" s="63" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B216" s="63"/>
       <c r="C216" s="63"/>
@@ -34168,7 +34221,7 @@
     </row>
     <row r="217" spans="1:20" ht="15" customHeight="1">
       <c r="A217" s="66" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B217" s="66"/>
       <c r="C217" s="66"/>
@@ -34203,7 +34256,7 @@
     </row>
     <row r="218" spans="1:20" ht="15" customHeight="1">
       <c r="A218" s="63" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B218" s="63"/>
       <c r="C218" s="63"/>
@@ -34238,7 +34291,7 @@
     </row>
     <row r="219" spans="1:20" ht="15" customHeight="1">
       <c r="A219" s="66" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B219" s="63"/>
       <c r="C219" s="63"/>
@@ -34273,7 +34326,7 @@
     </row>
     <row r="220" spans="1:20" ht="15" customHeight="1">
       <c r="A220" s="63" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B220" s="66"/>
       <c r="C220" s="66"/>
@@ -34308,7 +34361,7 @@
     </row>
     <row r="221" spans="1:20" ht="15" customHeight="1">
       <c r="A221" s="66" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B221" s="63"/>
       <c r="C221" s="63"/>
@@ -34343,7 +34396,7 @@
     </row>
     <row r="222" spans="1:20" ht="15" customHeight="1">
       <c r="A222" s="63" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B222" s="66"/>
       <c r="C222" s="66"/>
@@ -34378,7 +34431,7 @@
     </row>
     <row r="223" spans="1:20" ht="15" customHeight="1">
       <c r="A223" s="66" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B223" s="63"/>
       <c r="C223" s="63"/>
@@ -34413,7 +34466,7 @@
     </row>
     <row r="224" spans="1:20" ht="15" customHeight="1">
       <c r="A224" s="63" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B224" s="63"/>
       <c r="C224" s="63"/>
@@ -34448,7 +34501,7 @@
     </row>
     <row r="225" spans="1:20" ht="15" customHeight="1">
       <c r="A225" s="66" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B225" s="66"/>
       <c r="C225" s="66"/>
@@ -34483,7 +34536,7 @@
     </row>
     <row r="226" spans="1:20" ht="15" customHeight="1">
       <c r="A226" s="63" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B226" s="63"/>
       <c r="C226" s="63"/>
@@ -38398,7 +38451,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="92" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B1" s="92"/>
     </row>
@@ -38407,7 +38460,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -38439,25 +38492,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="83" t="s">
+        <v>1059</v>
+      </c>
+      <c r="C7" s="83" t="s">
         <v>1060</v>
       </c>
-      <c r="C7" s="83" t="s">
+      <c r="D7" s="83" t="s">
         <v>1061</v>
       </c>
-      <c r="D7" s="83" t="s">
+      <c r="E7" s="83" t="s">
         <v>1062</v>
       </c>
-      <c r="E7" s="83" t="s">
+      <c r="F7" s="83" t="s">
         <v>1063</v>
       </c>
-      <c r="F7" s="83" t="s">
+      <c r="G7" s="83" t="s">
         <v>1064</v>
       </c>
-      <c r="G7" s="83" t="s">
+      <c r="H7" s="83" t="s">
         <v>1065</v>
-      </c>
-      <c r="H7" s="83" t="s">
-        <v>1066</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -38561,7 +38614,7 @@
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="93" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B12" s="93"/>
       <c r="C12" s="93"/>
@@ -38574,13 +38627,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="83" t="s">
+        <v>1067</v>
+      </c>
+      <c r="C13" s="83" t="s">
         <v>1068</v>
       </c>
-      <c r="C13" s="83" t="s">
+      <c r="D13" s="83" t="s">
         <v>1069</v>
-      </c>
-      <c r="D13" s="83" t="s">
-        <v>1070</v>
       </c>
       <c r="E13" s="83" t="s">
         <v>99</v>
@@ -38594,7 +38647,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -38612,7 +38665,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -38666,7 +38719,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -38684,7 +38737,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -38702,7 +38755,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -38720,7 +38773,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -38738,7 +38791,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -38774,7 +38827,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -38810,7 +38863,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -38828,7 +38881,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -38911,7 +38964,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
     </row>
   </sheetData>
@@ -38941,7 +38994,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="90" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="84" customFormat="1" ht="13.5" customHeight="1">
@@ -38949,22 +39002,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="83" t="s">
+        <v>1073</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>1058</v>
+      </c>
+      <c r="D3" s="83" t="s">
         <v>1074</v>
       </c>
-      <c r="C3" s="83" t="s">
-        <v>1059</v>
-      </c>
-      <c r="D3" s="83" t="s">
+      <c r="E3" s="83" t="s">
         <v>1075</v>
       </c>
-      <c r="E3" s="83" t="s">
+      <c r="F3" s="83" t="s">
         <v>1076</v>
       </c>
-      <c r="F3" s="83" t="s">
+      <c r="G3" s="83" t="s">
         <v>1077</v>
-      </c>
-      <c r="G3" s="83" t="s">
-        <v>1078</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -38973,7 +39026,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>375433</v>
+        <v>378862</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -38981,11 +39034,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>147558.50579999998</v>
+        <v>148701.73439999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>227874.49420000002</v>
+        <v>230160.26560000001</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -38993,7 +39046,7 @@
       </c>
       <c r="G4" s="85">
         <f>E4+F4</f>
-        <v>90564.468200000003</v>
+        <v>92850.239600000001</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -39010,11 +39063,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>147469.9884</v>
+        <v>148612.5312</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-92845.988400000002</v>
+        <v>-93988.531199999998</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39022,7 +39075,7 @@
       </c>
       <c r="G5" s="86">
         <f>E5+F5</f>
-        <v>-21258.946400000001</v>
+        <v>-22401.489199999996</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -39039,11 +39092,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>147558.50579999998</v>
+        <v>148701.73439999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-135028.50579999998</v>
+        <v>-136171.73439999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39051,7 +39104,7 @@
       </c>
       <c r="G6" s="85">
         <f>E6+F6</f>
-        <v>-69305.521799999973</v>
+        <v>-70448.750399999975</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -39061,27 +39114,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
7/13 Sales & purchase
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C95EFE2-6570-164C-897F-14767FEE7873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7996C2A6-68C2-3040-8098-70F65C3A49B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2930" uniqueCount="1161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2942" uniqueCount="1164">
   <si>
     <t>Notes:</t>
   </si>
@@ -3426,12 +3426,6 @@
     <t>Komalavalli</t>
   </si>
   <si>
-    <t>Komalavalli - Blue</t>
-  </si>
-  <si>
-    <t>pink, yellow, maroon, deep blue, green</t>
-  </si>
-  <si>
     <t>Banarasi bulk order - Komappas</t>
   </si>
   <si>
@@ -3541,13 +3535,28 @@
     <t>Preeha Rajeevan</t>
   </si>
   <si>
-    <t>Irene, Preetha Rajeevan</t>
-  </si>
-  <si>
     <t>Chithra - XL, Shanu - XXL (1350)</t>
   </si>
   <si>
     <t>CHR-154 Dark Brown Salwar with mirrion work - XL</t>
+  </si>
+  <si>
+    <t>Gokul</t>
+  </si>
+  <si>
+    <t>Irene, Preetha Rajeevan, Gokul</t>
+  </si>
+  <si>
+    <t>CHR-201 Tusser Saree Maroon &amp; Blue</t>
+  </si>
+  <si>
+    <t>Anjumol Canada</t>
+  </si>
+  <si>
+    <t>Komalavalli - Blue, Anjumol canada - Blue &amp; Red</t>
+  </si>
+  <si>
+    <t>Green, Pink, Yellow</t>
   </si>
 </sst>
 </file>
@@ -4427,7 +4436,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>271</c:v>
+                  <c:v>274</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>95</c:v>
@@ -4530,7 +4539,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>149</c:v>
+                  <c:v>147</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>53</c:v>
@@ -4863,7 +4872,7 @@
                   <c:v>56434</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>116423.43</c:v>
+                  <c:v>115064.43</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>590</c:v>
@@ -5196,7 +5205,7 @@
                   <c:v>99043</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>57074</c:v>
+                  <c:v>63028</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5356,7 +5365,7 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>27448</c:v>
+                  <c:v>31147</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5796,7 +5805,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-29626</c:v>
+                  <c:v>-31881</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6260,10 +6269,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>371</c:v>
+                  <c:v>374</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-279</c:v>
+                  <c:v>-281</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7435,7 +7444,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>511221</v>
+        <v>517175</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7450,7 +7459,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>446016</v>
+        <v>449715</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7467,7 +7476,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>455946</v>
+        <v>459645</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7484,7 +7493,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-65205</v>
+        <v>-67460</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7519,7 +7528,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>53443.66</v>
+        <v>57412.993333333347</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7529,7 +7538,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>24420.67</v>
+        <v>22436.003333333341</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7539,7 +7548,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-77864.33</v>
+        <v>-79848.996666666659</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7578,15 +7587,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>242154</v>
+        <v>248108</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>170407</v>
+        <v>172391.66666666666</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>71747</v>
+        <v>75716.333333333343</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7594,11 +7603,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>53443.66</v>
+        <v>57412.993333333347</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹53,444</v>
+        <v>Receive ₹57,413</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7612,11 +7621,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>170407</v>
+        <v>172391.66666666666</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>66060</v>
+        <v>64075.333333333343</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7624,11 +7633,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>24420.67</v>
+        <v>22436.003333333341</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹24,421</v>
+        <v>Receive ₹22,436</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7642,11 +7651,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>170407</v>
+        <v>172391.66666666666</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-137807</v>
+        <v>-139791.66666666666</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7654,11 +7663,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-77864.33</v>
+        <v>-79848.996666666659</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹77,864</v>
+        <v>Pay ₹79,849</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7696,15 +7705,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>378862</v>
+        <v>382561</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>148701.73439999999</v>
+        <v>149934.981</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>230160.26560000001</v>
+        <v>232626.019</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7712,11 +7721,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>92850.239600000001</v>
+        <v>95315.992999999988</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹92,850</v>
+        <v>Pay ₹95,316</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7730,11 +7739,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>148612.5312</v>
+        <v>149845.038</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-93988.531199999998</v>
+        <v>-95221.038</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7742,11 +7751,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-22401.489199999996</v>
+        <v>-23633.995999999999</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹22,401</v>
+        <v>Receive ₹23,634</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7760,11 +7769,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>148701.73439999999</v>
+        <v>149934.981</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-136171.73439999999</v>
+        <v>-137404.981</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7772,11 +7781,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-70448.750399999975</v>
+        <v>-71681.996999999988</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹70,449</v>
+        <v>Receive ₹71,682</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7888,7 +7897,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46215</v>
+        <v>46217</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7897,14 +7906,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>511221</v>
+        <v>517175</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>446016</v>
+        <v>449715</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7913,14 +7922,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-65205</v>
+        <v>-67460</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>163826.63</v>
+        <v>162467.63</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7972,7 +7981,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>371</v>
+        <v>374</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -7996,7 +8005,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>-279</v>
+        <v>-281</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8073,15 +8082,15 @@
       </c>
       <c r="B16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A16)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>57074</v>
+        <v>63028</v>
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$995,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$995)=$B$7)*Sales!$C$2:$C$995),0)</f>
-        <v>27448</v>
+        <v>31147</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-29626</v>
+        <v>-31881</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8192,11 +8201,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8223,7 +8232,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>116423.43</v>
+        <v>115064.43</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9596,7 +9605,7 @@
         <v>28526</v>
       </c>
       <c r="D91" s="39" t="s">
-        <v>1122</v>
+        <v>1120</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" customHeight="1">
@@ -9642,10 +9651,18 @@
       </c>
     </row>
     <row r="95" spans="1:4" ht="15" customHeight="1">
-      <c r="A95" s="38"/>
-      <c r="B95" s="39"/>
-      <c r="C95" s="40"/>
-      <c r="D95" s="39"/>
+      <c r="A95" s="38">
+        <v>46216</v>
+      </c>
+      <c r="B95" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C95" s="40">
+        <v>5954</v>
+      </c>
+      <c r="D95" s="39" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="96" spans="1:4" ht="15" customHeight="1">
       <c r="A96" s="35"/>
@@ -18208,7 +18225,7 @@
         <v>46205</v>
       </c>
       <c r="B261" s="53" t="s">
-        <v>1124</v>
+        <v>1122</v>
       </c>
       <c r="C261" s="54">
         <v>1900</v>
@@ -18218,7 +18235,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>356</v>
@@ -18229,7 +18246,7 @@
         <v>46206</v>
       </c>
       <c r="B262" s="49" t="s">
-        <v>1129</v>
+        <v>1127</v>
       </c>
       <c r="C262" s="50">
         <v>1380</v>
@@ -18254,7 +18271,7 @@
         <v>46206</v>
       </c>
       <c r="B263" s="53" t="s">
-        <v>1130</v>
+        <v>1128</v>
       </c>
       <c r="C263" s="54">
         <v>1380</v>
@@ -18279,7 +18296,7 @@
         <v>46206</v>
       </c>
       <c r="B264" s="49" t="s">
-        <v>1141</v>
+        <v>1139</v>
       </c>
       <c r="C264" s="50">
         <v>2500</v>
@@ -18293,7 +18310,7 @@
       <c r="F264" s="49"/>
       <c r="G264" s="49"/>
       <c r="H264" s="51" t="s">
-        <v>1142</v>
+        <v>1140</v>
       </c>
       <c r="I264" s="49" t="s">
         <v>356</v>
@@ -18304,7 +18321,7 @@
         <v>46206</v>
       </c>
       <c r="B265" s="53" t="s">
-        <v>1133</v>
+        <v>1131</v>
       </c>
       <c r="C265" s="54">
         <v>1300</v>
@@ -18318,7 +18335,7 @@
       <c r="F265" s="56"/>
       <c r="G265" s="56"/>
       <c r="H265" s="57" t="s">
-        <v>1151</v>
+        <v>1149</v>
       </c>
       <c r="I265" s="53" t="s">
         <v>356</v>
@@ -18343,7 +18360,7 @@
       <c r="F266" s="49"/>
       <c r="G266" s="49"/>
       <c r="H266" s="51" t="s">
-        <v>1134</v>
+        <v>1132</v>
       </c>
       <c r="I266" s="49" t="s">
         <v>148</v>
@@ -18368,7 +18385,7 @@
       <c r="F267" s="56"/>
       <c r="G267" s="56"/>
       <c r="H267" s="57" t="s">
-        <v>1135</v>
+        <v>1133</v>
       </c>
       <c r="I267" s="53" t="s">
         <v>148</v>
@@ -18379,7 +18396,7 @@
         <v>46208</v>
       </c>
       <c r="B268" s="49" t="s">
-        <v>1140</v>
+        <v>1138</v>
       </c>
       <c r="C268" s="50">
         <v>2350</v>
@@ -18389,7 +18406,7 @@
       <c r="F268" s="49"/>
       <c r="G268" s="49"/>
       <c r="H268" s="51" t="s">
-        <v>1152</v>
+        <v>1150</v>
       </c>
       <c r="I268" s="49" t="s">
         <v>356</v>
@@ -18400,7 +18417,7 @@
         <v>46209</v>
       </c>
       <c r="B269" s="53" t="s">
-        <v>1138</v>
+        <v>1136</v>
       </c>
       <c r="C269" s="54">
         <v>1100</v>
@@ -18414,7 +18431,7 @@
       <c r="F269" s="56"/>
       <c r="G269" s="56"/>
       <c r="H269" s="57" t="s">
-        <v>1139</v>
+        <v>1137</v>
       </c>
       <c r="I269" s="53" t="s">
         <v>148</v>
@@ -18425,7 +18442,7 @@
         <v>46210</v>
       </c>
       <c r="B270" s="49" t="s">
-        <v>1145</v>
+        <v>1143</v>
       </c>
       <c r="C270" s="50">
         <v>3200</v>
@@ -18439,7 +18456,7 @@
       <c r="F270" s="49"/>
       <c r="G270" s="49"/>
       <c r="H270" s="51" t="s">
-        <v>1146</v>
+        <v>1144</v>
       </c>
       <c r="I270" s="49" t="s">
         <v>148</v>
@@ -18450,7 +18467,7 @@
         <v>46211</v>
       </c>
       <c r="B271" s="53" t="s">
-        <v>1147</v>
+        <v>1145</v>
       </c>
       <c r="C271" s="54">
         <v>1380</v>
@@ -18464,7 +18481,7 @@
       <c r="F271" s="56"/>
       <c r="G271" s="56"/>
       <c r="H271" s="57" t="s">
-        <v>1148</v>
+        <v>1146</v>
       </c>
       <c r="I271" s="53" t="s">
         <v>148</v>
@@ -18475,7 +18492,7 @@
         <v>46215</v>
       </c>
       <c r="B272" s="49" t="s">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="C272" s="50">
         <v>1380</v>
@@ -18500,7 +18517,7 @@
         <v>46215</v>
       </c>
       <c r="B273" s="53" t="s">
-        <v>1157</v>
+        <v>1155</v>
       </c>
       <c r="C273" s="54">
         <v>699</v>
@@ -18539,33 +18556,61 @@
       <c r="F274" s="49"/>
       <c r="G274" s="49"/>
       <c r="H274" s="51" t="s">
-        <v>1160</v>
+        <v>1157</v>
       </c>
       <c r="I274" s="49" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="275" spans="1:9">
-      <c r="A275" s="52"/>
-      <c r="B275" s="53"/>
-      <c r="C275" s="54"/>
-      <c r="D275" s="53"/>
-      <c r="E275" s="53"/>
+    <row r="275" spans="1:9" ht="14">
+      <c r="A275" s="52">
+        <v>46216</v>
+      </c>
+      <c r="B275" s="53" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C275" s="54">
+        <v>699</v>
+      </c>
+      <c r="D275" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E275" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F275" s="56"/>
       <c r="G275" s="56"/>
-      <c r="H275" s="57"/>
-      <c r="I275" s="53"/>
-    </row>
-    <row r="276" spans="1:9">
-      <c r="A276" s="48"/>
-      <c r="B276" s="49"/>
-      <c r="C276" s="50"/>
-      <c r="D276" s="49"/>
-      <c r="E276" s="49"/>
+      <c r="H275" s="57" t="s">
+        <v>1112</v>
+      </c>
+      <c r="I275" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="276" spans="1:9" ht="14">
+      <c r="A276" s="48">
+        <v>46216</v>
+      </c>
+      <c r="B276" s="49" t="s">
+        <v>1161</v>
+      </c>
+      <c r="C276" s="50">
+        <v>3000</v>
+      </c>
+      <c r="D276" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E276" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F276" s="49"/>
       <c r="G276" s="49"/>
-      <c r="H276" s="51"/>
-      <c r="I276" s="49"/>
+      <c r="H276" s="51" t="s">
+        <v>1160</v>
+      </c>
+      <c r="I276" s="49" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="277" spans="1:9">
       <c r="A277" s="52"/>
@@ -25365,7 +25410,7 @@
         <v>1145</v>
       </c>
       <c r="L59" s="66" t="s">
-        <v>1143</v>
+        <v>1141</v>
       </c>
       <c r="M59" s="66"/>
       <c r="N59" s="66" t="s">
@@ -26911,7 +26956,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="63" t="s">
-        <v>1144</v>
+        <v>1142</v>
       </c>
       <c r="M88" s="63"/>
       <c r="N88" s="63" t="s">
@@ -27171,7 +27216,7 @@
         <v>0</v>
       </c>
       <c r="L93" s="66" t="s">
-        <v>1128</v>
+        <v>1126</v>
       </c>
       <c r="M93" s="66"/>
       <c r="N93" s="63" t="s">
@@ -31069,14 +31114,14 @@
         <v>949</v>
       </c>
       <c r="L154" s="63" t="s">
-        <v>1131</v>
+        <v>1129</v>
       </c>
       <c r="M154" s="63"/>
       <c r="N154" s="63" t="s">
         <v>589</v>
       </c>
       <c r="O154" s="63" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="P154" s="63"/>
       <c r="Q154" s="63"/>
@@ -31123,14 +31168,14 @@
         <v>949</v>
       </c>
       <c r="L155" s="66" t="s">
-        <v>1159</v>
+        <v>1156</v>
       </c>
       <c r="M155" s="66"/>
       <c r="N155" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O155" s="66" t="s">
-        <v>1127</v>
+        <v>1125</v>
       </c>
       <c r="P155" s="66"/>
       <c r="Q155" s="66"/>
@@ -31177,7 +31222,7 @@
         <v>1900</v>
       </c>
       <c r="L156" s="63" t="s">
-        <v>1132</v>
+        <v>1130</v>
       </c>
       <c r="M156" s="63"/>
       <c r="N156" s="63" t="s">
@@ -32503,14 +32548,14 @@
         <v>3057</v>
       </c>
       <c r="L181" s="66" t="s">
-        <v>1125</v>
+        <v>1123</v>
       </c>
       <c r="M181" s="66"/>
       <c r="N181" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O181" s="66" t="s">
-        <v>1126</v>
+        <v>1124</v>
       </c>
       <c r="P181" s="66" t="s">
         <v>959</v>
@@ -32589,10 +32634,10 @@
         <v>699</v>
       </c>
       <c r="F183" s="76">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G183" s="76">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H183" s="75">
         <v>0</v>
@@ -32603,14 +32648,14 @@
       </c>
       <c r="J183" s="75">
         <f t="shared" si="9"/>
-        <v>838</v>
+        <v>1257</v>
       </c>
       <c r="K183" s="75">
         <f t="shared" si="10"/>
-        <v>2514</v>
+        <v>2095</v>
       </c>
       <c r="L183" s="66" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="M183" s="66"/>
       <c r="N183" s="66" t="s">
@@ -32662,7 +32707,7 @@
         <v>2673</v>
       </c>
       <c r="L184" s="63" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="M184" s="63"/>
       <c r="N184" s="63" t="s">
@@ -32866,7 +32911,7 @@
         <v>0</v>
       </c>
       <c r="L188" s="63" t="s">
-        <v>1154</v>
+        <v>1152</v>
       </c>
       <c r="M188" s="63"/>
       <c r="N188" s="63" t="s">
@@ -32918,7 +32963,7 @@
         <v>1782</v>
       </c>
       <c r="L189" s="66" t="s">
-        <v>1150</v>
+        <v>1148</v>
       </c>
       <c r="M189" s="66"/>
       <c r="N189" s="66" t="s">
@@ -32926,7 +32971,7 @@
       </c>
       <c r="O189" s="66"/>
       <c r="P189" s="66" t="s">
-        <v>1149</v>
+        <v>1147</v>
       </c>
       <c r="Q189" s="66"/>
       <c r="R189" s="66"/>
@@ -33548,14 +33593,14 @@
         <v>1500</v>
       </c>
       <c r="F202" s="78">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G202" s="78">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H202" s="77">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I202" s="77">
         <f>IF(D202&lt;&gt;"",D202,IFERROR(E202/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -33563,21 +33608,21 @@
       </c>
       <c r="J202" s="77">
         <f t="shared" si="13"/>
-        <v>940</v>
+        <v>2820</v>
       </c>
       <c r="K202" s="77">
         <f t="shared" si="14"/>
-        <v>3760</v>
+        <v>2820</v>
       </c>
       <c r="L202" s="63" t="s">
-        <v>1120</v>
+        <v>1162</v>
       </c>
       <c r="M202" s="63"/>
       <c r="N202" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="58" t="s">
-        <v>1121</v>
+        <v>1163</v>
       </c>
       <c r="S202" s="58"/>
       <c r="T202" s="58"/>
@@ -33672,14 +33717,14 @@
         <v>880</v>
       </c>
       <c r="L204" s="63" t="s">
-        <v>1137</v>
+        <v>1135</v>
       </c>
       <c r="M204" s="63"/>
       <c r="N204" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P204" s="58" t="s">
-        <v>1136</v>
+        <v>1134</v>
       </c>
       <c r="S204" s="58"/>
       <c r="T204" s="58"/>
@@ -34038,7 +34083,7 @@
         <v>1042</v>
       </c>
       <c r="B212" s="66" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="C212" s="66" t="s">
         <v>95</v>
@@ -38519,15 +38564,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>242154</v>
+        <v>248108</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>170407</v>
+        <v>172391.66666666666</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>71747</v>
+        <v>75716.333333333343</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38535,7 +38580,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>71747</v>
+        <v>75716.333333333343</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -38543,7 +38588,7 @@
       </c>
       <c r="H8" s="85">
         <f>F8-G8</f>
-        <v>53443.66</v>
+        <v>57412.993333333347</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -38556,11 +38601,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>170407</v>
+        <v>172391.66666666666</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>66060</v>
+        <v>64075.333333333343</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38568,7 +38613,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>66060</v>
+        <v>64075.333333333343</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -38576,7 +38621,7 @@
       </c>
       <c r="H9" s="86">
         <f>F9-G9</f>
-        <v>24420.67</v>
+        <v>22436.003333333341</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -38589,11 +38634,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>170407</v>
+        <v>172391.66666666666</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-137807</v>
+        <v>-139791.66666666666</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38601,7 +38646,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-137807</v>
+        <v>-139791.66666666666</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -38609,7 +38654,7 @@
       </c>
       <c r="H10" s="85">
         <f>F10-G10</f>
-        <v>-77864.33</v>
+        <v>-79848.996666666659</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">
@@ -39026,7 +39071,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>378862</v>
+        <v>382561</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -39034,11 +39079,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>148701.73439999999</v>
+        <v>149934.981</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>230160.26560000001</v>
+        <v>232626.019</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39046,7 +39091,7 @@
       </c>
       <c r="G4" s="85">
         <f>E4+F4</f>
-        <v>92850.239600000001</v>
+        <v>95315.992999999988</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -39063,11 +39108,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>148612.5312</v>
+        <v>149845.038</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-93988.531199999998</v>
+        <v>-95221.038</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39075,7 +39120,7 @@
       </c>
       <c r="G5" s="86">
         <f>E5+F5</f>
-        <v>-22401.489199999996</v>
+        <v>-23633.995999999999</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -39092,11 +39137,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>148701.73439999999</v>
+        <v>149934.981</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-136171.73439999999</v>
+        <v>-137404.981</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39104,7 +39149,7 @@
       </c>
       <c r="G6" s="85">
         <f>E6+F6</f>
-        <v>-70448.750399999975</v>
+        <v>-71681.996999999988</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
7/16 sales & purchases
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7996C2A6-68C2-3040-8098-70F65C3A49B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98B3CA0A-5160-5D49-AA92-91EAE213649B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2942" uniqueCount="1164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2978" uniqueCount="1173">
   <si>
     <t>Notes:</t>
   </si>
@@ -2635,18 +2635,12 @@
     <t>Soft Cotton Saree (with butterfly design on Pallu)</t>
   </si>
   <si>
-    <t>Latha(Yellow), Sari(Peach)</t>
-  </si>
-  <si>
     <t>CHR-148</t>
   </si>
   <si>
     <t>SAREES 5619 (Tissue Silk Saree Golden Color)</t>
   </si>
   <si>
-    <t>Chris (Goldern with flowers), Indu Varrier</t>
-  </si>
-  <si>
     <t>CHR-149</t>
   </si>
   <si>
@@ -2771,12 +2765,6 @@
   </si>
   <si>
     <t>Narayanpet sarees</t>
-  </si>
-  <si>
-    <t>Chithra- peacok blue, Indu Varier - Green, Susmi - Maroon, Jaimy - Purple/Bottle Green</t>
-  </si>
-  <si>
-    <t>Grey-Black/Red</t>
   </si>
   <si>
     <t>CHR-164</t>
@@ -3324,12 +3312,6 @@
   </si>
   <si>
     <t>Net Kota Stairs</t>
-  </si>
-  <si>
-    <t>Mustard, navy, rani pink, olive green (×2)</t>
-  </si>
-  <si>
-    <t>purple - Malini</t>
   </si>
   <si>
     <t>Linu Goerge</t>
@@ -3508,12 +3490,6 @@
     <t>CHR-187 - Banarasi Silk (Golden Yellow Blue)</t>
   </si>
   <si>
-    <t>mustard/blue, golden yellow &amp; green triangle</t>
-  </si>
-  <si>
-    <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim, Rust Orange/Coffee Brown - Nishida, Chikku Maroon(1200) - Nishida, Komalavalli - Red/green, peacock blue/navy - returned</t>
-  </si>
-  <si>
     <t>CHR-76 (XXL Plus white salwar) - 1100 advance, 200 balance</t>
   </si>
   <si>
@@ -3529,9 +3505,6 @@
     <t>Urmila</t>
   </si>
   <si>
-    <t>Sheeba George, Soji Thomas, Jessy Joseph, Jeeja Anil ,Sanam, Geetha, Sushama Bhaskar, Divya Jacob, Baby Johny, Jayasree, Navya, Bindu Saji, Vanajakshi, Dison Jose, Akshitha, Bahuleyan, Urmila</t>
-  </si>
-  <si>
     <t>Preeha Rajeevan</t>
   </si>
   <si>
@@ -3557,6 +3530,60 @@
   </si>
   <si>
     <t>Green, Pink, Yellow</t>
+  </si>
+  <si>
+    <t>Gincy Jibi</t>
+  </si>
+  <si>
+    <t>Sheeba George, Soji Thomas, Jessy Joseph, Jeeja Anil ,Sanam, Geetha, Sushama Bhaskar, Divya Jacob, Baby Johny, Jayasree, Navya, Bindu Saji, Vanajakshi, Dison Jose, Akshitha, Bahuleyan, Urmila, Gincy Jibi, Razia Salim</t>
+  </si>
+  <si>
+    <t>Green/maroon - Rajitha Teacher,  chikku green - Razia Salim, Rust Orange/Coffee Brown - Nishida, Chikku Maroon(1200) - Nishida, Komalavalli - Red/green, peacock blue/navy - returned, mustard/blue - girija(1200)</t>
+  </si>
+  <si>
+    <t>Golden yellow &amp; green triangle, Red &amp; Green</t>
+  </si>
+  <si>
+    <t>mustard/blue CHR-188</t>
+  </si>
+  <si>
+    <t>Courier Charges</t>
+  </si>
+  <si>
+    <t>Butter paper, courier covers etc</t>
+  </si>
+  <si>
+    <t>Sticker</t>
+  </si>
+  <si>
+    <t>Latha(Yellow), Sari(Peach),</t>
+  </si>
+  <si>
+    <t>Chris (Goldern with flowers), Indu Varrier, Nalini</t>
+  </si>
+  <si>
+    <t>CHR-205 Matka, CHR-148 Tissue</t>
+  </si>
+  <si>
+    <t>Linen Saree with elephant print</t>
+  </si>
+  <si>
+    <t>Latha - Red</t>
+  </si>
+  <si>
+    <t>yellow(4), red, Green, blue, purple</t>
+  </si>
+  <si>
+    <t>purple - Malini, Olive green - Latha</t>
+  </si>
+  <si>
+    <t>Navy, rani pink, olive green(2)</t>
+  </si>
+  <si>
+    <t>Chithra- peacok blue, Indu Varier - Green, Susmi - Maroon, Jaimy - Purple/Bottle Green, Latha - Grey</t>
+  </si>
+  <si>
+    <t>CHR-212-Red, CHR-195-Mustard,CHR-163 -Grey Narayanpet</t>
   </si>
 </sst>
 </file>
@@ -4436,7 +4463,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>274</c:v>
+                  <c:v>281</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>95</c:v>
@@ -4539,7 +4566,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>147</c:v>
+                  <c:v>152</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>53</c:v>
@@ -4872,7 +4899,7 @@
                   <c:v>56434</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>115064.43</c:v>
+                  <c:v>116473.43</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>590</c:v>
@@ -5205,7 +5232,7 @@
                   <c:v>99043</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>63028</c:v>
+                  <c:v>64662</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5365,7 +5392,7 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>31147</c:v>
+                  <c:v>40807</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5805,7 +5832,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-31881</c:v>
+                  <c:v>-23855</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6269,10 +6296,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>374</c:v>
+                  <c:v>381</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-281</c:v>
+                  <c:v>-248</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7444,7 +7471,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>517175</v>
+        <v>518809</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7459,7 +7486,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>449715</v>
+        <v>459375</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7476,7 +7503,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>459645</v>
+        <v>469305</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7493,7 +7520,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-67460</v>
+        <v>-59434</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7528,7 +7555,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>57412.993333333347</v>
+        <v>58502.32666666666</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7538,7 +7565,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>22436.003333333341</v>
+        <v>21891.336666666655</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7548,7 +7575,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-79848.996666666659</v>
+        <v>-80393.663333333345</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7587,15 +7614,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>248108</v>
+        <v>249742</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>172391.66666666666</v>
+        <v>172936.33333333334</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>75716.333333333343</v>
+        <v>76805.666666666657</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7603,11 +7630,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>57412.993333333347</v>
+        <v>58502.32666666666</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹57,413</v>
+        <v>Receive ₹58,502</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7621,11 +7648,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>172391.66666666666</v>
+        <v>172936.33333333334</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>64075.333333333343</v>
+        <v>63530.666666666657</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7633,11 +7660,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>22436.003333333341</v>
+        <v>21891.336666666655</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹22,436</v>
+        <v>Receive ₹21,891</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7651,11 +7678,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>172391.66666666666</v>
+        <v>172936.33333333334</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-139791.66666666666</v>
+        <v>-140336.33333333334</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7663,11 +7690,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-79848.996666666659</v>
+        <v>-80393.663333333345</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹79,849</v>
+        <v>Pay ₹80,394</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7705,15 +7732,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>382561</v>
+        <v>392221</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>149934.981</v>
+        <v>153155.625</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>232626.019</v>
+        <v>239065.375</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7721,11 +7748,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>95315.992999999988</v>
+        <v>101755.34899999999</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹95,316</v>
+        <v>Pay ₹101,755</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7739,11 +7766,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>149845.038</v>
+        <v>153063.75</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-95221.038</v>
+        <v>-98439.75</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7751,11 +7778,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-23633.995999999999</v>
+        <v>-26852.707999999999</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹23,634</v>
+        <v>Receive ₹26,853</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7769,11 +7796,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>149934.981</v>
+        <v>153155.625</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-137404.981</v>
+        <v>-140625.625</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7781,11 +7808,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-71681.996999999988</v>
+        <v>-74902.640999999989</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹71,682</v>
+        <v>Receive ₹74,903</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7897,7 +7924,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46217</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7906,14 +7933,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>517175</v>
+        <v>518809</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>449715</v>
+        <v>459375</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7922,14 +7949,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-67460</v>
+        <v>-59434</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>162467.63</v>
+        <v>163876.63</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -7981,7 +8008,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>374</v>
+        <v>381</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8005,7 +8032,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>-281</v>
+        <v>-248</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8082,15 +8109,15 @@
       </c>
       <c r="B16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A16)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>63028</v>
+        <v>64662</v>
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$995,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$995)=$B$7)*Sales!$C$2:$C$995),0)</f>
-        <v>31147</v>
+        <v>40807</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-31881</v>
+        <v>-23855</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8201,11 +8228,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8232,7 +8259,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>115064.43</v>
+        <v>116473.43</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9605,7 +9632,7 @@
         <v>28526</v>
       </c>
       <c r="D91" s="39" t="s">
-        <v>1120</v>
+        <v>1114</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" customHeight="1">
@@ -9665,22 +9692,46 @@
       </c>
     </row>
     <row r="96" spans="1:4" ht="15" customHeight="1">
-      <c r="A96" s="35"/>
-      <c r="B96" s="36"/>
-      <c r="C96" s="37"/>
-      <c r="D96" s="36"/>
+      <c r="A96" s="35">
+        <v>46217</v>
+      </c>
+      <c r="B96" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C96" s="37">
+        <v>70</v>
+      </c>
+      <c r="D96" s="36" t="s">
+        <v>1160</v>
+      </c>
     </row>
     <row r="97" spans="1:4" ht="15" customHeight="1">
-      <c r="A97" s="38"/>
-      <c r="B97" s="39"/>
-      <c r="C97" s="40"/>
-      <c r="D97" s="39"/>
+      <c r="A97" s="38">
+        <v>46218</v>
+      </c>
+      <c r="B97" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C97" s="40">
+        <v>1375</v>
+      </c>
+      <c r="D97" s="39" t="s">
+        <v>1161</v>
+      </c>
     </row>
     <row r="98" spans="1:4" ht="15" customHeight="1">
-      <c r="A98" s="35"/>
-      <c r="B98" s="36"/>
-      <c r="C98" s="37"/>
-      <c r="D98" s="36"/>
+      <c r="A98" s="35">
+        <v>46219</v>
+      </c>
+      <c r="B98" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C98" s="37">
+        <v>189</v>
+      </c>
+      <c r="D98" s="36" t="s">
+        <v>1162</v>
+      </c>
     </row>
     <row r="99" spans="1:4" ht="15" customHeight="1">
       <c r="A99" s="38"/>
@@ -17118,7 +17169,7 @@
       <c r="F216" s="56"/>
       <c r="G216" s="56"/>
       <c r="H216" s="57" t="s">
-        <v>1105</v>
+        <v>1099</v>
       </c>
       <c r="I216" s="53" t="s">
         <v>148</v>
@@ -17943,7 +17994,7 @@
       <c r="F249" s="56"/>
       <c r="G249" s="56"/>
       <c r="H249" s="57" t="s">
-        <v>1085</v>
+        <v>1081</v>
       </c>
       <c r="I249" s="53" t="s">
         <v>148</v>
@@ -17964,7 +18015,7 @@
       <c r="F250" s="49"/>
       <c r="G250" s="49"/>
       <c r="H250" s="51" t="s">
-        <v>1087</v>
+        <v>1083</v>
       </c>
       <c r="I250" s="49" t="s">
         <v>356</v>
@@ -17975,7 +18026,7 @@
         <v>46201</v>
       </c>
       <c r="B251" s="53" t="s">
-        <v>1106</v>
+        <v>1100</v>
       </c>
       <c r="C251" s="54">
         <v>1380</v>
@@ -18000,7 +18051,7 @@
         <v>46201</v>
       </c>
       <c r="B252" s="49" t="s">
-        <v>1090</v>
+        <v>1084</v>
       </c>
       <c r="C252" s="50">
         <v>699</v>
@@ -18014,7 +18065,7 @@
       <c r="F252" s="49"/>
       <c r="G252" s="49"/>
       <c r="H252" s="51" t="s">
-        <v>1091</v>
+        <v>1085</v>
       </c>
       <c r="I252" s="49" t="s">
         <v>148</v>
@@ -18025,7 +18076,7 @@
         <v>46201</v>
       </c>
       <c r="B253" s="53" t="s">
-        <v>1092</v>
+        <v>1086</v>
       </c>
       <c r="C253" s="54">
         <v>699</v>
@@ -18039,7 +18090,7 @@
       <c r="F253" s="56"/>
       <c r="G253" s="56"/>
       <c r="H253" s="57" t="s">
-        <v>1093</v>
+        <v>1087</v>
       </c>
       <c r="I253" s="53" t="s">
         <v>148</v>
@@ -18050,7 +18101,7 @@
         <v>46201</v>
       </c>
       <c r="B254" s="49" t="s">
-        <v>1094</v>
+        <v>1088</v>
       </c>
       <c r="C254" s="50">
         <v>699</v>
@@ -18064,7 +18115,7 @@
       <c r="F254" s="49"/>
       <c r="G254" s="49"/>
       <c r="H254" s="51" t="s">
-        <v>1095</v>
+        <v>1089</v>
       </c>
       <c r="I254" s="49" t="s">
         <v>148</v>
@@ -18089,7 +18140,7 @@
       <c r="F255" s="56"/>
       <c r="G255" s="56"/>
       <c r="H255" s="57" t="s">
-        <v>1098</v>
+        <v>1092</v>
       </c>
       <c r="I255" s="53" t="s">
         <v>148</v>
@@ -18100,7 +18151,7 @@
         <v>46203</v>
       </c>
       <c r="B256" s="49" t="s">
-        <v>1107</v>
+        <v>1101</v>
       </c>
       <c r="C256" s="50">
         <v>950</v>
@@ -18114,7 +18165,7 @@
       <c r="F256" s="49"/>
       <c r="G256" s="49"/>
       <c r="H256" s="51" t="s">
-        <v>1108</v>
+        <v>1102</v>
       </c>
       <c r="I256" s="49" t="s">
         <v>148</v>
@@ -18125,7 +18176,7 @@
         <v>46204</v>
       </c>
       <c r="B257" s="53" t="s">
-        <v>1111</v>
+        <v>1105</v>
       </c>
       <c r="C257" s="54">
         <v>699</v>
@@ -18139,7 +18190,7 @@
       <c r="F257" s="56"/>
       <c r="G257" s="56"/>
       <c r="H257" s="57" t="s">
-        <v>1112</v>
+        <v>1106</v>
       </c>
       <c r="I257" s="53" t="s">
         <v>148</v>
@@ -18150,7 +18201,7 @@
         <v>46205</v>
       </c>
       <c r="B258" s="49" t="s">
-        <v>1113</v>
+        <v>1107</v>
       </c>
       <c r="C258" s="50">
         <v>1500</v>
@@ -18164,7 +18215,7 @@
       <c r="F258" s="49"/>
       <c r="G258" s="49"/>
       <c r="H258" s="51" t="s">
-        <v>1114</v>
+        <v>1108</v>
       </c>
       <c r="I258" s="49" t="s">
         <v>148</v>
@@ -18175,7 +18226,7 @@
         <v>46205</v>
       </c>
       <c r="B259" s="53" t="s">
-        <v>1113</v>
+        <v>1107</v>
       </c>
       <c r="C259" s="54">
         <v>1200</v>
@@ -18189,7 +18240,7 @@
       <c r="F259" s="56"/>
       <c r="G259" s="56"/>
       <c r="H259" s="57" t="s">
-        <v>1117</v>
+        <v>1111</v>
       </c>
       <c r="I259" s="53" t="s">
         <v>148</v>
@@ -18200,7 +18251,7 @@
         <v>46205</v>
       </c>
       <c r="B260" s="49" t="s">
-        <v>1119</v>
+        <v>1113</v>
       </c>
       <c r="C260" s="50">
         <v>1500</v>
@@ -18214,7 +18265,7 @@
       <c r="F260" s="49"/>
       <c r="G260" s="49"/>
       <c r="H260" s="51" t="s">
-        <v>1118</v>
+        <v>1112</v>
       </c>
       <c r="I260" s="49" t="s">
         <v>148</v>
@@ -18225,7 +18276,7 @@
         <v>46205</v>
       </c>
       <c r="B261" s="53" t="s">
-        <v>1122</v>
+        <v>1116</v>
       </c>
       <c r="C261" s="54">
         <v>1900</v>
@@ -18235,7 +18286,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1151</v>
+        <v>1143</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>356</v>
@@ -18246,7 +18297,7 @@
         <v>46206</v>
       </c>
       <c r="B262" s="49" t="s">
-        <v>1127</v>
+        <v>1121</v>
       </c>
       <c r="C262" s="50">
         <v>1380</v>
@@ -18271,7 +18322,7 @@
         <v>46206</v>
       </c>
       <c r="B263" s="53" t="s">
-        <v>1128</v>
+        <v>1122</v>
       </c>
       <c r="C263" s="54">
         <v>1380</v>
@@ -18296,7 +18347,7 @@
         <v>46206</v>
       </c>
       <c r="B264" s="49" t="s">
-        <v>1139</v>
+        <v>1133</v>
       </c>
       <c r="C264" s="50">
         <v>2500</v>
@@ -18310,7 +18361,7 @@
       <c r="F264" s="49"/>
       <c r="G264" s="49"/>
       <c r="H264" s="51" t="s">
-        <v>1140</v>
+        <v>1134</v>
       </c>
       <c r="I264" s="49" t="s">
         <v>356</v>
@@ -18321,7 +18372,7 @@
         <v>46206</v>
       </c>
       <c r="B265" s="53" t="s">
-        <v>1131</v>
+        <v>1125</v>
       </c>
       <c r="C265" s="54">
         <v>1300</v>
@@ -18335,7 +18386,7 @@
       <c r="F265" s="56"/>
       <c r="G265" s="56"/>
       <c r="H265" s="57" t="s">
-        <v>1149</v>
+        <v>1141</v>
       </c>
       <c r="I265" s="53" t="s">
         <v>356</v>
@@ -18346,7 +18397,7 @@
         <v>46206</v>
       </c>
       <c r="B266" s="49" t="s">
-        <v>1119</v>
+        <v>1113</v>
       </c>
       <c r="C266" s="50">
         <v>1380</v>
@@ -18360,7 +18411,7 @@
       <c r="F266" s="49"/>
       <c r="G266" s="49"/>
       <c r="H266" s="51" t="s">
-        <v>1132</v>
+        <v>1126</v>
       </c>
       <c r="I266" s="49" t="s">
         <v>148</v>
@@ -18385,7 +18436,7 @@
       <c r="F267" s="56"/>
       <c r="G267" s="56"/>
       <c r="H267" s="57" t="s">
-        <v>1133</v>
+        <v>1127</v>
       </c>
       <c r="I267" s="53" t="s">
         <v>148</v>
@@ -18396,7 +18447,7 @@
         <v>46208</v>
       </c>
       <c r="B268" s="49" t="s">
-        <v>1138</v>
+        <v>1132</v>
       </c>
       <c r="C268" s="50">
         <v>2350</v>
@@ -18406,7 +18457,7 @@
       <c r="F268" s="49"/>
       <c r="G268" s="49"/>
       <c r="H268" s="51" t="s">
-        <v>1150</v>
+        <v>1142</v>
       </c>
       <c r="I268" s="49" t="s">
         <v>356</v>
@@ -18417,7 +18468,7 @@
         <v>46209</v>
       </c>
       <c r="B269" s="53" t="s">
-        <v>1136</v>
+        <v>1130</v>
       </c>
       <c r="C269" s="54">
         <v>1100</v>
@@ -18431,7 +18482,7 @@
       <c r="F269" s="56"/>
       <c r="G269" s="56"/>
       <c r="H269" s="57" t="s">
-        <v>1137</v>
+        <v>1131</v>
       </c>
       <c r="I269" s="53" t="s">
         <v>148</v>
@@ -18442,7 +18493,7 @@
         <v>46210</v>
       </c>
       <c r="B270" s="49" t="s">
-        <v>1143</v>
+        <v>1137</v>
       </c>
       <c r="C270" s="50">
         <v>3200</v>
@@ -18456,7 +18507,7 @@
       <c r="F270" s="49"/>
       <c r="G270" s="49"/>
       <c r="H270" s="51" t="s">
-        <v>1144</v>
+        <v>1138</v>
       </c>
       <c r="I270" s="49" t="s">
         <v>148</v>
@@ -18467,7 +18518,7 @@
         <v>46211</v>
       </c>
       <c r="B271" s="53" t="s">
-        <v>1145</v>
+        <v>1139</v>
       </c>
       <c r="C271" s="54">
         <v>1380</v>
@@ -18481,7 +18532,7 @@
       <c r="F271" s="56"/>
       <c r="G271" s="56"/>
       <c r="H271" s="57" t="s">
-        <v>1146</v>
+        <v>1140</v>
       </c>
       <c r="I271" s="53" t="s">
         <v>148</v>
@@ -18492,7 +18543,7 @@
         <v>46215</v>
       </c>
       <c r="B272" s="49" t="s">
-        <v>1153</v>
+        <v>1145</v>
       </c>
       <c r="C272" s="50">
         <v>1380</v>
@@ -18517,7 +18568,7 @@
         <v>46215</v>
       </c>
       <c r="B273" s="53" t="s">
-        <v>1155</v>
+        <v>1146</v>
       </c>
       <c r="C273" s="54">
         <v>699</v>
@@ -18531,7 +18582,7 @@
       <c r="F273" s="56"/>
       <c r="G273" s="56"/>
       <c r="H273" s="57" t="s">
-        <v>1112</v>
+        <v>1106</v>
       </c>
       <c r="I273" s="53" t="s">
         <v>148</v>
@@ -18556,7 +18607,7 @@
       <c r="F274" s="49"/>
       <c r="G274" s="49"/>
       <c r="H274" s="51" t="s">
-        <v>1157</v>
+        <v>1148</v>
       </c>
       <c r="I274" s="49" t="s">
         <v>148</v>
@@ -18567,7 +18618,7 @@
         <v>46216</v>
       </c>
       <c r="B275" s="53" t="s">
-        <v>1158</v>
+        <v>1149</v>
       </c>
       <c r="C275" s="54">
         <v>699</v>
@@ -18581,7 +18632,7 @@
       <c r="F275" s="56"/>
       <c r="G275" s="56"/>
       <c r="H275" s="57" t="s">
-        <v>1112</v>
+        <v>1106</v>
       </c>
       <c r="I275" s="53" t="s">
         <v>148</v>
@@ -18592,7 +18643,7 @@
         <v>46216</v>
       </c>
       <c r="B276" s="49" t="s">
-        <v>1161</v>
+        <v>1152</v>
       </c>
       <c r="C276" s="50">
         <v>3000</v>
@@ -18606,66 +18657,136 @@
       <c r="F276" s="49"/>
       <c r="G276" s="49"/>
       <c r="H276" s="51" t="s">
-        <v>1160</v>
+        <v>1151</v>
       </c>
       <c r="I276" s="49" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="277" spans="1:9">
-      <c r="A277" s="52"/>
-      <c r="B277" s="53"/>
-      <c r="C277" s="54"/>
-      <c r="D277" s="53"/>
-      <c r="E277" s="53"/>
+    <row r="277" spans="1:9" ht="14">
+      <c r="A277" s="52">
+        <v>46219</v>
+      </c>
+      <c r="B277" s="53" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C277" s="54">
+        <v>1380</v>
+      </c>
+      <c r="D277" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E277" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F277" s="56"/>
       <c r="G277" s="56"/>
-      <c r="H277" s="57"/>
-      <c r="I277" s="53"/>
-    </row>
-    <row r="278" spans="1:9">
-      <c r="A278" s="48"/>
-      <c r="B278" s="49"/>
-      <c r="C278" s="50"/>
-      <c r="D278" s="49"/>
-      <c r="E278" s="49"/>
+      <c r="H277" s="57" t="s">
+        <v>366</v>
+      </c>
+      <c r="I277" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="278" spans="1:9" ht="14">
+      <c r="A278" s="48">
+        <v>46219</v>
+      </c>
+      <c r="B278" s="49" t="s">
+        <v>482</v>
+      </c>
+      <c r="C278" s="50">
+        <v>1380</v>
+      </c>
+      <c r="D278" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E278" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F278" s="49"/>
       <c r="G278" s="49"/>
-      <c r="H278" s="51"/>
-      <c r="I278" s="49"/>
-    </row>
-    <row r="279" spans="1:9">
-      <c r="A279" s="52"/>
-      <c r="B279" s="53"/>
-      <c r="C279" s="54"/>
-      <c r="D279" s="53"/>
-      <c r="E279" s="53"/>
+      <c r="H278" s="51" t="s">
+        <v>366</v>
+      </c>
+      <c r="I278" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="279" spans="1:9" ht="14">
+      <c r="A279" s="52">
+        <v>46219</v>
+      </c>
+      <c r="B279" s="53" t="s">
+        <v>224</v>
+      </c>
+      <c r="C279" s="54">
+        <v>1200</v>
+      </c>
+      <c r="D279" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E279" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F279" s="56"/>
       <c r="G279" s="56"/>
-      <c r="H279" s="57"/>
-      <c r="I279" s="53"/>
-    </row>
-    <row r="280" spans="1:9">
-      <c r="A280" s="48"/>
-      <c r="B280" s="49"/>
-      <c r="C280" s="50"/>
-      <c r="D280" s="49"/>
-      <c r="E280" s="49"/>
+      <c r="H279" s="57" t="s">
+        <v>1159</v>
+      </c>
+      <c r="I279" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="280" spans="1:9" ht="14">
+      <c r="A280" s="48">
+        <v>46219</v>
+      </c>
+      <c r="B280" s="49" t="s">
+        <v>220</v>
+      </c>
+      <c r="C280" s="50">
+        <v>2500</v>
+      </c>
+      <c r="D280" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E280" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F280" s="49"/>
       <c r="G280" s="49"/>
-      <c r="H280" s="51"/>
-      <c r="I280" s="49"/>
-    </row>
-    <row r="281" spans="1:9">
-      <c r="A281" s="52"/>
-      <c r="B281" s="53"/>
-      <c r="C281" s="54"/>
-      <c r="D281" s="53"/>
-      <c r="E281" s="53"/>
+      <c r="H280" s="51" t="s">
+        <v>1165</v>
+      </c>
+      <c r="I280" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="281" spans="1:9" ht="14">
+      <c r="A281" s="52">
+        <v>46219</v>
+      </c>
+      <c r="B281" s="53" t="s">
+        <v>153</v>
+      </c>
+      <c r="C281" s="54">
+        <v>3200</v>
+      </c>
+      <c r="D281" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E281" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F281" s="56"/>
       <c r="G281" s="56"/>
-      <c r="H281" s="57"/>
-      <c r="I281" s="53"/>
+      <c r="H281" s="57" t="s">
+        <v>1172</v>
+      </c>
+      <c r="I281" s="53" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="282" spans="1:9">
       <c r="A282" s="48"/>
@@ -25410,7 +25531,7 @@
         <v>1145</v>
       </c>
       <c r="L59" s="66" t="s">
-        <v>1141</v>
+        <v>1135</v>
       </c>
       <c r="M59" s="66"/>
       <c r="N59" s="66" t="s">
@@ -26956,7 +27077,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="63" t="s">
-        <v>1142</v>
+        <v>1136</v>
       </c>
       <c r="M88" s="63"/>
       <c r="N88" s="63" t="s">
@@ -27216,7 +27337,7 @@
         <v>0</v>
       </c>
       <c r="L93" s="66" t="s">
-        <v>1126</v>
+        <v>1120</v>
       </c>
       <c r="M93" s="66"/>
       <c r="N93" s="63" t="s">
@@ -28650,7 +28771,7 @@
         <v>1256.859999999999</v>
       </c>
       <c r="L120" s="63" t="s">
-        <v>1096</v>
+        <v>1090</v>
       </c>
       <c r="M120" s="63" t="s">
         <v>49</v>
@@ -28660,7 +28781,7 @@
       </c>
       <c r="O120" s="63"/>
       <c r="P120" s="63" t="s">
-        <v>1097</v>
+        <v>1091</v>
       </c>
       <c r="Q120" s="63"/>
       <c r="R120" s="63"/>
@@ -29758,7 +29879,7 @@
         <v>0</v>
       </c>
       <c r="L128" s="63" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
       <c r="M128" s="63"/>
       <c r="N128" s="63" t="s">
@@ -30740,7 +30861,7 @@
         <v>1438</v>
       </c>
       <c r="L147" s="66" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
       <c r="M147" s="66"/>
       <c r="N147" s="66" t="s">
@@ -30748,7 +30869,7 @@
       </c>
       <c r="O147" s="66"/>
       <c r="P147" s="66" t="s">
-        <v>1084</v>
+        <v>1080</v>
       </c>
       <c r="Q147" s="66"/>
       <c r="R147" s="66"/>
@@ -30772,10 +30893,10 @@
         <v>850</v>
       </c>
       <c r="F148" s="78">
+        <v>1</v>
+      </c>
+      <c r="G148" s="78">
         <v>2</v>
-      </c>
-      <c r="G148" s="78">
-        <v>1</v>
       </c>
       <c r="H148" s="77">
         <f t="shared" si="8"/>
@@ -30787,14 +30908,14 @@
       </c>
       <c r="J148" s="77">
         <f t="shared" si="9"/>
-        <v>1004</v>
+        <v>502</v>
       </c>
       <c r="K148" s="77">
         <f t="shared" si="10"/>
-        <v>502</v>
+        <v>1004</v>
       </c>
       <c r="L148" s="63" t="s">
-        <v>858</v>
+        <v>1163</v>
       </c>
       <c r="M148" s="63"/>
       <c r="N148" s="63" t="s">
@@ -30809,10 +30930,10 @@
     </row>
     <row r="149" spans="1:20" ht="15" customHeight="1">
       <c r="A149" s="66" t="s">
+        <v>858</v>
+      </c>
+      <c r="B149" s="66" t="s">
         <v>859</v>
-      </c>
-      <c r="B149" s="66" t="s">
-        <v>860</v>
       </c>
       <c r="C149" s="66" t="s">
         <v>95</v>
@@ -30824,10 +30945,10 @@
         <v>1450</v>
       </c>
       <c r="F149" s="76">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G149" s="76">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H149" s="75">
         <f t="shared" si="8"/>
@@ -30839,18 +30960,18 @@
       </c>
       <c r="J149" s="75">
         <f t="shared" si="9"/>
-        <v>2048</v>
+        <v>3072</v>
       </c>
       <c r="K149" s="75">
         <f t="shared" si="10"/>
-        <v>1024</v>
+        <v>0</v>
       </c>
       <c r="L149" s="66" t="s">
-        <v>861</v>
+        <v>1164</v>
       </c>
       <c r="M149" s="66"/>
       <c r="N149" s="66" t="s">
-        <v>589</v>
+        <v>504</v>
       </c>
       <c r="O149" s="66"/>
       <c r="P149" s="66"/>
@@ -30861,10 +30982,10 @@
     </row>
     <row r="150" spans="1:20" ht="15" customHeight="1">
       <c r="A150" s="63" t="s">
-        <v>862</v>
+        <v>860</v>
       </c>
       <c r="B150" s="63" t="s">
-        <v>863</v>
+        <v>861</v>
       </c>
       <c r="C150" s="63" t="s">
         <v>95</v>
@@ -30911,10 +31032,10 @@
     </row>
     <row r="151" spans="1:20" ht="15" customHeight="1">
       <c r="A151" s="66" t="s">
-        <v>864</v>
+        <v>862</v>
       </c>
       <c r="B151" s="66" t="s">
-        <v>865</v>
+        <v>863</v>
       </c>
       <c r="C151" s="66" t="s">
         <v>96</v>
@@ -30948,7 +31069,7 @@
         <v>645</v>
       </c>
       <c r="L151" s="66" t="s">
-        <v>866</v>
+        <v>864</v>
       </c>
       <c r="M151" s="66"/>
       <c r="N151" s="66" t="s">
@@ -30958,7 +31079,7 @@
         <v>216</v>
       </c>
       <c r="P151" s="66" t="s">
-        <v>867</v>
+        <v>865</v>
       </c>
       <c r="Q151" s="66"/>
       <c r="R151" s="66"/>
@@ -30967,10 +31088,10 @@
     </row>
     <row r="152" spans="1:20" ht="15" customHeight="1">
       <c r="A152" s="63" t="s">
-        <v>868</v>
+        <v>866</v>
       </c>
       <c r="B152" s="63" t="s">
-        <v>869</v>
+        <v>867</v>
       </c>
       <c r="C152" s="63" t="s">
         <v>97</v>
@@ -31004,17 +31125,17 @@
         <v>590</v>
       </c>
       <c r="L152" s="63" t="s">
-        <v>870</v>
+        <v>868</v>
       </c>
       <c r="M152" s="63"/>
       <c r="N152" s="63" t="s">
         <v>589</v>
       </c>
       <c r="O152" s="63" t="s">
-        <v>871</v>
+        <v>869</v>
       </c>
       <c r="P152" s="63" t="s">
-        <v>872</v>
+        <v>870</v>
       </c>
       <c r="Q152" s="63"/>
       <c r="R152" s="63"/>
@@ -31023,10 +31144,10 @@
     </row>
     <row r="153" spans="1:20" ht="15" customHeight="1">
       <c r="A153" s="66" t="s">
-        <v>873</v>
+        <v>871</v>
       </c>
       <c r="B153" s="66" t="s">
-        <v>874</v>
+        <v>872</v>
       </c>
       <c r="C153" s="66" t="s">
         <v>95</v>
@@ -31060,7 +31181,7 @@
         <v>0</v>
       </c>
       <c r="L153" s="66" t="s">
-        <v>875</v>
+        <v>873</v>
       </c>
       <c r="M153" s="66"/>
       <c r="N153" s="66" t="s">
@@ -31068,7 +31189,7 @@
       </c>
       <c r="O153" s="66"/>
       <c r="P153" s="66" t="s">
-        <v>876</v>
+        <v>874</v>
       </c>
       <c r="Q153" s="66"/>
       <c r="R153" s="66"/>
@@ -31077,10 +31198,10 @@
     </row>
     <row r="154" spans="1:20" ht="15" customHeight="1">
       <c r="A154" s="63" t="s">
-        <v>877</v>
+        <v>875</v>
       </c>
       <c r="B154" s="63" t="s">
-        <v>878</v>
+        <v>876</v>
       </c>
       <c r="C154" s="63" t="s">
         <v>96</v>
@@ -31114,14 +31235,14 @@
         <v>949</v>
       </c>
       <c r="L154" s="63" t="s">
-        <v>1129</v>
+        <v>1123</v>
       </c>
       <c r="M154" s="63"/>
       <c r="N154" s="63" t="s">
         <v>589</v>
       </c>
       <c r="O154" s="63" t="s">
-        <v>1125</v>
+        <v>1119</v>
       </c>
       <c r="P154" s="63"/>
       <c r="Q154" s="63"/>
@@ -31131,10 +31252,10 @@
     </row>
     <row r="155" spans="1:20" ht="15" customHeight="1">
       <c r="A155" s="66" t="s">
-        <v>879</v>
+        <v>877</v>
       </c>
       <c r="B155" s="66" t="s">
-        <v>880</v>
+        <v>878</v>
       </c>
       <c r="C155" s="66" t="s">
         <v>96</v>
@@ -31168,14 +31289,14 @@
         <v>949</v>
       </c>
       <c r="L155" s="66" t="s">
-        <v>1156</v>
+        <v>1147</v>
       </c>
       <c r="M155" s="66"/>
       <c r="N155" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O155" s="66" t="s">
-        <v>1125</v>
+        <v>1119</v>
       </c>
       <c r="P155" s="66"/>
       <c r="Q155" s="66"/>
@@ -31185,10 +31306,10 @@
     </row>
     <row r="156" spans="1:20" ht="15" customHeight="1">
       <c r="A156" s="63" t="s">
-        <v>881</v>
+        <v>879</v>
       </c>
       <c r="B156" s="63" t="s">
-        <v>882</v>
+        <v>880</v>
       </c>
       <c r="C156" s="63" t="s">
         <v>96</v>
@@ -31222,7 +31343,7 @@
         <v>1900</v>
       </c>
       <c r="L156" s="63" t="s">
-        <v>1130</v>
+        <v>1124</v>
       </c>
       <c r="M156" s="63"/>
       <c r="N156" s="63" t="s">
@@ -31239,10 +31360,10 @@
     </row>
     <row r="157" spans="1:20" ht="15" customHeight="1">
       <c r="A157" s="66" t="s">
-        <v>883</v>
+        <v>881</v>
       </c>
       <c r="B157" s="66" t="s">
-        <v>884</v>
+        <v>882</v>
       </c>
       <c r="C157" s="66" t="s">
         <v>96</v>
@@ -31276,7 +31397,7 @@
         <v>1050</v>
       </c>
       <c r="L157" s="66" t="s">
-        <v>885</v>
+        <v>883</v>
       </c>
       <c r="M157" s="66"/>
       <c r="N157" s="66" t="s">
@@ -31293,10 +31414,10 @@
     </row>
     <row r="158" spans="1:20" ht="15" customHeight="1">
       <c r="A158" s="63" t="s">
-        <v>886</v>
+        <v>884</v>
       </c>
       <c r="B158" s="63" t="s">
-        <v>887</v>
+        <v>885</v>
       </c>
       <c r="C158" s="63" t="s">
         <v>96</v>
@@ -31330,14 +31451,14 @@
         <v>3356</v>
       </c>
       <c r="L158" s="63" t="s">
-        <v>888</v>
+        <v>886</v>
       </c>
       <c r="M158" s="63"/>
       <c r="N158" s="63" t="s">
         <v>678</v>
       </c>
       <c r="O158" s="63" t="s">
-        <v>889</v>
+        <v>887</v>
       </c>
       <c r="P158" s="63"/>
       <c r="Q158" s="63"/>
@@ -31347,10 +31468,10 @@
     </row>
     <row r="159" spans="1:20" ht="15" customHeight="1">
       <c r="A159" s="66" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="B159" s="66" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="C159" s="66" t="s">
         <v>96</v>
@@ -31384,14 +31505,14 @@
         <v>2517</v>
       </c>
       <c r="L159" s="66" t="s">
-        <v>892</v>
+        <v>890</v>
       </c>
       <c r="M159" s="66"/>
       <c r="N159" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O159" s="66" t="s">
-        <v>893</v>
+        <v>891</v>
       </c>
       <c r="P159" s="66"/>
       <c r="Q159" s="66"/>
@@ -31401,10 +31522,10 @@
     </row>
     <row r="160" spans="1:20" ht="15" customHeight="1">
       <c r="A160" s="63" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="B160" s="63" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="C160" s="63" t="s">
         <v>95</v>
@@ -31453,10 +31574,10 @@
     </row>
     <row r="161" spans="1:20" ht="15" customHeight="1">
       <c r="A161" s="66" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="B161" s="66" t="s">
-        <v>897</v>
+        <v>895</v>
       </c>
       <c r="C161" s="66" t="s">
         <v>95</v>
@@ -31505,10 +31626,10 @@
     </row>
     <row r="162" spans="1:20" ht="15" customHeight="1">
       <c r="A162" s="63" t="s">
-        <v>898</v>
+        <v>896</v>
       </c>
       <c r="B162" s="63" t="s">
-        <v>899</v>
+        <v>897</v>
       </c>
       <c r="C162" s="63" t="s">
         <v>95</v>
@@ -31557,10 +31678,10 @@
     </row>
     <row r="163" spans="1:20" ht="15" customHeight="1">
       <c r="A163" s="66" t="s">
-        <v>900</v>
+        <v>898</v>
       </c>
       <c r="B163" s="66" t="s">
-        <v>901</v>
+        <v>899</v>
       </c>
       <c r="C163" s="66" t="s">
         <v>95</v>
@@ -31607,10 +31728,10 @@
     </row>
     <row r="164" spans="1:20" ht="60" customHeight="1">
       <c r="A164" s="63" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="B164" s="63" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="C164" s="63" t="s">
         <v>95</v>
@@ -31622,10 +31743,10 @@
         <v>1499</v>
       </c>
       <c r="F164" s="78">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G164" s="78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H164" s="77">
         <f t="shared" si="11"/>
@@ -31637,23 +31758,21 @@
       </c>
       <c r="J164" s="77">
         <f t="shared" si="9"/>
-        <v>4052</v>
+        <v>5065</v>
       </c>
       <c r="K164" s="77">
         <f t="shared" si="10"/>
-        <v>1013</v>
+        <v>0</v>
       </c>
       <c r="L164" s="63" t="s">
-        <v>904</v>
+        <v>1171</v>
       </c>
       <c r="M164" s="63"/>
       <c r="N164" s="63" t="s">
-        <v>589</v>
+        <v>504</v>
       </c>
       <c r="O164" s="63"/>
-      <c r="P164" s="63" t="s">
-        <v>905</v>
-      </c>
+      <c r="P164" s="63"/>
       <c r="Q164" s="63"/>
       <c r="R164" s="63"/>
       <c r="S164" s="63"/>
@@ -31661,10 +31780,10 @@
     </row>
     <row r="165" spans="1:20" ht="15" customHeight="1">
       <c r="A165" s="66" t="s">
-        <v>906</v>
+        <v>902</v>
       </c>
       <c r="B165" s="66" t="s">
-        <v>907</v>
+        <v>903</v>
       </c>
       <c r="C165" s="66" t="s">
         <v>95</v>
@@ -31706,7 +31825,7 @@
       </c>
       <c r="O165" s="66"/>
       <c r="P165" s="66" t="s">
-        <v>908</v>
+        <v>904</v>
       </c>
       <c r="Q165" s="66"/>
       <c r="R165" s="66"/>
@@ -31715,10 +31834,10 @@
     </row>
     <row r="166" spans="1:20" ht="15" customHeight="1">
       <c r="A166" s="63" t="s">
-        <v>909</v>
+        <v>905</v>
       </c>
       <c r="B166" s="63" t="s">
-        <v>910</v>
+        <v>906</v>
       </c>
       <c r="C166" s="63" t="s">
         <v>95</v>
@@ -31752,7 +31871,7 @@
         <v>1212</v>
       </c>
       <c r="L166" s="63" t="s">
-        <v>1109</v>
+        <v>1103</v>
       </c>
       <c r="M166" s="63"/>
       <c r="N166" s="63" t="s">
@@ -31760,7 +31879,7 @@
       </c>
       <c r="O166" s="63"/>
       <c r="P166" s="63" t="s">
-        <v>1110</v>
+        <v>1104</v>
       </c>
       <c r="Q166" s="63"/>
       <c r="R166" s="63"/>
@@ -31769,10 +31888,10 @@
     </row>
     <row r="167" spans="1:20" ht="15" customHeight="1">
       <c r="A167" s="66" t="s">
-        <v>911</v>
+        <v>907</v>
       </c>
       <c r="B167" s="66" t="s">
-        <v>912</v>
+        <v>908</v>
       </c>
       <c r="C167" s="66" t="s">
         <v>95</v>
@@ -31806,7 +31925,7 @@
         <v>2220</v>
       </c>
       <c r="L167" s="66" t="s">
-        <v>913</v>
+        <v>909</v>
       </c>
       <c r="M167" s="66"/>
       <c r="N167" s="66" t="s">
@@ -31814,7 +31933,7 @@
       </c>
       <c r="O167" s="66"/>
       <c r="P167" s="66" t="s">
-        <v>914</v>
+        <v>910</v>
       </c>
       <c r="Q167" s="66"/>
       <c r="R167" s="66"/>
@@ -31823,10 +31942,10 @@
     </row>
     <row r="168" spans="1:20" ht="15" customHeight="1">
       <c r="A168" s="63" t="s">
-        <v>915</v>
+        <v>911</v>
       </c>
       <c r="B168" s="63" t="s">
-        <v>916</v>
+        <v>912</v>
       </c>
       <c r="C168" s="63" t="s">
         <v>95</v>
@@ -31860,7 +31979,7 @@
         <v>1216</v>
       </c>
       <c r="L168" s="63" t="s">
-        <v>917</v>
+        <v>913</v>
       </c>
       <c r="M168" s="63"/>
       <c r="N168" s="63" t="s">
@@ -31868,7 +31987,7 @@
       </c>
       <c r="O168" s="63"/>
       <c r="P168" s="63" t="s">
-        <v>918</v>
+        <v>914</v>
       </c>
       <c r="Q168" s="63"/>
       <c r="R168" s="63"/>
@@ -31877,10 +31996,10 @@
     </row>
     <row r="169" spans="1:20" ht="15" customHeight="1">
       <c r="A169" s="66" t="s">
-        <v>919</v>
+        <v>915</v>
       </c>
       <c r="B169" s="66" t="s">
-        <v>920</v>
+        <v>916</v>
       </c>
       <c r="C169" s="66" t="s">
         <v>95</v>
@@ -31920,7 +32039,7 @@
       </c>
       <c r="O169" s="66"/>
       <c r="P169" s="66" t="s">
-        <v>921</v>
+        <v>917</v>
       </c>
       <c r="Q169" s="66"/>
       <c r="R169" s="66"/>
@@ -31929,10 +32048,10 @@
     </row>
     <row r="170" spans="1:20" ht="30" customHeight="1">
       <c r="A170" s="63" t="s">
-        <v>922</v>
+        <v>918</v>
       </c>
       <c r="B170" s="63" t="s">
-        <v>923</v>
+        <v>919</v>
       </c>
       <c r="C170" s="63" t="s">
         <v>95</v>
@@ -31966,7 +32085,7 @@
         <v>0</v>
       </c>
       <c r="L170" s="63" t="s">
-        <v>924</v>
+        <v>920</v>
       </c>
       <c r="M170" s="63"/>
       <c r="N170" s="63" t="s">
@@ -31974,7 +32093,7 @@
       </c>
       <c r="O170" s="63"/>
       <c r="P170" s="63" t="s">
-        <v>925</v>
+        <v>921</v>
       </c>
       <c r="Q170" s="63"/>
       <c r="R170" s="63"/>
@@ -31983,10 +32102,10 @@
     </row>
     <row r="171" spans="1:20" ht="31.5" customHeight="1">
       <c r="A171" s="66" t="s">
-        <v>926</v>
+        <v>922</v>
       </c>
       <c r="B171" s="63" t="s">
-        <v>927</v>
+        <v>923</v>
       </c>
       <c r="C171" s="66" t="s">
         <v>95</v>
@@ -32020,7 +32139,7 @@
         <v>0</v>
       </c>
       <c r="L171" s="66" t="s">
-        <v>928</v>
+        <v>924</v>
       </c>
       <c r="M171" s="66"/>
       <c r="N171" s="66" t="s">
@@ -32035,10 +32154,10 @@
     </row>
     <row r="172" spans="1:20" ht="15" customHeight="1">
       <c r="A172" s="63" t="s">
-        <v>929</v>
+        <v>925</v>
       </c>
       <c r="B172" s="63" t="s">
-        <v>930</v>
+        <v>926</v>
       </c>
       <c r="C172" s="63" t="s">
         <v>95</v>
@@ -32053,11 +32172,11 @@
         <v>2</v>
       </c>
       <c r="G172" s="78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H172" s="77">
         <f t="shared" si="11"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I172" s="77">
         <f>IF(D172&lt;&gt;"",D172,IFERROR(E172/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -32069,10 +32188,10 @@
       </c>
       <c r="K172" s="77">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1047</v>
       </c>
       <c r="L172" s="63" t="s">
-        <v>931</v>
+        <v>927</v>
       </c>
       <c r="M172" s="63"/>
       <c r="N172" s="63" t="s">
@@ -32087,10 +32206,10 @@
     </row>
     <row r="173" spans="1:20" ht="15" customHeight="1">
       <c r="A173" s="66" t="s">
-        <v>932</v>
+        <v>928</v>
       </c>
       <c r="B173" s="66" t="s">
-        <v>933</v>
+        <v>929</v>
       </c>
       <c r="C173" s="66" t="s">
         <v>95</v>
@@ -32139,10 +32258,10 @@
     </row>
     <row r="174" spans="1:20" ht="15" customHeight="1">
       <c r="A174" s="63" t="s">
-        <v>934</v>
+        <v>930</v>
       </c>
       <c r="B174" s="63" t="s">
-        <v>935</v>
+        <v>931</v>
       </c>
       <c r="C174" s="63" t="s">
         <v>95</v>
@@ -32176,7 +32295,7 @@
         <v>0</v>
       </c>
       <c r="L174" s="63" t="s">
-        <v>936</v>
+        <v>932</v>
       </c>
       <c r="M174" s="63"/>
       <c r="N174" s="63" t="s">
@@ -32191,10 +32310,10 @@
     </row>
     <row r="175" spans="1:20" ht="90" customHeight="1">
       <c r="A175" s="66" t="s">
-        <v>937</v>
+        <v>933</v>
       </c>
       <c r="B175" s="66" t="s">
-        <v>938</v>
+        <v>934</v>
       </c>
       <c r="C175" s="66" t="s">
         <v>95</v>
@@ -32228,7 +32347,7 @@
         <v>3491.25</v>
       </c>
       <c r="L175" s="66" t="s">
-        <v>1116</v>
+        <v>1110</v>
       </c>
       <c r="M175" s="66"/>
       <c r="N175" s="66" t="s">
@@ -32236,7 +32355,7 @@
       </c>
       <c r="O175" s="66"/>
       <c r="P175" s="66" t="s">
-        <v>1115</v>
+        <v>1109</v>
       </c>
       <c r="Q175" s="66"/>
       <c r="R175" s="66"/>
@@ -32245,10 +32364,10 @@
     </row>
     <row r="176" spans="1:20" ht="24" customHeight="1">
       <c r="A176" s="63" t="s">
-        <v>939</v>
+        <v>935</v>
       </c>
       <c r="B176" s="63" t="s">
-        <v>940</v>
+        <v>936</v>
       </c>
       <c r="C176" s="63" t="s">
         <v>95</v>
@@ -32282,7 +32401,7 @@
         <v>0</v>
       </c>
       <c r="L176" s="63" t="s">
-        <v>941</v>
+        <v>937</v>
       </c>
       <c r="M176" s="63"/>
       <c r="N176" s="63" t="s">
@@ -32297,10 +32416,10 @@
     </row>
     <row r="177" spans="1:20" ht="33.75" customHeight="1">
       <c r="A177" s="66" t="s">
-        <v>942</v>
+        <v>938</v>
       </c>
       <c r="B177" s="66" t="s">
-        <v>943</v>
+        <v>939</v>
       </c>
       <c r="C177" s="66" t="s">
         <v>95</v>
@@ -32334,7 +32453,7 @@
         <v>0</v>
       </c>
       <c r="L177" s="66" t="s">
-        <v>944</v>
+        <v>940</v>
       </c>
       <c r="M177" s="66"/>
       <c r="N177" s="66" t="s">
@@ -32342,7 +32461,7 @@
       </c>
       <c r="O177" s="66"/>
       <c r="P177" s="66" t="s">
-        <v>945</v>
+        <v>941</v>
       </c>
       <c r="Q177" s="66"/>
       <c r="R177" s="66"/>
@@ -32351,10 +32470,10 @@
     </row>
     <row r="178" spans="1:20" ht="15" customHeight="1">
       <c r="A178" s="63" t="s">
-        <v>946</v>
+        <v>942</v>
       </c>
       <c r="B178" s="63" t="s">
-        <v>947</v>
+        <v>943</v>
       </c>
       <c r="C178" s="63" t="s">
         <v>95</v>
@@ -32388,7 +32507,7 @@
         <v>0</v>
       </c>
       <c r="L178" s="63" t="s">
-        <v>948</v>
+        <v>944</v>
       </c>
       <c r="M178" s="63"/>
       <c r="N178" s="63" t="s">
@@ -32396,7 +32515,7 @@
       </c>
       <c r="O178" s="63"/>
       <c r="P178" s="63" t="s">
-        <v>949</v>
+        <v>945</v>
       </c>
       <c r="Q178" s="63"/>
       <c r="R178" s="63"/>
@@ -32405,10 +32524,10 @@
     </row>
     <row r="179" spans="1:20" ht="30" customHeight="1">
       <c r="A179" s="66" t="s">
-        <v>950</v>
+        <v>946</v>
       </c>
       <c r="B179" s="66" t="s">
-        <v>951</v>
+        <v>947</v>
       </c>
       <c r="C179" s="66" t="s">
         <v>95</v>
@@ -32442,7 +32561,7 @@
         <v>0</v>
       </c>
       <c r="L179" s="66" t="s">
-        <v>952</v>
+        <v>948</v>
       </c>
       <c r="M179" s="66"/>
       <c r="N179" s="66" t="s">
@@ -32450,7 +32569,7 @@
       </c>
       <c r="O179" s="66"/>
       <c r="P179" s="66" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
       <c r="Q179" s="66"/>
       <c r="R179" s="66"/>
@@ -32459,10 +32578,10 @@
     </row>
     <row r="180" spans="1:20" ht="33.75" customHeight="1">
       <c r="A180" s="63" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
       <c r="B180" s="63" t="s">
-        <v>955</v>
+        <v>951</v>
       </c>
       <c r="C180" s="63" t="s">
         <v>95</v>
@@ -32496,7 +32615,7 @@
         <v>0</v>
       </c>
       <c r="L180" s="63" t="s">
-        <v>956</v>
+        <v>952</v>
       </c>
       <c r="M180" s="63"/>
       <c r="N180" s="63" t="s">
@@ -32511,10 +32630,10 @@
     </row>
     <row r="181" spans="1:20" ht="15" customHeight="1">
       <c r="A181" s="66" t="s">
-        <v>957</v>
+        <v>953</v>
       </c>
       <c r="B181" s="66" t="s">
-        <v>958</v>
+        <v>954</v>
       </c>
       <c r="C181" s="66" t="s">
         <v>96</v>
@@ -32548,17 +32667,17 @@
         <v>3057</v>
       </c>
       <c r="L181" s="66" t="s">
-        <v>1123</v>
+        <v>1117</v>
       </c>
       <c r="M181" s="66"/>
       <c r="N181" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O181" s="66" t="s">
-        <v>1124</v>
+        <v>1118</v>
       </c>
       <c r="P181" s="66" t="s">
-        <v>959</v>
+        <v>955</v>
       </c>
       <c r="Q181" s="66"/>
       <c r="R181" s="66"/>
@@ -32567,10 +32686,10 @@
     </row>
     <row r="182" spans="1:20" ht="15" customHeight="1">
       <c r="A182" s="63" t="s">
-        <v>960</v>
+        <v>956</v>
       </c>
       <c r="B182" s="63" t="s">
-        <v>961</v>
+        <v>957</v>
       </c>
       <c r="C182" s="63" t="s">
         <v>95</v>
@@ -32610,7 +32729,7 @@
       </c>
       <c r="O182" s="63"/>
       <c r="P182" s="63" t="s">
-        <v>962</v>
+        <v>958</v>
       </c>
       <c r="Q182" s="63"/>
       <c r="R182" s="63"/>
@@ -32619,10 +32738,10 @@
     </row>
     <row r="183" spans="1:20" ht="15" customHeight="1">
       <c r="A183" s="66" t="s">
-        <v>963</v>
+        <v>959</v>
       </c>
       <c r="B183" s="66" t="s">
-        <v>964</v>
+        <v>960</v>
       </c>
       <c r="C183" s="66" t="s">
         <v>95</v>
@@ -32655,7 +32774,7 @@
         <v>2095</v>
       </c>
       <c r="L183" s="66" t="s">
-        <v>1159</v>
+        <v>1150</v>
       </c>
       <c r="M183" s="66"/>
       <c r="N183" s="66" t="s">
@@ -32670,10 +32789,10 @@
     </row>
     <row r="184" spans="1:20" ht="52" customHeight="1">
       <c r="A184" s="63" t="s">
-        <v>965</v>
+        <v>961</v>
       </c>
       <c r="B184" s="63" t="s">
-        <v>966</v>
+        <v>962</v>
       </c>
       <c r="C184" s="63" t="s">
         <v>95</v>
@@ -32685,10 +32804,10 @@
         <v>1380</v>
       </c>
       <c r="F184" s="78">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G184" s="78">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H184" s="77">
         <f t="shared" ref="H184:H226" si="12">F184+IF(LEN(G184)=0,0,G184)</f>
@@ -32700,14 +32819,14 @@
       </c>
       <c r="J184" s="77">
         <f t="shared" si="9"/>
-        <v>15147</v>
+        <v>16929</v>
       </c>
       <c r="K184" s="77">
         <f t="shared" si="10"/>
-        <v>2673</v>
+        <v>891</v>
       </c>
       <c r="L184" s="63" t="s">
-        <v>1154</v>
+        <v>1156</v>
       </c>
       <c r="M184" s="63"/>
       <c r="N184" s="63" t="s">
@@ -32722,10 +32841,10 @@
     </row>
     <row r="185" spans="1:20" ht="15" customHeight="1">
       <c r="A185" s="66" t="s">
-        <v>967</v>
+        <v>963</v>
       </c>
       <c r="B185" s="66" t="s">
-        <v>968</v>
+        <v>964</v>
       </c>
       <c r="C185" s="66" t="s">
         <v>95</v>
@@ -32759,7 +32878,7 @@
         <v>0</v>
       </c>
       <c r="L185" s="66" t="s">
-        <v>969</v>
+        <v>965</v>
       </c>
       <c r="M185" s="66"/>
       <c r="N185" s="66" t="s">
@@ -32774,7 +32893,7 @@
     </row>
     <row r="186" spans="1:20" ht="15" customHeight="1">
       <c r="A186" s="63" t="s">
-        <v>970</v>
+        <v>966</v>
       </c>
       <c r="B186" s="63" t="s">
         <v>790</v>
@@ -32824,10 +32943,10 @@
     </row>
     <row r="187" spans="1:20" ht="15" customHeight="1">
       <c r="A187" s="66" t="s">
-        <v>971</v>
+        <v>967</v>
       </c>
       <c r="B187" s="66" t="s">
-        <v>972</v>
+        <v>968</v>
       </c>
       <c r="C187" s="66" t="s">
         <v>95</v>
@@ -32874,10 +32993,10 @@
     </row>
     <row r="188" spans="1:20" ht="15" customHeight="1">
       <c r="A188" s="63" t="s">
-        <v>973</v>
+        <v>969</v>
       </c>
       <c r="B188" s="63" t="s">
-        <v>974</v>
+        <v>970</v>
       </c>
       <c r="C188" s="63" t="s">
         <v>95</v>
@@ -32911,7 +33030,7 @@
         <v>0</v>
       </c>
       <c r="L188" s="63" t="s">
-        <v>1152</v>
+        <v>1144</v>
       </c>
       <c r="M188" s="63"/>
       <c r="N188" s="63" t="s">
@@ -32926,10 +33045,10 @@
     </row>
     <row r="189" spans="1:20" ht="52" customHeight="1">
       <c r="A189" s="66" t="s">
-        <v>975</v>
+        <v>971</v>
       </c>
       <c r="B189" s="63" t="s">
-        <v>976</v>
+        <v>972</v>
       </c>
       <c r="C189" s="63" t="s">
         <v>95</v>
@@ -32941,14 +33060,14 @@
         <v>1380</v>
       </c>
       <c r="F189" s="76">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G189" s="76">
         <v>2</v>
       </c>
       <c r="H189" s="75">
         <f t="shared" si="12"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I189" s="75">
         <f>IF(D189&lt;&gt;"",D189,IFERROR(E189/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -32956,14 +33075,14 @@
       </c>
       <c r="J189" s="75">
         <f t="shared" si="9"/>
-        <v>4455</v>
+        <v>5346</v>
       </c>
       <c r="K189" s="75">
         <f t="shared" si="10"/>
         <v>1782</v>
       </c>
       <c r="L189" s="66" t="s">
-        <v>1148</v>
+        <v>1157</v>
       </c>
       <c r="M189" s="66"/>
       <c r="N189" s="66" t="s">
@@ -32971,7 +33090,7 @@
       </c>
       <c r="O189" s="66"/>
       <c r="P189" s="66" t="s">
-        <v>1147</v>
+        <v>1158</v>
       </c>
       <c r="Q189" s="66"/>
       <c r="R189" s="66"/>
@@ -32980,10 +33099,10 @@
     </row>
     <row r="190" spans="1:20" ht="15" customHeight="1">
       <c r="A190" s="63" t="s">
-        <v>977</v>
+        <v>973</v>
       </c>
       <c r="B190" s="66" t="s">
-        <v>978</v>
+        <v>974</v>
       </c>
       <c r="C190" s="66" t="s">
         <v>95</v>
@@ -33019,20 +33138,20 @@
       <c r="L190" s="63"/>
       <c r="M190" s="63"/>
       <c r="N190" s="58" t="s">
-        <v>979</v>
+        <v>975</v>
       </c>
       <c r="P190" s="58" t="s">
-        <v>980</v>
+        <v>976</v>
       </c>
       <c r="S190" s="58"/>
       <c r="T190" s="58"/>
     </row>
     <row r="191" spans="1:20" ht="30" customHeight="1">
       <c r="A191" s="66" t="s">
-        <v>981</v>
+        <v>977</v>
       </c>
       <c r="B191" s="63" t="s">
-        <v>982</v>
+        <v>978</v>
       </c>
       <c r="C191" s="63" t="s">
         <v>95</v>
@@ -33071,17 +33190,17 @@
         <v>678</v>
       </c>
       <c r="P191" s="58" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="S191" s="58"/>
       <c r="T191" s="58"/>
     </row>
     <row r="192" spans="1:20" ht="15" customHeight="1">
       <c r="A192" s="63" t="s">
-        <v>984</v>
+        <v>980</v>
       </c>
       <c r="B192" s="66" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
       <c r="C192" s="66" t="s">
         <v>95</v>
@@ -33115,24 +33234,24 @@
         <v>1616</v>
       </c>
       <c r="L192" s="63" t="s">
-        <v>1099</v>
+        <v>1093</v>
       </c>
       <c r="M192" s="63"/>
       <c r="N192" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P192" s="58" t="s">
-        <v>1100</v>
+        <v>1094</v>
       </c>
       <c r="S192" s="58"/>
       <c r="T192" s="58"/>
     </row>
     <row r="193" spans="1:20" ht="15" customHeight="1">
       <c r="A193" s="66" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
       <c r="B193" s="63" t="s">
-        <v>987</v>
+        <v>983</v>
       </c>
       <c r="C193" s="63" t="s">
         <v>95</v>
@@ -33171,17 +33290,17 @@
         <v>678</v>
       </c>
       <c r="P193" s="58" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="S193" s="58"/>
       <c r="T193" s="58"/>
     </row>
     <row r="194" spans="1:20" ht="15" customHeight="1">
       <c r="A194" s="63" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="B194" s="63" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="C194" s="63" t="s">
         <v>95</v>
@@ -33220,17 +33339,17 @@
         <v>678</v>
       </c>
       <c r="P194" s="58" t="s">
-        <v>991</v>
+        <v>987</v>
       </c>
       <c r="S194" s="58"/>
       <c r="T194" s="58"/>
     </row>
     <row r="195" spans="1:20" ht="15" customHeight="1">
       <c r="A195" s="66" t="s">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="B195" s="66" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="C195" s="66" t="s">
         <v>95</v>
@@ -33264,24 +33383,24 @@
         <v>5467</v>
       </c>
       <c r="L195" s="66" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="M195" s="66"/>
       <c r="N195" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P195" s="58" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
       <c r="S195" s="58"/>
       <c r="T195" s="58"/>
     </row>
     <row r="196" spans="1:20" ht="15" customHeight="1">
       <c r="A196" s="63" t="s">
-        <v>996</v>
+        <v>992</v>
       </c>
       <c r="B196" s="63" t="s">
-        <v>997</v>
+        <v>993</v>
       </c>
       <c r="C196" s="63" t="s">
         <v>95</v>
@@ -33293,14 +33412,14 @@
         <v>1250</v>
       </c>
       <c r="F196" s="78">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G196" s="78">
         <v>5</v>
       </c>
       <c r="H196" s="77">
         <f t="shared" si="12"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I196" s="77">
         <f>IF(D196&lt;&gt;"",D196,IFERROR(E196/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -33308,31 +33427,31 @@
       </c>
       <c r="J196" s="77">
         <f t="shared" si="13"/>
-        <v>797</v>
+        <v>1594</v>
       </c>
       <c r="K196" s="77">
         <f t="shared" si="14"/>
         <v>3985</v>
       </c>
       <c r="L196" s="63" t="s">
-        <v>1089</v>
+        <v>1169</v>
       </c>
       <c r="M196" s="63"/>
       <c r="N196" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P196" s="58" t="s">
-        <v>1088</v>
+        <v>1170</v>
       </c>
       <c r="S196" s="58"/>
       <c r="T196" s="58"/>
     </row>
     <row r="197" spans="1:20" ht="15" customHeight="1">
       <c r="A197" s="66" t="s">
-        <v>998</v>
+        <v>994</v>
       </c>
       <c r="B197" s="66" t="s">
-        <v>999</v>
+        <v>995</v>
       </c>
       <c r="C197" s="66" t="s">
         <v>95</v>
@@ -33371,17 +33490,17 @@
         <v>678</v>
       </c>
       <c r="P197" s="58" t="s">
-        <v>1000</v>
+        <v>996</v>
       </c>
       <c r="S197" s="58"/>
       <c r="T197" s="58"/>
     </row>
     <row r="198" spans="1:20" ht="15" customHeight="1">
       <c r="A198" s="63" t="s">
-        <v>1001</v>
+        <v>997</v>
       </c>
       <c r="B198" s="63" t="s">
-        <v>1002</v>
+        <v>998</v>
       </c>
       <c r="C198" s="63" t="s">
         <v>95</v>
@@ -33420,17 +33539,17 @@
         <v>678</v>
       </c>
       <c r="P198" s="58" t="s">
-        <v>1003</v>
+        <v>999</v>
       </c>
       <c r="S198" s="58"/>
       <c r="T198" s="58"/>
     </row>
     <row r="199" spans="1:20" ht="15" customHeight="1">
       <c r="A199" s="66" t="s">
-        <v>1004</v>
+        <v>1000</v>
       </c>
       <c r="B199" s="63" t="s">
-        <v>1005</v>
+        <v>1001</v>
       </c>
       <c r="C199" s="63" t="s">
         <v>95</v>
@@ -33469,17 +33588,17 @@
         <v>678</v>
       </c>
       <c r="P199" s="58" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
       <c r="S199" s="58"/>
       <c r="T199" s="58"/>
     </row>
     <row r="200" spans="1:20" ht="30" customHeight="1">
       <c r="A200" s="63" t="s">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="B200" s="66" t="s">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="C200" s="66" t="s">
         <v>95</v>
@@ -33513,24 +33632,24 @@
         <v>2598</v>
       </c>
       <c r="L200" s="63" t="s">
-        <v>1103</v>
+        <v>1097</v>
       </c>
       <c r="M200" s="63"/>
       <c r="N200" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P200" s="58" t="s">
-        <v>1104</v>
+        <v>1098</v>
       </c>
       <c r="S200" s="58"/>
       <c r="T200" s="58"/>
     </row>
     <row r="201" spans="1:20" ht="15" customHeight="1">
       <c r="A201" s="66" t="s">
-        <v>1009</v>
+        <v>1005</v>
       </c>
       <c r="B201" s="63" t="s">
-        <v>1010</v>
+        <v>1006</v>
       </c>
       <c r="C201" s="63" t="s">
         <v>95</v>
@@ -33564,24 +33683,24 @@
         <v>724</v>
       </c>
       <c r="L201" s="66" t="s">
-        <v>1011</v>
+        <v>1007</v>
       </c>
       <c r="M201" s="66"/>
       <c r="N201" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P201" s="58" t="s">
-        <v>1012</v>
+        <v>1008</v>
       </c>
       <c r="S201" s="58"/>
       <c r="T201" s="58"/>
     </row>
     <row r="202" spans="1:20" ht="15" customHeight="1">
       <c r="A202" s="63" t="s">
-        <v>1013</v>
+        <v>1009</v>
       </c>
       <c r="B202" s="66" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
       <c r="C202" s="66" t="s">
         <v>95</v>
@@ -33615,24 +33734,24 @@
         <v>2820</v>
       </c>
       <c r="L202" s="63" t="s">
-        <v>1162</v>
+        <v>1153</v>
       </c>
       <c r="M202" s="63"/>
       <c r="N202" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="58" t="s">
-        <v>1163</v>
+        <v>1154</v>
       </c>
       <c r="S202" s="58"/>
       <c r="T202" s="58"/>
     </row>
     <row r="203" spans="1:20" ht="15" customHeight="1">
       <c r="A203" s="66" t="s">
-        <v>1015</v>
+        <v>1011</v>
       </c>
       <c r="B203" s="63" t="s">
-        <v>1016</v>
+        <v>1012</v>
       </c>
       <c r="C203" s="63" t="s">
         <v>95</v>
@@ -33666,24 +33785,24 @@
         <v>0</v>
       </c>
       <c r="L203" s="66" t="s">
-        <v>1017</v>
+        <v>1013</v>
       </c>
       <c r="M203" s="66"/>
       <c r="N203" s="58" t="s">
         <v>504</v>
       </c>
       <c r="P203" s="58" t="s">
-        <v>1018</v>
+        <v>1014</v>
       </c>
       <c r="S203" s="58"/>
       <c r="T203" s="58"/>
     </row>
     <row r="204" spans="1:20" ht="15" customHeight="1">
       <c r="A204" s="63" t="s">
-        <v>1019</v>
+        <v>1015</v>
       </c>
       <c r="B204" s="63" t="s">
-        <v>1020</v>
+        <v>1016</v>
       </c>
       <c r="C204" s="63" t="s">
         <v>95</v>
@@ -33717,24 +33836,24 @@
         <v>880</v>
       </c>
       <c r="L204" s="63" t="s">
-        <v>1135</v>
+        <v>1129</v>
       </c>
       <c r="M204" s="63"/>
       <c r="N204" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P204" s="58" t="s">
-        <v>1134</v>
+        <v>1128</v>
       </c>
       <c r="S204" s="58"/>
       <c r="T204" s="58"/>
     </row>
     <row r="205" spans="1:20" ht="15" customHeight="1">
       <c r="A205" s="66" t="s">
-        <v>1021</v>
+        <v>1017</v>
       </c>
       <c r="B205" s="66" t="s">
-        <v>1022</v>
+        <v>1018</v>
       </c>
       <c r="C205" s="66" t="s">
         <v>95</v>
@@ -33768,24 +33887,24 @@
         <v>1522</v>
       </c>
       <c r="L205" s="66" t="s">
-        <v>1023</v>
+        <v>1019</v>
       </c>
       <c r="M205" s="66"/>
       <c r="N205" s="58" t="s">
         <v>678</v>
       </c>
       <c r="P205" s="58" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="S205" s="58"/>
       <c r="T205" s="58"/>
     </row>
     <row r="206" spans="1:20" ht="15" customHeight="1">
       <c r="A206" s="63" t="s">
-        <v>1025</v>
+        <v>1021</v>
       </c>
       <c r="B206" s="63" t="s">
-        <v>1026</v>
+        <v>1022</v>
       </c>
       <c r="C206" s="63" t="s">
         <v>95</v>
@@ -33797,10 +33916,10 @@
         <v>1250</v>
       </c>
       <c r="F206" s="78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G206" s="78">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H206" s="77">
         <f t="shared" si="12"/>
@@ -33812,29 +33931,31 @@
       </c>
       <c r="J206" s="77">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="K206" s="77">
         <f t="shared" si="14"/>
-        <v>761</v>
-      </c>
-      <c r="L206" s="63"/>
+        <v>0</v>
+      </c>
+      <c r="L206" s="63" t="s">
+        <v>220</v>
+      </c>
       <c r="M206" s="63"/>
       <c r="N206" s="58" t="s">
-        <v>678</v>
+        <v>504</v>
       </c>
       <c r="P206" s="58" t="s">
-        <v>1027</v>
+        <v>1023</v>
       </c>
       <c r="S206" s="58"/>
       <c r="T206" s="58"/>
     </row>
     <row r="207" spans="1:20" ht="15" customHeight="1">
       <c r="A207" s="66" t="s">
-        <v>1028</v>
+        <v>1024</v>
       </c>
       <c r="B207" s="66" t="s">
-        <v>1029</v>
+        <v>1025</v>
       </c>
       <c r="C207" s="66" t="s">
         <v>95</v>
@@ -33868,24 +33989,24 @@
         <v>3312</v>
       </c>
       <c r="L207" s="66" t="s">
-        <v>1030</v>
+        <v>1026</v>
       </c>
       <c r="M207" s="66"/>
       <c r="N207" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P207" s="58" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="S207" s="58"/>
       <c r="T207" s="58"/>
     </row>
     <row r="208" spans="1:20" ht="30" customHeight="1">
       <c r="A208" s="63" t="s">
-        <v>1032</v>
+        <v>1028</v>
       </c>
       <c r="B208" s="63" t="s">
-        <v>1033</v>
+        <v>1029</v>
       </c>
       <c r="C208" s="63" t="s">
         <v>95</v>
@@ -33924,17 +34045,17 @@
         <v>678</v>
       </c>
       <c r="P208" s="58" t="s">
-        <v>1034</v>
+        <v>1030</v>
       </c>
       <c r="S208" s="58"/>
       <c r="T208" s="58"/>
     </row>
     <row r="209" spans="1:20" ht="15" customHeight="1">
       <c r="A209" s="66" t="s">
-        <v>1035</v>
+        <v>1031</v>
       </c>
       <c r="B209" s="63" t="s">
-        <v>1036</v>
+        <v>1032</v>
       </c>
       <c r="C209" s="63" t="s">
         <v>95</v>
@@ -33968,24 +34089,24 @@
         <v>982</v>
       </c>
       <c r="L209" s="66" t="s">
-        <v>1102</v>
+        <v>1096</v>
       </c>
       <c r="M209" s="66"/>
       <c r="N209" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P209" s="58" t="s">
-        <v>1101</v>
+        <v>1095</v>
       </c>
       <c r="S209" s="58"/>
       <c r="T209" s="58"/>
     </row>
     <row r="210" spans="1:20" ht="15" customHeight="1">
       <c r="A210" s="63" t="s">
-        <v>1037</v>
+        <v>1033</v>
       </c>
       <c r="B210" s="66" t="s">
-        <v>1038</v>
+        <v>1034</v>
       </c>
       <c r="C210" s="66" t="s">
         <v>95</v>
@@ -34024,17 +34145,17 @@
         <v>678</v>
       </c>
       <c r="P210" s="58" t="s">
-        <v>1039</v>
+        <v>1035</v>
       </c>
       <c r="S210" s="58"/>
       <c r="T210" s="58"/>
     </row>
     <row r="211" spans="1:20" ht="15" customHeight="1">
       <c r="A211" s="66" t="s">
-        <v>1040</v>
+        <v>1036</v>
       </c>
       <c r="B211" s="63" t="s">
-        <v>903</v>
+        <v>901</v>
       </c>
       <c r="C211" s="63" t="s">
         <v>95</v>
@@ -34073,17 +34194,17 @@
         <v>678</v>
       </c>
       <c r="P211" s="58" t="s">
-        <v>1041</v>
+        <v>1037</v>
       </c>
       <c r="S211" s="58"/>
       <c r="T211" s="58"/>
     </row>
     <row r="212" spans="1:20" ht="15" customHeight="1">
       <c r="A212" s="63" t="s">
-        <v>1042</v>
+        <v>1038</v>
       </c>
       <c r="B212" s="66" t="s">
-        <v>1121</v>
+        <v>1115</v>
       </c>
       <c r="C212" s="66" t="s">
         <v>95</v>
@@ -34126,42 +34247,58 @@
     </row>
     <row r="213" spans="1:20" ht="15" customHeight="1">
       <c r="A213" s="66" t="s">
-        <v>1043</v>
-      </c>
-      <c r="B213" s="63"/>
-      <c r="C213" s="63"/>
-      <c r="D213" s="64"/>
-      <c r="E213" s="64"/>
+        <v>1039</v>
+      </c>
+      <c r="B213" s="63" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C213" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="D213" s="64">
+        <v>555</v>
+      </c>
+      <c r="E213" s="64">
+        <v>850</v>
+      </c>
       <c r="F213" s="76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G213" s="76">
-        <v>-28</v>
+        <v>8</v>
       </c>
       <c r="H213" s="75">
         <f t="shared" si="12"/>
-        <v>-28</v>
+        <v>9</v>
       </c>
       <c r="I213" s="75">
         <f>IF(D213&lt;&gt;"",D213,IFERROR(E213/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>555</v>
       </c>
       <c r="J213" s="75">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>555</v>
       </c>
       <c r="K213" s="75">
         <f t="shared" si="14"/>
-        <v>0</v>
-      </c>
-      <c r="L213" s="66"/>
+        <v>4440</v>
+      </c>
+      <c r="L213" s="66" t="s">
+        <v>1167</v>
+      </c>
       <c r="M213" s="66"/>
+      <c r="N213" s="58" t="s">
+        <v>589</v>
+      </c>
+      <c r="P213" s="58" t="s">
+        <v>1168</v>
+      </c>
       <c r="S213" s="58"/>
       <c r="T213" s="58"/>
     </row>
     <row r="214" spans="1:20" ht="15" customHeight="1">
       <c r="A214" s="63" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="B214" s="63"/>
       <c r="C214" s="63"/>
@@ -34196,7 +34333,7 @@
     </row>
     <row r="215" spans="1:20" ht="15" customHeight="1">
       <c r="A215" s="66" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="B215" s="66"/>
       <c r="C215" s="66"/>
@@ -34231,7 +34368,7 @@
     </row>
     <row r="216" spans="1:20" ht="15" customHeight="1">
       <c r="A216" s="63" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
       <c r="B216" s="63"/>
       <c r="C216" s="63"/>
@@ -34266,7 +34403,7 @@
     </row>
     <row r="217" spans="1:20" ht="15" customHeight="1">
       <c r="A217" s="66" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="B217" s="66"/>
       <c r="C217" s="66"/>
@@ -34301,7 +34438,7 @@
     </row>
     <row r="218" spans="1:20" ht="15" customHeight="1">
       <c r="A218" s="63" t="s">
-        <v>1048</v>
+        <v>1044</v>
       </c>
       <c r="B218" s="63"/>
       <c r="C218" s="63"/>
@@ -34336,7 +34473,7 @@
     </row>
     <row r="219" spans="1:20" ht="15" customHeight="1">
       <c r="A219" s="66" t="s">
-        <v>1049</v>
+        <v>1045</v>
       </c>
       <c r="B219" s="63"/>
       <c r="C219" s="63"/>
@@ -34371,7 +34508,7 @@
     </row>
     <row r="220" spans="1:20" ht="15" customHeight="1">
       <c r="A220" s="63" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="B220" s="66"/>
       <c r="C220" s="66"/>
@@ -34406,7 +34543,7 @@
     </row>
     <row r="221" spans="1:20" ht="15" customHeight="1">
       <c r="A221" s="66" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="B221" s="63"/>
       <c r="C221" s="63"/>
@@ -34441,7 +34578,7 @@
     </row>
     <row r="222" spans="1:20" ht="15" customHeight="1">
       <c r="A222" s="63" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
       <c r="B222" s="66"/>
       <c r="C222" s="66"/>
@@ -34476,7 +34613,7 @@
     </row>
     <row r="223" spans="1:20" ht="15" customHeight="1">
       <c r="A223" s="66" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="B223" s="63"/>
       <c r="C223" s="63"/>
@@ -34511,7 +34648,7 @@
     </row>
     <row r="224" spans="1:20" ht="15" customHeight="1">
       <c r="A224" s="63" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
       <c r="B224" s="63"/>
       <c r="C224" s="63"/>
@@ -34546,7 +34683,7 @@
     </row>
     <row r="225" spans="1:20" ht="15" customHeight="1">
       <c r="A225" s="66" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="B225" s="66"/>
       <c r="C225" s="66"/>
@@ -34581,7 +34718,7 @@
     </row>
     <row r="226" spans="1:20" ht="15" customHeight="1">
       <c r="A226" s="63" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="B226" s="63"/>
       <c r="C226" s="63"/>
@@ -38496,7 +38633,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="92" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
       <c r="B1" s="92"/>
     </row>
@@ -38505,7 +38642,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -38537,25 +38674,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="83" t="s">
+        <v>1055</v>
+      </c>
+      <c r="C7" s="83" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D7" s="83" t="s">
+        <v>1057</v>
+      </c>
+      <c r="E7" s="83" t="s">
+        <v>1058</v>
+      </c>
+      <c r="F7" s="83" t="s">
         <v>1059</v>
       </c>
-      <c r="C7" s="83" t="s">
+      <c r="G7" s="83" t="s">
         <v>1060</v>
       </c>
-      <c r="D7" s="83" t="s">
+      <c r="H7" s="83" t="s">
         <v>1061</v>
-      </c>
-      <c r="E7" s="83" t="s">
-        <v>1062</v>
-      </c>
-      <c r="F7" s="83" t="s">
-        <v>1063</v>
-      </c>
-      <c r="G7" s="83" t="s">
-        <v>1064</v>
-      </c>
-      <c r="H7" s="83" t="s">
-        <v>1065</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -38564,15 +38701,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>248108</v>
+        <v>249742</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>172391.66666666666</v>
+        <v>172936.33333333334</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>75716.333333333343</v>
+        <v>76805.666666666657</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38580,7 +38717,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>75716.333333333343</v>
+        <v>76805.666666666657</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -38588,7 +38725,7 @@
       </c>
       <c r="H8" s="85">
         <f>F8-G8</f>
-        <v>57412.993333333347</v>
+        <v>58502.32666666666</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -38601,11 +38738,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>172391.66666666666</v>
+        <v>172936.33333333334</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>64075.333333333343</v>
+        <v>63530.666666666657</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38613,7 +38750,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>64075.333333333343</v>
+        <v>63530.666666666657</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -38621,7 +38758,7 @@
       </c>
       <c r="H9" s="86">
         <f>F9-G9</f>
-        <v>22436.003333333341</v>
+        <v>21891.336666666655</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -38634,11 +38771,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>172391.66666666666</v>
+        <v>172936.33333333334</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-139791.66666666666</v>
+        <v>-140336.33333333334</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38646,7 +38783,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-139791.66666666666</v>
+        <v>-140336.33333333334</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -38654,12 +38791,12 @@
       </c>
       <c r="H10" s="85">
         <f>F10-G10</f>
-        <v>-79848.996666666659</v>
+        <v>-80393.663333333345</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="93" t="s">
-        <v>1066</v>
+        <v>1062</v>
       </c>
       <c r="B12" s="93"/>
       <c r="C12" s="93"/>
@@ -38672,13 +38809,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="83" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="C13" s="83" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
       <c r="D13" s="83" t="s">
-        <v>1069</v>
+        <v>1065</v>
       </c>
       <c r="E13" s="83" t="s">
         <v>99</v>
@@ -38692,7 +38829,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -38710,7 +38847,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -38764,7 +38901,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -38782,7 +38919,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -38800,7 +38937,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -38818,7 +38955,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -38836,7 +38973,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -38872,7 +39009,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -38908,7 +39045,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -38926,7 +39063,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -39009,7 +39146,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>1071</v>
+        <v>1067</v>
       </c>
     </row>
   </sheetData>
@@ -39039,7 +39176,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="90" t="s">
-        <v>1072</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="84" customFormat="1" ht="13.5" customHeight="1">
@@ -39047,22 +39184,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="83" t="s">
+        <v>1069</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D3" s="83" t="s">
+        <v>1070</v>
+      </c>
+      <c r="E3" s="83" t="s">
+        <v>1071</v>
+      </c>
+      <c r="F3" s="83" t="s">
+        <v>1072</v>
+      </c>
+      <c r="G3" s="83" t="s">
         <v>1073</v>
-      </c>
-      <c r="C3" s="83" t="s">
-        <v>1058</v>
-      </c>
-      <c r="D3" s="83" t="s">
-        <v>1074</v>
-      </c>
-      <c r="E3" s="83" t="s">
-        <v>1075</v>
-      </c>
-      <c r="F3" s="83" t="s">
-        <v>1076</v>
-      </c>
-      <c r="G3" s="83" t="s">
-        <v>1077</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -39071,7 +39208,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>382561</v>
+        <v>392221</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -39079,11 +39216,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>149934.981</v>
+        <v>153155.625</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>232626.019</v>
+        <v>239065.375</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39091,7 +39228,7 @@
       </c>
       <c r="G4" s="85">
         <f>E4+F4</f>
-        <v>95315.992999999988</v>
+        <v>101755.34899999999</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -39108,11 +39245,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>149845.038</v>
+        <v>153063.75</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-95221.038</v>
+        <v>-98439.75</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39120,7 +39257,7 @@
       </c>
       <c r="G5" s="86">
         <f>E5+F5</f>
-        <v>-23633.995999999999</v>
+        <v>-26852.707999999999</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -39137,11 +39274,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>149934.981</v>
+        <v>153155.625</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-137404.981</v>
+        <v>-140625.625</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39149,7 +39286,7 @@
       </c>
       <c r="G6" s="85">
         <f>E6+F6</f>
-        <v>-71681.996999999988</v>
+        <v>-74902.640999999989</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -39159,27 +39296,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>1079</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>1080</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>1081</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
7/18 & 7/19 Sales and purchases
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9050C1C-FF82-F645-B893-7A21E3C455B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F19A9105-1663-6341-B149-82AFBEC83C9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3006" uniqueCount="1186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3038" uniqueCount="1196">
   <si>
     <t>Notes:</t>
   </si>
@@ -3067,9 +3067,6 @@
     <t>Semi Silk Saree Collections</t>
   </si>
   <si>
-    <t>Peach, light blue, pink, light green</t>
-  </si>
-  <si>
     <t>CHR-199</t>
   </si>
   <si>
@@ -3298,13 +3295,6 @@
     <t>5. Cash Position After Settlements = Over/(Under) + Net Cash Settlements.</t>
   </si>
   <si>
-    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200, Black/Golden yellow - Kavya(Kasargod) - 1200, Back/Yellow - Subha - 1200, Navy Blue/Bottle Green - Latha</t>
-  </si>
-  <si>
-    <t>Bottle Green/Golden Yellow - 1
-Navy Blue/Bottle Green - 1</t>
-  </si>
-  <si>
     <t>Matka old design - Navy Blue/Bottle Green</t>
   </si>
   <si>
@@ -3330,14 +3320,6 @@
   </si>
   <si>
     <t>CHR-119 Maroon</t>
-  </si>
-  <si>
-    <t>First Set: Aruna - violet, Resmi - navy blue, Malini - Rani Pink
-Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Shaino Benny - Navy blue, Simi Sudhir - Navy Blue, Supriya - Green, Mercy - Black, Kalisari - Green, Latha Suresh - Black, Shinoob cousin - mustard yellow, off white returned, Sumi Boben (Jet black), Jinu (Blue), Raji VT(Black), Nishitha friend (Orange), Karthika (Blue), SIndhu (White), Linu George (Black), Sheeja S(White), Sarnya (Maroon)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-White(3)</t>
   </si>
   <si>
     <t>CHR-191 (Floral Green) &amp; CHR-208 (Kathakali)</t>
@@ -3526,12 +3508,6 @@
     <t>Anjumol Canada</t>
   </si>
   <si>
-    <t>Komalavalli - Blue, Anjumol canada - Blue &amp; Red</t>
-  </si>
-  <si>
-    <t>Green, Pink, Yellow</t>
-  </si>
-  <si>
     <t>Gincy Jibi</t>
   </si>
   <si>
@@ -3623,6 +3599,59 @@
   </si>
   <si>
     <t>Rose pink, dusty lavender, brick red, champagne, chocolate brown, magenta</t>
+  </si>
+  <si>
+    <t>Lekha</t>
+  </si>
+  <si>
+    <t>CHR-201 Yellow</t>
+  </si>
+  <si>
+    <t>Komalavalli - Blue, Anjumol canada - Blue &amp; Red, Lekha - Yellow</t>
+  </si>
+  <si>
+    <t>Green, Pink</t>
+  </si>
+  <si>
+    <t>Suma Soman</t>
+  </si>
+  <si>
+    <t>CHR-146 - Green/Yellow</t>
+  </si>
+  <si>
+    <t>Teena Mathew</t>
+  </si>
+  <si>
+    <t>CHR-198 Semi Silk Peach</t>
+  </si>
+  <si>
+    <t>Teena mathew - Paeach</t>
+  </si>
+  <si>
+    <t>light blue, pink, light green</t>
+  </si>
+  <si>
+    <t>Ancy Philip</t>
+  </si>
+  <si>
+    <t>CHR-146 - Navy Blue/Bottle Green</t>
+  </si>
+  <si>
+    <t>Blue/bottle green - Saranya Hyd, Blue/red - Jothika, Mustard - Vineetha, Bottle Green/Golden Yellow - Swapna (Thrissur)-1200, Black/Golden yellow - Kavya(Kasargod) - 1200, Back/Yellow - Subha - 1200, Navy Blue/Bottle Green - Latha, Suma Soman - Green/Yellow(1100), Ancy Philip - Navy Blue/Bottle Green(1250)</t>
+  </si>
+  <si>
+    <t>Saneesh Devasia</t>
+  </si>
+  <si>
+    <t>Sabida</t>
+  </si>
+  <si>
+    <t>First Set: Aruna - violet, Resmi - navy blue, Malini - Rani Pink
+Second Set: Sreelekha - Black, Dona - navy Blue, Jayalakshmi - Pink, Jyothimol - Navy Blue, Amrutha - Maroon, Athira - Black, Jini - Maroon, Gopika - Black, Aji Roy - Black, Aji Roy - Mustard, Lili Kutty - Maroon, Sindhu - Black, Asha - Green, Soorya - Rani Pink, Asha Latha - Offwhite, Susmi - Off white, Revathi - Maroon &amp; Orange, Saritha - Rani Pink, Rose - Black, Bindu Krisharaj - Black, Kavitha - off white, Jisha Suresh - Rani Pink(2), Sudharma - Navy Blue, SIndrella - Maroon, Shaino Benny - Navy blue, Simi Sudhir - Navy Blue, Supriya - Green, Mercy - Black, Kalisari - Green, Latha Suresh - Black, Shinoob cousin - mustard yellow, off white returned, Sumi Boben (Jet black), Jinu (Blue), Raji VT(Black), Nishitha friend (Orange), Karthika (Blue), SIndhu (White), Linu George (Black), Sheeja S(White), Sarnya (Maroon), Saneesh (Maroon), Sabida(Maroon)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+White(3), maroon(3)</t>
   </si>
 </sst>
 </file>
@@ -4502,7 +4531,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>281</c:v>
+                  <c:v>286</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>95</c:v>
@@ -4938,7 +4967,7 @@
                   <c:v>56434</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>140954.43</c:v>
+                  <c:v>139264.19666666666</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>590</c:v>
@@ -5271,7 +5300,7 @@
                   <c:v>99043</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>64662</c:v>
+                  <c:v>64848</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5431,7 +5460,7 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>40807</c:v>
+                  <c:v>46906</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5871,7 +5900,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-23855</c:v>
+                  <c:v>-17942</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6335,7 +6364,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>381</c:v>
+                  <c:v>386</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>8</c:v>
@@ -7510,7 +7539,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>518809</v>
+        <v>518995</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7525,7 +7554,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>459375</v>
+        <v>465474</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7542,7 +7571,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>469305</v>
+        <v>475404</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7559,7 +7588,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-59434</v>
+        <v>-53521</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7594,7 +7623,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>58502.32666666666</v>
+        <v>58626.32666666666</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7604,7 +7633,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>21891.336666666655</v>
+        <v>21829.336666666655</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7614,7 +7643,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-80393.663333333345</v>
+        <v>-80455.663333333345</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7653,15 +7682,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>249742</v>
+        <v>249928</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>172936.33333333334</v>
+        <v>172998.33333333334</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>76805.666666666657</v>
+        <v>76929.666666666657</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7669,11 +7698,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>58502.32666666666</v>
+        <v>58626.32666666666</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹58,502</v>
+        <v>Receive ₹58,626</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7687,11 +7716,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>172936.33333333334</v>
+        <v>172998.33333333334</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>63530.666666666657</v>
+        <v>63468.666666666657</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7699,11 +7728,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>21891.336666666655</v>
+        <v>21829.336666666655</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹21,891</v>
+        <v>Receive ₹21,829</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7717,11 +7746,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>172936.33333333334</v>
+        <v>172998.33333333334</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-140336.33333333334</v>
+        <v>-140398.33333333334</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7729,11 +7758,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-80393.663333333345</v>
+        <v>-80455.663333333345</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹80,394</v>
+        <v>Pay ₹80,456</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7771,15 +7800,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>392221</v>
+        <v>398320</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>153155.625</v>
+        <v>155189.03159999999</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>239065.375</v>
+        <v>243130.96840000001</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7787,11 +7816,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>101755.34899999999</v>
+        <v>105820.9424</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹101,755</v>
+        <v>Pay ₹105,821</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7805,11 +7834,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>153063.75</v>
+        <v>155095.9368</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-98439.75</v>
+        <v>-100471.9368</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7817,11 +7846,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-26852.707999999999</v>
+        <v>-28884.894799999995</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹26,853</v>
+        <v>Receive ₹28,885</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7835,11 +7864,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>153155.625</v>
+        <v>155189.03159999999</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-140625.625</v>
+        <v>-142659.03159999999</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7847,11 +7876,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-74902.640999999989</v>
+        <v>-76936.047599999976</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹74,903</v>
+        <v>Receive ₹76,936</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -7963,7 +7992,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46219</v>
+        <v>46222</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -7972,14 +8001,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>518809</v>
+        <v>518995</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>459375</v>
+        <v>465474</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -7988,14 +8017,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-59434</v>
+        <v>-53521</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>188357.63</v>
+        <v>186667.39666666667</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8047,7 +8076,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>381</v>
+        <v>386</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8148,15 +8177,15 @@
       </c>
       <c r="B16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A16)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>64662</v>
+        <v>64848</v>
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$995,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$995)=$B$7)*Sales!$C$2:$C$995),0)</f>
-        <v>40807</v>
+        <v>46906</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-23855</v>
+        <v>-17942</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8267,7 +8296,7 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
@@ -8298,7 +8327,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>140954.43</v>
+        <v>139264.19666666666</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9671,7 +9700,7 @@
         <v>28526</v>
       </c>
       <c r="D91" s="39" t="s">
-        <v>1114</v>
+        <v>1109</v>
       </c>
     </row>
     <row r="92" spans="1:4" ht="15" customHeight="1">
@@ -9741,7 +9770,7 @@
         <v>70</v>
       </c>
       <c r="D96" s="36" t="s">
-        <v>1160</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15" customHeight="1">
@@ -9755,7 +9784,7 @@
         <v>1375</v>
       </c>
       <c r="D97" s="39" t="s">
-        <v>1161</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="98" spans="1:4" ht="15" customHeight="1">
@@ -9769,14 +9798,22 @@
         <v>189</v>
       </c>
       <c r="D98" s="36" t="s">
-        <v>1162</v>
+        <v>1155</v>
       </c>
     </row>
     <row r="99" spans="1:4" ht="15" customHeight="1">
-      <c r="A99" s="38"/>
-      <c r="B99" s="39"/>
-      <c r="C99" s="40"/>
-      <c r="D99" s="39"/>
+      <c r="A99" s="38">
+        <v>46220</v>
+      </c>
+      <c r="B99" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C99" s="40">
+        <v>186</v>
+      </c>
+      <c r="D99" s="39" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="100" spans="1:4" ht="15" customHeight="1">
       <c r="A100" s="35"/>
@@ -17208,7 +17245,7 @@
       <c r="F216" s="56"/>
       <c r="G216" s="56"/>
       <c r="H216" s="57" t="s">
-        <v>1099</v>
+        <v>1094</v>
       </c>
       <c r="I216" s="53" t="s">
         <v>148</v>
@@ -18033,7 +18070,7 @@
       <c r="F249" s="56"/>
       <c r="G249" s="56"/>
       <c r="H249" s="57" t="s">
-        <v>1081</v>
+        <v>1078</v>
       </c>
       <c r="I249" s="53" t="s">
         <v>148</v>
@@ -18054,7 +18091,7 @@
       <c r="F250" s="49"/>
       <c r="G250" s="49"/>
       <c r="H250" s="51" t="s">
-        <v>1083</v>
+        <v>1080</v>
       </c>
       <c r="I250" s="49" t="s">
         <v>356</v>
@@ -18065,7 +18102,7 @@
         <v>46201</v>
       </c>
       <c r="B251" s="53" t="s">
-        <v>1100</v>
+        <v>1095</v>
       </c>
       <c r="C251" s="54">
         <v>1380</v>
@@ -18090,7 +18127,7 @@
         <v>46201</v>
       </c>
       <c r="B252" s="49" t="s">
-        <v>1084</v>
+        <v>1081</v>
       </c>
       <c r="C252" s="50">
         <v>699</v>
@@ -18104,7 +18141,7 @@
       <c r="F252" s="49"/>
       <c r="G252" s="49"/>
       <c r="H252" s="51" t="s">
-        <v>1085</v>
+        <v>1082</v>
       </c>
       <c r="I252" s="49" t="s">
         <v>148</v>
@@ -18115,7 +18152,7 @@
         <v>46201</v>
       </c>
       <c r="B253" s="53" t="s">
-        <v>1086</v>
+        <v>1083</v>
       </c>
       <c r="C253" s="54">
         <v>699</v>
@@ -18129,7 +18166,7 @@
       <c r="F253" s="56"/>
       <c r="G253" s="56"/>
       <c r="H253" s="57" t="s">
-        <v>1087</v>
+        <v>1084</v>
       </c>
       <c r="I253" s="53" t="s">
         <v>148</v>
@@ -18140,7 +18177,7 @@
         <v>46201</v>
       </c>
       <c r="B254" s="49" t="s">
-        <v>1088</v>
+        <v>1085</v>
       </c>
       <c r="C254" s="50">
         <v>699</v>
@@ -18154,7 +18191,7 @@
       <c r="F254" s="49"/>
       <c r="G254" s="49"/>
       <c r="H254" s="51" t="s">
-        <v>1089</v>
+        <v>1086</v>
       </c>
       <c r="I254" s="49" t="s">
         <v>148</v>
@@ -18179,7 +18216,7 @@
       <c r="F255" s="56"/>
       <c r="G255" s="56"/>
       <c r="H255" s="57" t="s">
-        <v>1092</v>
+        <v>1087</v>
       </c>
       <c r="I255" s="53" t="s">
         <v>148</v>
@@ -18190,7 +18227,7 @@
         <v>46203</v>
       </c>
       <c r="B256" s="49" t="s">
-        <v>1101</v>
+        <v>1096</v>
       </c>
       <c r="C256" s="50">
         <v>950</v>
@@ -18204,7 +18241,7 @@
       <c r="F256" s="49"/>
       <c r="G256" s="49"/>
       <c r="H256" s="51" t="s">
-        <v>1102</v>
+        <v>1097</v>
       </c>
       <c r="I256" s="49" t="s">
         <v>148</v>
@@ -18215,7 +18252,7 @@
         <v>46204</v>
       </c>
       <c r="B257" s="53" t="s">
-        <v>1105</v>
+        <v>1100</v>
       </c>
       <c r="C257" s="54">
         <v>699</v>
@@ -18229,7 +18266,7 @@
       <c r="F257" s="56"/>
       <c r="G257" s="56"/>
       <c r="H257" s="57" t="s">
-        <v>1106</v>
+        <v>1101</v>
       </c>
       <c r="I257" s="53" t="s">
         <v>148</v>
@@ -18240,7 +18277,7 @@
         <v>46205</v>
       </c>
       <c r="B258" s="49" t="s">
-        <v>1107</v>
+        <v>1102</v>
       </c>
       <c r="C258" s="50">
         <v>1500</v>
@@ -18254,7 +18291,7 @@
       <c r="F258" s="49"/>
       <c r="G258" s="49"/>
       <c r="H258" s="51" t="s">
-        <v>1108</v>
+        <v>1103</v>
       </c>
       <c r="I258" s="49" t="s">
         <v>148</v>
@@ -18265,7 +18302,7 @@
         <v>46205</v>
       </c>
       <c r="B259" s="53" t="s">
-        <v>1107</v>
+        <v>1102</v>
       </c>
       <c r="C259" s="54">
         <v>1200</v>
@@ -18279,7 +18316,7 @@
       <c r="F259" s="56"/>
       <c r="G259" s="56"/>
       <c r="H259" s="57" t="s">
-        <v>1111</v>
+        <v>1106</v>
       </c>
       <c r="I259" s="53" t="s">
         <v>148</v>
@@ -18290,7 +18327,7 @@
         <v>46205</v>
       </c>
       <c r="B260" s="49" t="s">
-        <v>1113</v>
+        <v>1108</v>
       </c>
       <c r="C260" s="50">
         <v>1500</v>
@@ -18304,7 +18341,7 @@
       <c r="F260" s="49"/>
       <c r="G260" s="49"/>
       <c r="H260" s="51" t="s">
-        <v>1112</v>
+        <v>1107</v>
       </c>
       <c r="I260" s="49" t="s">
         <v>148</v>
@@ -18315,7 +18352,7 @@
         <v>46205</v>
       </c>
       <c r="B261" s="53" t="s">
-        <v>1116</v>
+        <v>1111</v>
       </c>
       <c r="C261" s="54">
         <v>1900</v>
@@ -18325,7 +18362,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1143</v>
+        <v>1138</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>356</v>
@@ -18336,7 +18373,7 @@
         <v>46206</v>
       </c>
       <c r="B262" s="49" t="s">
-        <v>1121</v>
+        <v>1116</v>
       </c>
       <c r="C262" s="50">
         <v>1380</v>
@@ -18361,7 +18398,7 @@
         <v>46206</v>
       </c>
       <c r="B263" s="53" t="s">
-        <v>1122</v>
+        <v>1117</v>
       </c>
       <c r="C263" s="54">
         <v>1380</v>
@@ -18386,7 +18423,7 @@
         <v>46206</v>
       </c>
       <c r="B264" s="49" t="s">
-        <v>1133</v>
+        <v>1128</v>
       </c>
       <c r="C264" s="50">
         <v>2500</v>
@@ -18400,7 +18437,7 @@
       <c r="F264" s="49"/>
       <c r="G264" s="49"/>
       <c r="H264" s="51" t="s">
-        <v>1134</v>
+        <v>1129</v>
       </c>
       <c r="I264" s="49" t="s">
         <v>356</v>
@@ -18411,7 +18448,7 @@
         <v>46206</v>
       </c>
       <c r="B265" s="53" t="s">
-        <v>1125</v>
+        <v>1120</v>
       </c>
       <c r="C265" s="54">
         <v>1300</v>
@@ -18425,7 +18462,7 @@
       <c r="F265" s="56"/>
       <c r="G265" s="56"/>
       <c r="H265" s="57" t="s">
-        <v>1141</v>
+        <v>1136</v>
       </c>
       <c r="I265" s="53" t="s">
         <v>356</v>
@@ -18436,7 +18473,7 @@
         <v>46206</v>
       </c>
       <c r="B266" s="49" t="s">
-        <v>1113</v>
+        <v>1108</v>
       </c>
       <c r="C266" s="50">
         <v>1380</v>
@@ -18450,7 +18487,7 @@
       <c r="F266" s="49"/>
       <c r="G266" s="49"/>
       <c r="H266" s="51" t="s">
-        <v>1126</v>
+        <v>1121</v>
       </c>
       <c r="I266" s="49" t="s">
         <v>148</v>
@@ -18475,7 +18512,7 @@
       <c r="F267" s="56"/>
       <c r="G267" s="56"/>
       <c r="H267" s="57" t="s">
-        <v>1127</v>
+        <v>1122</v>
       </c>
       <c r="I267" s="53" t="s">
         <v>148</v>
@@ -18486,7 +18523,7 @@
         <v>46208</v>
       </c>
       <c r="B268" s="49" t="s">
-        <v>1132</v>
+        <v>1127</v>
       </c>
       <c r="C268" s="50">
         <v>2350</v>
@@ -18496,7 +18533,7 @@
       <c r="F268" s="49"/>
       <c r="G268" s="49"/>
       <c r="H268" s="51" t="s">
-        <v>1142</v>
+        <v>1137</v>
       </c>
       <c r="I268" s="49" t="s">
         <v>356</v>
@@ -18507,7 +18544,7 @@
         <v>46209</v>
       </c>
       <c r="B269" s="53" t="s">
-        <v>1130</v>
+        <v>1125</v>
       </c>
       <c r="C269" s="54">
         <v>1100</v>
@@ -18521,7 +18558,7 @@
       <c r="F269" s="56"/>
       <c r="G269" s="56"/>
       <c r="H269" s="57" t="s">
-        <v>1131</v>
+        <v>1126</v>
       </c>
       <c r="I269" s="53" t="s">
         <v>148</v>
@@ -18532,7 +18569,7 @@
         <v>46210</v>
       </c>
       <c r="B270" s="49" t="s">
-        <v>1137</v>
+        <v>1132</v>
       </c>
       <c r="C270" s="50">
         <v>3200</v>
@@ -18546,7 +18583,7 @@
       <c r="F270" s="49"/>
       <c r="G270" s="49"/>
       <c r="H270" s="51" t="s">
-        <v>1138</v>
+        <v>1133</v>
       </c>
       <c r="I270" s="49" t="s">
         <v>148</v>
@@ -18557,7 +18594,7 @@
         <v>46211</v>
       </c>
       <c r="B271" s="53" t="s">
-        <v>1139</v>
+        <v>1134</v>
       </c>
       <c r="C271" s="54">
         <v>1380</v>
@@ -18571,7 +18608,7 @@
       <c r="F271" s="56"/>
       <c r="G271" s="56"/>
       <c r="H271" s="57" t="s">
-        <v>1140</v>
+        <v>1135</v>
       </c>
       <c r="I271" s="53" t="s">
         <v>148</v>
@@ -18582,7 +18619,7 @@
         <v>46215</v>
       </c>
       <c r="B272" s="49" t="s">
-        <v>1145</v>
+        <v>1140</v>
       </c>
       <c r="C272" s="50">
         <v>1380</v>
@@ -18607,7 +18644,7 @@
         <v>46215</v>
       </c>
       <c r="B273" s="53" t="s">
-        <v>1146</v>
+        <v>1141</v>
       </c>
       <c r="C273" s="54">
         <v>699</v>
@@ -18621,7 +18658,7 @@
       <c r="F273" s="56"/>
       <c r="G273" s="56"/>
       <c r="H273" s="57" t="s">
-        <v>1106</v>
+        <v>1101</v>
       </c>
       <c r="I273" s="53" t="s">
         <v>148</v>
@@ -18646,7 +18683,7 @@
       <c r="F274" s="49"/>
       <c r="G274" s="49"/>
       <c r="H274" s="51" t="s">
-        <v>1148</v>
+        <v>1143</v>
       </c>
       <c r="I274" s="49" t="s">
         <v>148</v>
@@ -18657,7 +18694,7 @@
         <v>46216</v>
       </c>
       <c r="B275" s="53" t="s">
-        <v>1149</v>
+        <v>1144</v>
       </c>
       <c r="C275" s="54">
         <v>699</v>
@@ -18671,7 +18708,7 @@
       <c r="F275" s="56"/>
       <c r="G275" s="56"/>
       <c r="H275" s="57" t="s">
-        <v>1106</v>
+        <v>1101</v>
       </c>
       <c r="I275" s="53" t="s">
         <v>148</v>
@@ -18682,7 +18719,7 @@
         <v>46216</v>
       </c>
       <c r="B276" s="49" t="s">
-        <v>1152</v>
+        <v>1147</v>
       </c>
       <c r="C276" s="50">
         <v>3000</v>
@@ -18696,7 +18733,7 @@
       <c r="F276" s="49"/>
       <c r="G276" s="49"/>
       <c r="H276" s="51" t="s">
-        <v>1151</v>
+        <v>1146</v>
       </c>
       <c r="I276" s="49" t="s">
         <v>148</v>
@@ -18707,7 +18744,7 @@
         <v>46219</v>
       </c>
       <c r="B277" s="53" t="s">
-        <v>1155</v>
+        <v>1148</v>
       </c>
       <c r="C277" s="54">
         <v>1380</v>
@@ -18771,7 +18808,7 @@
       <c r="F279" s="56"/>
       <c r="G279" s="56"/>
       <c r="H279" s="57" t="s">
-        <v>1159</v>
+        <v>1152</v>
       </c>
       <c r="I279" s="53" t="s">
         <v>148</v>
@@ -18796,7 +18833,7 @@
       <c r="F280" s="49"/>
       <c r="G280" s="49"/>
       <c r="H280" s="51" t="s">
-        <v>1165</v>
+        <v>1158</v>
       </c>
       <c r="I280" s="49" t="s">
         <v>148</v>
@@ -18821,77 +18858,161 @@
       <c r="F281" s="56"/>
       <c r="G281" s="56"/>
       <c r="H281" s="57" t="s">
-        <v>1171</v>
+        <v>1164</v>
       </c>
       <c r="I281" s="53" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="282" spans="1:9">
-      <c r="A282" s="48"/>
-      <c r="B282" s="49"/>
-      <c r="C282" s="50"/>
-      <c r="D282" s="49"/>
-      <c r="E282" s="49"/>
+    <row r="282" spans="1:9" ht="14">
+      <c r="A282" s="48">
+        <v>46220</v>
+      </c>
+      <c r="B282" s="49" t="s">
+        <v>1179</v>
+      </c>
+      <c r="C282" s="50">
+        <v>1500</v>
+      </c>
+      <c r="D282" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E282" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F282" s="49"/>
       <c r="G282" s="49"/>
-      <c r="H282" s="51"/>
-      <c r="I282" s="49"/>
-    </row>
-    <row r="283" spans="1:9">
-      <c r="A283" s="52"/>
-      <c r="B283" s="53"/>
-      <c r="C283" s="54"/>
-      <c r="D283" s="53"/>
-      <c r="E283" s="53"/>
+      <c r="H282" s="51" t="s">
+        <v>1180</v>
+      </c>
+      <c r="I282" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="283" spans="1:9" ht="14">
+      <c r="A283" s="52">
+        <v>46221</v>
+      </c>
+      <c r="B283" s="53" t="s">
+        <v>1183</v>
+      </c>
+      <c r="C283" s="54">
+        <v>1100</v>
+      </c>
+      <c r="D283" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E283" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F283" s="56"/>
       <c r="G283" s="56"/>
-      <c r="H283" s="57"/>
-      <c r="I283" s="53"/>
-    </row>
-    <row r="284" spans="1:9">
-      <c r="A284" s="48"/>
-      <c r="B284" s="49"/>
-      <c r="C284" s="50"/>
-      <c r="D284" s="49"/>
-      <c r="E284" s="49"/>
+      <c r="H283" s="57" t="s">
+        <v>1184</v>
+      </c>
+      <c r="I283" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="284" spans="1:9" ht="14">
+      <c r="A284" s="48">
+        <v>46222</v>
+      </c>
+      <c r="B284" s="49" t="s">
+        <v>1185</v>
+      </c>
+      <c r="C284" s="50">
+        <v>850</v>
+      </c>
+      <c r="D284" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E284" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F284" s="49"/>
       <c r="G284" s="49"/>
-      <c r="H284" s="51"/>
-      <c r="I284" s="49"/>
-    </row>
-    <row r="285" spans="1:9">
-      <c r="A285" s="52"/>
-      <c r="B285" s="53"/>
-      <c r="C285" s="54"/>
-      <c r="D285" s="53"/>
-      <c r="E285" s="53"/>
+      <c r="H284" s="51" t="s">
+        <v>1186</v>
+      </c>
+      <c r="I284" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="285" spans="1:9" ht="14">
+      <c r="A285" s="52">
+        <v>46222</v>
+      </c>
+      <c r="B285" s="53" t="s">
+        <v>1189</v>
+      </c>
+      <c r="C285" s="54">
+        <v>1250</v>
+      </c>
+      <c r="D285" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E285" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F285" s="56"/>
       <c r="G285" s="56"/>
-      <c r="H285" s="57"/>
-      <c r="I285" s="53"/>
-    </row>
-    <row r="286" spans="1:9">
-      <c r="A286" s="48"/>
-      <c r="B286" s="49"/>
-      <c r="C286" s="50"/>
-      <c r="D286" s="49"/>
-      <c r="E286" s="49"/>
+      <c r="H285" s="57" t="s">
+        <v>1190</v>
+      </c>
+      <c r="I285" s="53" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="286" spans="1:9" ht="14">
+      <c r="A286" s="48">
+        <v>46222</v>
+      </c>
+      <c r="B286" s="49" t="s">
+        <v>1192</v>
+      </c>
+      <c r="C286" s="50">
+        <v>700</v>
+      </c>
+      <c r="D286" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E286" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F286" s="49"/>
       <c r="G286" s="49"/>
-      <c r="H286" s="51"/>
-      <c r="I286" s="49"/>
-    </row>
-    <row r="287" spans="1:9">
-      <c r="A287" s="52"/>
-      <c r="B287" s="53"/>
-      <c r="C287" s="54"/>
-      <c r="D287" s="53"/>
-      <c r="E287" s="53"/>
+      <c r="H286" s="51" t="s">
+        <v>395</v>
+      </c>
+      <c r="I286" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="287" spans="1:9" ht="14">
+      <c r="A287" s="52">
+        <v>46222</v>
+      </c>
+      <c r="B287" s="53" t="s">
+        <v>1193</v>
+      </c>
+      <c r="C287" s="54">
+        <v>699</v>
+      </c>
+      <c r="D287" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="E287" s="53" t="s">
+        <v>49</v>
+      </c>
       <c r="F287" s="56"/>
       <c r="G287" s="56"/>
-      <c r="H287" s="57"/>
-      <c r="I287" s="53"/>
+      <c r="H287" s="57" t="s">
+        <v>395</v>
+      </c>
+      <c r="I287" s="53" t="s">
+        <v>148</v>
+      </c>
     </row>
     <row r="288" spans="1:9">
       <c r="A288" s="48"/>
@@ -25570,7 +25691,7 @@
         <v>1145</v>
       </c>
       <c r="L59" s="66" t="s">
-        <v>1135</v>
+        <v>1130</v>
       </c>
       <c r="M59" s="66"/>
       <c r="N59" s="66" t="s">
@@ -27116,7 +27237,7 @@
         <v>0</v>
       </c>
       <c r="L88" s="63" t="s">
-        <v>1136</v>
+        <v>1131</v>
       </c>
       <c r="M88" s="63"/>
       <c r="N88" s="63" t="s">
@@ -27376,7 +27497,7 @@
         <v>0</v>
       </c>
       <c r="L93" s="66" t="s">
-        <v>1120</v>
+        <v>1115</v>
       </c>
       <c r="M93" s="66"/>
       <c r="N93" s="63" t="s">
@@ -28791,11 +28912,11 @@
         <v>43</v>
       </c>
       <c r="G120" s="64">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H120" s="63">
         <f t="shared" si="7"/>
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="I120" s="63">
         <f>IF(D120&lt;&gt;"",D120,IFERROR(E120/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -28807,10 +28928,10 @@
       </c>
       <c r="K120" s="63">
         <f t="shared" si="6"/>
-        <v>1256.859999999999</v>
+        <v>3351.6266666666638</v>
       </c>
       <c r="L120" s="63" t="s">
-        <v>1090</v>
+        <v>1194</v>
       </c>
       <c r="M120" s="63" t="s">
         <v>49</v>
@@ -28820,7 +28941,7 @@
       </c>
       <c r="O120" s="63"/>
       <c r="P120" s="63" t="s">
-        <v>1091</v>
+        <v>1195</v>
       </c>
       <c r="Q120" s="63"/>
       <c r="R120" s="63"/>
@@ -29918,7 +30039,7 @@
         <v>0</v>
       </c>
       <c r="L128" s="63" t="s">
-        <v>1082</v>
+        <v>1079</v>
       </c>
       <c r="M128" s="63"/>
       <c r="N128" s="63" t="s">
@@ -30878,10 +30999,10 @@
         <v>1200</v>
       </c>
       <c r="F147" s="76">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G147" s="76">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H147" s="75">
         <f t="shared" si="8"/>
@@ -30893,23 +31014,21 @@
       </c>
       <c r="J147" s="75">
         <f t="shared" si="9"/>
-        <v>5752</v>
+        <v>7190</v>
       </c>
       <c r="K147" s="75">
         <f t="shared" si="10"/>
-        <v>1438</v>
+        <v>0</v>
       </c>
       <c r="L147" s="66" t="s">
-        <v>1079</v>
+        <v>1191</v>
       </c>
       <c r="M147" s="66"/>
       <c r="N147" s="66" t="s">
-        <v>589</v>
+        <v>504</v>
       </c>
       <c r="O147" s="66"/>
-      <c r="P147" s="66" t="s">
-        <v>1080</v>
-      </c>
+      <c r="P147" s="66"/>
       <c r="Q147" s="66"/>
       <c r="R147" s="66"/>
       <c r="S147" s="66"/>
@@ -30954,7 +31073,7 @@
         <v>1004</v>
       </c>
       <c r="L148" s="63" t="s">
-        <v>1163</v>
+        <v>1156</v>
       </c>
       <c r="M148" s="63"/>
       <c r="N148" s="63" t="s">
@@ -31006,7 +31125,7 @@
         <v>0</v>
       </c>
       <c r="L149" s="66" t="s">
-        <v>1164</v>
+        <v>1157</v>
       </c>
       <c r="M149" s="66"/>
       <c r="N149" s="66" t="s">
@@ -31274,14 +31393,14 @@
         <v>949</v>
       </c>
       <c r="L154" s="63" t="s">
-        <v>1123</v>
+        <v>1118</v>
       </c>
       <c r="M154" s="63"/>
       <c r="N154" s="63" t="s">
         <v>589</v>
       </c>
       <c r="O154" s="63" t="s">
-        <v>1119</v>
+        <v>1114</v>
       </c>
       <c r="P154" s="63"/>
       <c r="Q154" s="63"/>
@@ -31328,14 +31447,14 @@
         <v>949</v>
       </c>
       <c r="L155" s="66" t="s">
-        <v>1147</v>
+        <v>1142</v>
       </c>
       <c r="M155" s="66"/>
       <c r="N155" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O155" s="66" t="s">
-        <v>1119</v>
+        <v>1114</v>
       </c>
       <c r="P155" s="66"/>
       <c r="Q155" s="66"/>
@@ -31382,7 +31501,7 @@
         <v>1900</v>
       </c>
       <c r="L156" s="63" t="s">
-        <v>1124</v>
+        <v>1119</v>
       </c>
       <c r="M156" s="63"/>
       <c r="N156" s="63" t="s">
@@ -31804,7 +31923,7 @@
         <v>0</v>
       </c>
       <c r="L164" s="63" t="s">
-        <v>1170</v>
+        <v>1163</v>
       </c>
       <c r="M164" s="63"/>
       <c r="N164" s="63" t="s">
@@ -31910,7 +32029,7 @@
         <v>1212</v>
       </c>
       <c r="L166" s="63" t="s">
-        <v>1103</v>
+        <v>1098</v>
       </c>
       <c r="M166" s="63"/>
       <c r="N166" s="63" t="s">
@@ -31918,7 +32037,7 @@
       </c>
       <c r="O166" s="63"/>
       <c r="P166" s="63" t="s">
-        <v>1104</v>
+        <v>1099</v>
       </c>
       <c r="Q166" s="63"/>
       <c r="R166" s="63"/>
@@ -32386,7 +32505,7 @@
         <v>3491.25</v>
       </c>
       <c r="L175" s="66" t="s">
-        <v>1110</v>
+        <v>1105</v>
       </c>
       <c r="M175" s="66"/>
       <c r="N175" s="66" t="s">
@@ -32394,7 +32513,7 @@
       </c>
       <c r="O175" s="66"/>
       <c r="P175" s="66" t="s">
-        <v>1109</v>
+        <v>1104</v>
       </c>
       <c r="Q175" s="66"/>
       <c r="R175" s="66"/>
@@ -32706,14 +32825,14 @@
         <v>3057</v>
       </c>
       <c r="L181" s="66" t="s">
-        <v>1117</v>
+        <v>1112</v>
       </c>
       <c r="M181" s="66"/>
       <c r="N181" s="66" t="s">
         <v>589</v>
       </c>
       <c r="O181" s="66" t="s">
-        <v>1118</v>
+        <v>1113</v>
       </c>
       <c r="P181" s="66" t="s">
         <v>955</v>
@@ -32813,7 +32932,7 @@
         <v>2095</v>
       </c>
       <c r="L183" s="66" t="s">
-        <v>1150</v>
+        <v>1145</v>
       </c>
       <c r="M183" s="66"/>
       <c r="N183" s="66" t="s">
@@ -32865,7 +32984,7 @@
         <v>891</v>
       </c>
       <c r="L184" s="63" t="s">
-        <v>1156</v>
+        <v>1149</v>
       </c>
       <c r="M184" s="63"/>
       <c r="N184" s="63" t="s">
@@ -33069,7 +33188,7 @@
         <v>0</v>
       </c>
       <c r="L188" s="63" t="s">
-        <v>1144</v>
+        <v>1139</v>
       </c>
       <c r="M188" s="63"/>
       <c r="N188" s="63" t="s">
@@ -33121,7 +33240,7 @@
         <v>1782</v>
       </c>
       <c r="L189" s="66" t="s">
-        <v>1157</v>
+        <v>1150</v>
       </c>
       <c r="M189" s="66"/>
       <c r="N189" s="66" t="s">
@@ -33129,7 +33248,7 @@
       </c>
       <c r="O189" s="66"/>
       <c r="P189" s="66" t="s">
-        <v>1158</v>
+        <v>1151</v>
       </c>
       <c r="Q189" s="66"/>
       <c r="R189" s="66"/>
@@ -33273,14 +33392,14 @@
         <v>1616</v>
       </c>
       <c r="L192" s="63" t="s">
-        <v>1093</v>
+        <v>1088</v>
       </c>
       <c r="M192" s="63"/>
       <c r="N192" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P192" s="58" t="s">
-        <v>1094</v>
+        <v>1089</v>
       </c>
       <c r="S192" s="58"/>
       <c r="T192" s="58"/>
@@ -33473,14 +33592,14 @@
         <v>3985</v>
       </c>
       <c r="L196" s="63" t="s">
-        <v>1168</v>
+        <v>1161</v>
       </c>
       <c r="M196" s="63"/>
       <c r="N196" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P196" s="58" t="s">
-        <v>1169</v>
+        <v>1162</v>
       </c>
       <c r="S196" s="58"/>
       <c r="T196" s="58"/>
@@ -33600,10 +33719,10 @@
         <v>850</v>
       </c>
       <c r="F199" s="76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G199" s="76">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H199" s="75">
         <f t="shared" si="12"/>
@@ -33615,29 +33734,31 @@
       </c>
       <c r="J199" s="75">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>467</v>
       </c>
       <c r="K199" s="75">
         <f t="shared" si="14"/>
-        <v>1868</v>
-      </c>
-      <c r="L199" s="66"/>
+        <v>1401</v>
+      </c>
+      <c r="L199" s="66" t="s">
+        <v>1187</v>
+      </c>
       <c r="M199" s="66"/>
       <c r="N199" s="58" t="s">
-        <v>678</v>
+        <v>589</v>
       </c>
       <c r="P199" s="58" t="s">
-        <v>1002</v>
+        <v>1188</v>
       </c>
       <c r="S199" s="58"/>
       <c r="T199" s="58"/>
     </row>
     <row r="200" spans="1:20" ht="30" customHeight="1">
       <c r="A200" s="63" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B200" s="66" t="s">
         <v>1003</v>
-      </c>
-      <c r="B200" s="66" t="s">
-        <v>1004</v>
       </c>
       <c r="C200" s="66" t="s">
         <v>95</v>
@@ -33671,24 +33792,24 @@
         <v>2598</v>
       </c>
       <c r="L200" s="63" t="s">
-        <v>1097</v>
+        <v>1092</v>
       </c>
       <c r="M200" s="63"/>
       <c r="N200" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P200" s="58" t="s">
-        <v>1098</v>
+        <v>1093</v>
       </c>
       <c r="S200" s="58"/>
       <c r="T200" s="58"/>
     </row>
     <row r="201" spans="1:20" ht="15" customHeight="1">
       <c r="A201" s="66" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B201" s="63" t="s">
         <v>1005</v>
-      </c>
-      <c r="B201" s="63" t="s">
-        <v>1006</v>
       </c>
       <c r="C201" s="63" t="s">
         <v>95</v>
@@ -33722,24 +33843,24 @@
         <v>724</v>
       </c>
       <c r="L201" s="66" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="M201" s="66"/>
       <c r="N201" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P201" s="58" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="S201" s="58"/>
       <c r="T201" s="58"/>
     </row>
     <row r="202" spans="1:20" ht="15" customHeight="1">
       <c r="A202" s="63" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B202" s="66" t="s">
         <v>1009</v>
-      </c>
-      <c r="B202" s="66" t="s">
-        <v>1010</v>
       </c>
       <c r="C202" s="66" t="s">
         <v>95</v>
@@ -33751,10 +33872,10 @@
         <v>1500</v>
       </c>
       <c r="F202" s="78">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G202" s="78">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H202" s="77">
         <f t="shared" si="12"/>
@@ -33766,31 +33887,31 @@
       </c>
       <c r="J202" s="77">
         <f t="shared" si="13"/>
-        <v>2820</v>
+        <v>4700</v>
       </c>
       <c r="K202" s="77">
         <f t="shared" si="14"/>
-        <v>2820</v>
+        <v>940</v>
       </c>
       <c r="L202" s="63" t="s">
-        <v>1153</v>
+        <v>1181</v>
       </c>
       <c r="M202" s="63"/>
       <c r="N202" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="58" t="s">
-        <v>1154</v>
+        <v>1182</v>
       </c>
       <c r="S202" s="58"/>
       <c r="T202" s="58"/>
     </row>
     <row r="203" spans="1:20" ht="15" customHeight="1">
       <c r="A203" s="66" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B203" s="63" t="s">
         <v>1011</v>
-      </c>
-      <c r="B203" s="63" t="s">
-        <v>1012</v>
       </c>
       <c r="C203" s="63" t="s">
         <v>95</v>
@@ -33824,24 +33945,24 @@
         <v>0</v>
       </c>
       <c r="L203" s="66" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="M203" s="66"/>
       <c r="N203" s="58" t="s">
         <v>504</v>
       </c>
       <c r="P203" s="58" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="S203" s="58"/>
       <c r="T203" s="58"/>
     </row>
     <row r="204" spans="1:20" ht="15" customHeight="1">
       <c r="A204" s="63" t="s">
+        <v>1014</v>
+      </c>
+      <c r="B204" s="63" t="s">
         <v>1015</v>
-      </c>
-      <c r="B204" s="63" t="s">
-        <v>1016</v>
       </c>
       <c r="C204" s="63" t="s">
         <v>95</v>
@@ -33875,24 +33996,24 @@
         <v>880</v>
       </c>
       <c r="L204" s="63" t="s">
-        <v>1129</v>
+        <v>1124</v>
       </c>
       <c r="M204" s="63"/>
       <c r="N204" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P204" s="58" t="s">
-        <v>1128</v>
+        <v>1123</v>
       </c>
       <c r="S204" s="58"/>
       <c r="T204" s="58"/>
     </row>
     <row r="205" spans="1:20" ht="15" customHeight="1">
       <c r="A205" s="66" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B205" s="66" t="s">
         <v>1017</v>
-      </c>
-      <c r="B205" s="66" t="s">
-        <v>1018</v>
       </c>
       <c r="C205" s="66" t="s">
         <v>95</v>
@@ -33926,24 +34047,24 @@
         <v>1522</v>
       </c>
       <c r="L205" s="66" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="M205" s="66"/>
       <c r="N205" s="58" t="s">
         <v>678</v>
       </c>
       <c r="P205" s="58" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="S205" s="58"/>
       <c r="T205" s="58"/>
     </row>
     <row r="206" spans="1:20" ht="15" customHeight="1">
       <c r="A206" s="63" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B206" s="63" t="s">
         <v>1021</v>
-      </c>
-      <c r="B206" s="63" t="s">
-        <v>1022</v>
       </c>
       <c r="C206" s="63" t="s">
         <v>95</v>
@@ -33984,17 +34105,17 @@
         <v>504</v>
       </c>
       <c r="P206" s="58" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="S206" s="58"/>
       <c r="T206" s="58"/>
     </row>
     <row r="207" spans="1:20" ht="15" customHeight="1">
       <c r="A207" s="66" t="s">
+        <v>1023</v>
+      </c>
+      <c r="B207" s="66" t="s">
         <v>1024</v>
-      </c>
-      <c r="B207" s="66" t="s">
-        <v>1025</v>
       </c>
       <c r="C207" s="66" t="s">
         <v>95</v>
@@ -34028,24 +34149,24 @@
         <v>3312</v>
       </c>
       <c r="L207" s="66" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="M207" s="66"/>
       <c r="N207" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P207" s="58" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="S207" s="58"/>
       <c r="T207" s="58"/>
     </row>
     <row r="208" spans="1:20" ht="30" customHeight="1">
       <c r="A208" s="63" t="s">
+        <v>1027</v>
+      </c>
+      <c r="B208" s="63" t="s">
         <v>1028</v>
-      </c>
-      <c r="B208" s="63" t="s">
-        <v>1029</v>
       </c>
       <c r="C208" s="63" t="s">
         <v>95</v>
@@ -34084,17 +34205,17 @@
         <v>678</v>
       </c>
       <c r="P208" s="58" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="S208" s="58"/>
       <c r="T208" s="58"/>
     </row>
     <row r="209" spans="1:20" ht="15" customHeight="1">
       <c r="A209" s="66" t="s">
+        <v>1030</v>
+      </c>
+      <c r="B209" s="63" t="s">
         <v>1031</v>
-      </c>
-      <c r="B209" s="63" t="s">
-        <v>1032</v>
       </c>
       <c r="C209" s="63" t="s">
         <v>95</v>
@@ -34128,24 +34249,24 @@
         <v>982</v>
       </c>
       <c r="L209" s="66" t="s">
-        <v>1096</v>
+        <v>1091</v>
       </c>
       <c r="M209" s="66"/>
       <c r="N209" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P209" s="58" t="s">
-        <v>1095</v>
+        <v>1090</v>
       </c>
       <c r="S209" s="58"/>
       <c r="T209" s="58"/>
     </row>
     <row r="210" spans="1:20" ht="15" customHeight="1">
       <c r="A210" s="63" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B210" s="66" t="s">
         <v>1033</v>
-      </c>
-      <c r="B210" s="66" t="s">
-        <v>1034</v>
       </c>
       <c r="C210" s="66" t="s">
         <v>95</v>
@@ -34184,14 +34305,14 @@
         <v>678</v>
       </c>
       <c r="P210" s="58" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="S210" s="58"/>
       <c r="T210" s="58"/>
     </row>
     <row r="211" spans="1:20" ht="15" customHeight="1">
       <c r="A211" s="66" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B211" s="63" t="s">
         <v>901</v>
@@ -34233,17 +34354,17 @@
         <v>678</v>
       </c>
       <c r="P211" s="58" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="S211" s="58"/>
       <c r="T211" s="58"/>
     </row>
     <row r="212" spans="1:20" ht="15" customHeight="1">
       <c r="A212" s="63" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="B212" s="66" t="s">
-        <v>1115</v>
+        <v>1110</v>
       </c>
       <c r="C212" s="66" t="s">
         <v>95</v>
@@ -34286,10 +34407,10 @@
     </row>
     <row r="213" spans="1:20" ht="15" customHeight="1">
       <c r="A213" s="66" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="B213" s="63" t="s">
-        <v>1166</v>
+        <v>1159</v>
       </c>
       <c r="C213" s="63" t="s">
         <v>95</v>
@@ -34323,24 +34444,24 @@
         <v>4440</v>
       </c>
       <c r="L213" s="66" t="s">
-        <v>1167</v>
+        <v>1160</v>
       </c>
       <c r="M213" s="66"/>
       <c r="N213" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P213" s="58" t="s">
-        <v>1172</v>
+        <v>1165</v>
       </c>
       <c r="S213" s="58"/>
       <c r="T213" s="58"/>
     </row>
     <row r="214" spans="1:20" ht="15" customHeight="1">
       <c r="A214" s="63" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="B214" s="63" t="s">
-        <v>1173</v>
+        <v>1166</v>
       </c>
       <c r="C214" s="63" t="s">
         <v>95</v>
@@ -34379,17 +34500,17 @@
         <v>678</v>
       </c>
       <c r="P214" s="58" t="s">
-        <v>1174</v>
+        <v>1167</v>
       </c>
       <c r="S214" s="58"/>
       <c r="T214" s="58"/>
     </row>
     <row r="215" spans="1:20" ht="15" customHeight="1">
       <c r="A215" s="66" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="B215" s="66" t="s">
-        <v>1175</v>
+        <v>1168</v>
       </c>
       <c r="C215" s="66" t="s">
         <v>95</v>
@@ -34428,14 +34549,14 @@
         <v>678</v>
       </c>
       <c r="P215" s="58" t="s">
-        <v>1176</v>
+        <v>1169</v>
       </c>
       <c r="S215" s="58"/>
       <c r="T215" s="58"/>
     </row>
     <row r="216" spans="1:20" ht="30">
       <c r="A216" s="63" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B216" s="63" t="s">
         <v>1001</v>
@@ -34477,17 +34598,17 @@
         <v>678</v>
       </c>
       <c r="P216" s="58" t="s">
-        <v>1177</v>
+        <v>1170</v>
       </c>
       <c r="S216" s="58"/>
       <c r="T216" s="58"/>
     </row>
     <row r="217" spans="1:20" ht="15" customHeight="1">
       <c r="A217" s="66" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="B217" s="66" t="s">
-        <v>1178</v>
+        <v>1171</v>
       </c>
       <c r="C217" s="66" t="s">
         <v>95</v>
@@ -34526,17 +34647,17 @@
         <v>678</v>
       </c>
       <c r="P217" s="58" t="s">
-        <v>1179</v>
+        <v>1172</v>
       </c>
       <c r="S217" s="58"/>
       <c r="T217" s="58"/>
     </row>
     <row r="218" spans="1:20" ht="30">
       <c r="A218" s="63" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B218" s="63" t="s">
-        <v>1181</v>
+        <v>1174</v>
       </c>
       <c r="C218" s="63" t="s">
         <v>95</v>
@@ -34575,17 +34696,17 @@
         <v>678</v>
       </c>
       <c r="P218" s="58" t="s">
-        <v>1180</v>
+        <v>1173</v>
       </c>
       <c r="S218" s="58"/>
       <c r="T218" s="58"/>
     </row>
     <row r="219" spans="1:20" ht="15" customHeight="1">
       <c r="A219" s="66" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B219" s="63" t="s">
-        <v>1182</v>
+        <v>1175</v>
       </c>
       <c r="C219" s="63" t="s">
         <v>95</v>
@@ -34624,17 +34745,17 @@
         <v>678</v>
       </c>
       <c r="P219" s="58" t="s">
-        <v>1183</v>
+        <v>1176</v>
       </c>
       <c r="S219" s="58"/>
       <c r="T219" s="58"/>
     </row>
     <row r="220" spans="1:20" ht="30">
       <c r="A220" s="63" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B220" s="66" t="s">
-        <v>1184</v>
+        <v>1177</v>
       </c>
       <c r="C220" s="66" t="s">
         <v>95</v>
@@ -34673,14 +34794,14 @@
         <v>678</v>
       </c>
       <c r="P220" s="58" t="s">
-        <v>1185</v>
+        <v>1178</v>
       </c>
       <c r="S220" s="58"/>
       <c r="T220" s="58"/>
     </row>
     <row r="221" spans="1:20" ht="15" customHeight="1">
       <c r="A221" s="66" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B221" s="63"/>
       <c r="C221" s="63"/>
@@ -34715,7 +34836,7 @@
     </row>
     <row r="222" spans="1:20" ht="15" customHeight="1">
       <c r="A222" s="63" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B222" s="66"/>
       <c r="C222" s="66"/>
@@ -34750,7 +34871,7 @@
     </row>
     <row r="223" spans="1:20" ht="15" customHeight="1">
       <c r="A223" s="66" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B223" s="63"/>
       <c r="C223" s="63"/>
@@ -34785,7 +34906,7 @@
     </row>
     <row r="224" spans="1:20" ht="15" customHeight="1">
       <c r="A224" s="63" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B224" s="63"/>
       <c r="C224" s="63"/>
@@ -34820,7 +34941,7 @@
     </row>
     <row r="225" spans="1:20" ht="15" customHeight="1">
       <c r="A225" s="66" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B225" s="66"/>
       <c r="C225" s="66"/>
@@ -34855,7 +34976,7 @@
     </row>
     <row r="226" spans="1:20" ht="15" customHeight="1">
       <c r="A226" s="63" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B226" s="63"/>
       <c r="C226" s="63"/>
@@ -38770,7 +38891,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="15" customHeight="1">
       <c r="A1" s="92" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B1" s="92"/>
     </row>
@@ -38779,7 +38900,7 @@
         <v>42</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="13.5" customHeight="1">
@@ -38811,25 +38932,25 @@
         <v>42</v>
       </c>
       <c r="B7" s="83" t="s">
+        <v>1054</v>
+      </c>
+      <c r="C7" s="83" t="s">
         <v>1055</v>
       </c>
-      <c r="C7" s="83" t="s">
+      <c r="D7" s="83" t="s">
         <v>1056</v>
       </c>
-      <c r="D7" s="83" t="s">
+      <c r="E7" s="83" t="s">
         <v>1057</v>
       </c>
-      <c r="E7" s="83" t="s">
+      <c r="F7" s="83" t="s">
         <v>1058</v>
       </c>
-      <c r="F7" s="83" t="s">
+      <c r="G7" s="83" t="s">
         <v>1059</v>
       </c>
-      <c r="G7" s="83" t="s">
+      <c r="H7" s="83" t="s">
         <v>1060</v>
-      </c>
-      <c r="H7" s="83" t="s">
-        <v>1061</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="13.5" customHeight="1">
@@ -38838,15 +38959,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>249742</v>
+        <v>249928</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>172936.33333333334</v>
+        <v>172998.33333333334</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>76805.666666666657</v>
+        <v>76929.666666666657</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38854,7 +38975,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>76805.666666666657</v>
+        <v>76929.666666666657</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -38862,7 +38983,7 @@
       </c>
       <c r="H8" s="85">
         <f>F8-G8</f>
-        <v>58502.32666666666</v>
+        <v>58626.32666666666</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -38875,11 +38996,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>172936.33333333334</v>
+        <v>172998.33333333334</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>63530.666666666657</v>
+        <v>63468.666666666657</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38887,7 +39008,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>63530.666666666657</v>
+        <v>63468.666666666657</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -38895,7 +39016,7 @@
       </c>
       <c r="H9" s="86">
         <f>F9-G9</f>
-        <v>21891.336666666655</v>
+        <v>21829.336666666655</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -38908,11 +39029,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>172936.33333333334</v>
+        <v>172998.33333333334</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-140336.33333333334</v>
+        <v>-140398.33333333334</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -38920,7 +39041,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-140336.33333333334</v>
+        <v>-140398.33333333334</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -38928,12 +39049,12 @@
       </c>
       <c r="H10" s="85">
         <f>F10-G10</f>
-        <v>-80393.663333333345</v>
+        <v>-80455.663333333345</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">
       <c r="A12" s="93" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B12" s="93"/>
       <c r="C12" s="93"/>
@@ -38946,13 +39067,13 @@
         <v>98</v>
       </c>
       <c r="B13" s="83" t="s">
+        <v>1062</v>
+      </c>
+      <c r="C13" s="83" t="s">
         <v>1063</v>
       </c>
-      <c r="C13" s="83" t="s">
+      <c r="D13" s="83" t="s">
         <v>1064</v>
-      </c>
-      <c r="D13" s="83" t="s">
-        <v>1065</v>
       </c>
       <c r="E13" s="83" t="s">
         <v>99</v>
@@ -38966,7 +39087,7 @@
         <v>45952</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C14" s="9" t="s">
         <v>51</v>
@@ -38984,7 +39105,7 @@
         <v>45952</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>51</v>
@@ -39038,7 +39159,7 @@
         <v>45970</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>50</v>
@@ -39056,7 +39177,7 @@
         <v>45970</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>50</v>
@@ -39074,7 +39195,7 @@
         <v>45973</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C20" s="9" t="s">
         <v>50</v>
@@ -39092,7 +39213,7 @@
         <v>45973</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>49</v>
@@ -39110,7 +39231,7 @@
         <v>46058</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C22" s="9" t="s">
         <v>51</v>
@@ -39146,7 +39267,7 @@
         <v>46059</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>49</v>
@@ -39182,7 +39303,7 @@
         <v>46093</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C26" s="9" t="s">
         <v>50</v>
@@ -39200,7 +39321,7 @@
         <v>46093</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>51</v>
@@ -39283,7 +39404,7 @@
     </row>
     <row r="58" spans="2:2" ht="13.5" customHeight="1">
       <c r="B58" s="6" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
     </row>
   </sheetData>
@@ -39313,7 +39434,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="13.5" customHeight="1">
       <c r="A1" s="90" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="84" customFormat="1" ht="13.5" customHeight="1">
@@ -39321,22 +39442,22 @@
         <v>42</v>
       </c>
       <c r="B3" s="83" t="s">
+        <v>1068</v>
+      </c>
+      <c r="C3" s="83" t="s">
+        <v>1053</v>
+      </c>
+      <c r="D3" s="83" t="s">
         <v>1069</v>
       </c>
-      <c r="C3" s="83" t="s">
-        <v>1054</v>
-      </c>
-      <c r="D3" s="83" t="s">
+      <c r="E3" s="83" t="s">
         <v>1070</v>
       </c>
-      <c r="E3" s="83" t="s">
+      <c r="F3" s="83" t="s">
         <v>1071</v>
       </c>
-      <c r="F3" s="83" t="s">
+      <c r="G3" s="83" t="s">
         <v>1072</v>
-      </c>
-      <c r="G3" s="83" t="s">
-        <v>1073</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="13.5" customHeight="1">
@@ -39345,7 +39466,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>392221</v>
+        <v>398320</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -39353,11 +39474,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>153155.625</v>
+        <v>155189.03159999999</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>239065.375</v>
+        <v>243130.96840000001</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39365,7 +39486,7 @@
       </c>
       <c r="G4" s="85">
         <f>E4+F4</f>
-        <v>101755.34899999999</v>
+        <v>105820.9424</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -39382,11 +39503,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>153063.75</v>
+        <v>155095.9368</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-98439.75</v>
+        <v>-100471.9368</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39394,7 +39515,7 @@
       </c>
       <c r="G5" s="86">
         <f>E5+F5</f>
-        <v>-26852.707999999999</v>
+        <v>-28884.894799999995</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -39411,11 +39532,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>153155.625</v>
+        <v>155189.03159999999</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-140625.625</v>
+        <v>-142659.03159999999</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39423,7 +39544,7 @@
       </c>
       <c r="G6" s="85">
         <f>E6+F6</f>
-        <v>-74902.640999999989</v>
+        <v>-76936.047599999976</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">
@@ -39433,27 +39554,27 @@
     </row>
     <row r="10" spans="1:7" ht="13.5" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="13.5" customHeight="1">
       <c r="A11" s="6" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="13.5" customHeight="1">
       <c r="A12" s="6" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="13.5" customHeight="1">
       <c r="A13" s="6" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="13.5" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
7/25 & 7/26 Sales
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2539D27-BCD0-8F46-96B6-5D9251EBB0C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07D14D5B-0541-8F45-88E8-8609962C9C2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3060" uniqueCount="1201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3078" uniqueCount="1207">
   <si>
     <t>Notes:</t>
   </si>
@@ -3586,9 +3586,6 @@
     <t>Mul Tissue saree Collection</t>
   </si>
   <si>
-    <t>Rose pink, dusty lavender, brick red, champagne, chocolate brown, magenta</t>
-  </si>
-  <si>
     <t>Lekha</t>
   </si>
   <si>
@@ -3667,6 +3664,27 @@
   </si>
   <si>
     <t>CHR-189 - Light Green</t>
+  </si>
+  <si>
+    <t>Jisha Bank -950</t>
+  </si>
+  <si>
+    <t>CHR-95 Chinon Silk</t>
+  </si>
+  <si>
+    <t>Banarasi Saree with Rich Gold Zari Border</t>
+  </si>
+  <si>
+    <t>Black</t>
+  </si>
+  <si>
+    <t>CHR-219 Brick red</t>
+  </si>
+  <si>
+    <t>Baby khadeeja (brick red) - 1250</t>
+  </si>
+  <si>
+    <t>Rose pink, dusty lavender, champagne, chocolate brown, magenta</t>
   </si>
 </sst>
 </file>
@@ -4546,7 +4564,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>289</c:v>
+                  <c:v>291</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>95</c:v>
@@ -4649,7 +4667,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>181</c:v>
+                  <c:v>184</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>53</c:v>
@@ -4982,7 +5000,7 @@
                   <c:v>56434</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>136591.19666666666</c:v>
+                  <c:v>138930.19666666666</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5315,7 +5333,7 @@
                   <c:v>99043</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>65078</c:v>
+                  <c:v>67350</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5475,7 +5493,7 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>51746</c:v>
+                  <c:v>53946</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5915,7 +5933,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-13332</c:v>
+                  <c:v>-13404</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6379,10 +6397,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>389</c:v>
+                  <c:v>391</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>6</c:v>
+                  <c:v>45</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7554,7 +7572,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>519225</v>
+        <v>521497</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7569,7 +7587,7 @@
       </c>
       <c r="B4" s="10">
         <f>SUMIFS(Sales!C:C, Sales!I:I, "Completed")</f>
-        <v>472214</v>
+        <v>473464</v>
       </c>
       <c r="E4" s="9" t="str">
         <f>PartnerShares!A3</f>
@@ -7586,7 +7604,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>480244</v>
+        <v>482444</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7603,7 +7621,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-47011</v>
+        <v>-48033</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7638,7 +7656,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>58779.66</v>
+        <v>60294.32666666666</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7648,7 +7666,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>21752.67</v>
+        <v>20995.336666666655</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7658,7 +7676,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-80532.33</v>
+        <v>-81289.663333333345</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7697,15 +7715,15 @@
       </c>
       <c r="B18" s="10">
         <f>PartnerShares!B8</f>
-        <v>250158</v>
+        <v>252430</v>
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>173075</v>
+        <v>173832.33333333334</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>77083</v>
+        <v>78597.666666666657</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7713,11 +7731,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>58779.66</v>
+        <v>60294.32666666666</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹58,780</v>
+        <v>Receive ₹60,294</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7731,11 +7749,11 @@
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>173075</v>
+        <v>173832.33333333334</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>63392</v>
+        <v>62634.666666666657</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7743,11 +7761,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>21752.67</v>
+        <v>20995.336666666655</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹21,753</v>
+        <v>Receive ₹20,995</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7761,11 +7779,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>173075</v>
+        <v>173832.33333333334</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-140475</v>
+        <v>-141232.33333333334</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7773,11 +7791,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-80532.33</v>
+        <v>-81289.663333333345</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹80,532</v>
+        <v>Pay ₹81,290</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -7815,15 +7833,15 @@
       </c>
       <c r="B26" s="10">
         <f>'Cash Pool'!B4</f>
-        <v>405060</v>
+        <v>406310</v>
       </c>
       <c r="C26" s="10">
         <f>'Cash Pool'!D4</f>
-        <v>157436.1476</v>
+        <v>157852.8976</v>
       </c>
       <c r="D26" s="10">
         <f>'Cash Pool'!E4</f>
-        <v>247623.8524</v>
+        <v>248457.1024</v>
       </c>
       <c r="E26" s="10">
         <f>'Cash Pool'!F4</f>
@@ -7831,11 +7849,11 @@
       </c>
       <c r="F26" s="13">
         <f>'Cash Pool'!G4</f>
-        <v>110313.82639999999</v>
+        <v>111147.07639999999</v>
       </c>
       <c r="G26" s="17" t="str">
         <f>IF(ROUND(F26,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F26),"#,##0"),IF(ROUND(F26,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F26),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹110,314</v>
+        <v>Pay ₹111,147</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="13.5" customHeight="1">
@@ -7849,11 +7867,11 @@
       </c>
       <c r="C27" s="12">
         <f>'Cash Pool'!D5</f>
-        <v>157341.70480000001</v>
+        <v>157758.20480000001</v>
       </c>
       <c r="D27" s="12">
         <f>'Cash Pool'!E5</f>
-        <v>-102717.70480000001</v>
+        <v>-103134.20480000001</v>
       </c>
       <c r="E27" s="12">
         <f>'Cash Pool'!F5</f>
@@ -7861,11 +7879,11 @@
       </c>
       <c r="F27" s="14">
         <f>'Cash Pool'!G5</f>
-        <v>-31130.662800000006</v>
+        <v>-31547.162800000006</v>
       </c>
       <c r="G27" s="18" t="str">
         <f>IF(ROUND(F27,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F27),"#,##0"),IF(ROUND(F27,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F27),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹31,131</v>
+        <v>Receive ₹31,547</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="13.5" customHeight="1">
@@ -7879,11 +7897,11 @@
       </c>
       <c r="C28" s="10">
         <f>'Cash Pool'!D6</f>
-        <v>157436.1476</v>
+        <v>157852.8976</v>
       </c>
       <c r="D28" s="10">
         <f>'Cash Pool'!E6</f>
-        <v>-144906.1476</v>
+        <v>-145322.8976</v>
       </c>
       <c r="E28" s="10">
         <f>'Cash Pool'!F6</f>
@@ -7891,11 +7909,11 @@
       </c>
       <c r="F28" s="13">
         <f>'Cash Pool'!G6</f>
-        <v>-79183.163599999985</v>
+        <v>-79599.913599999985</v>
       </c>
       <c r="G28" s="16" t="str">
         <f>IF(ROUND(F28,0)&gt;0,"Pay ₹"&amp;TEXT(ABS(F28),"#,##0"),IF(ROUND(F28,0)&lt;0,"Receive ₹"&amp;TEXT(ABS(F28),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹79,183</v>
+        <v>Receive ₹79,600</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="15.75" customHeight="1">
@@ -8007,7 +8025,7 @@
       </c>
       <c r="B3" s="20">
         <f ca="1">TODAY()</f>
-        <v>46224</v>
+        <v>46229</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15" customHeight="1">
@@ -8016,14 +8034,14 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>519225</v>
+        <v>521497</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
       </c>
       <c r="E5" s="21">
         <f>Summary!B4</f>
-        <v>472214</v>
+        <v>473464</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" customHeight="1">
@@ -8032,14 +8050,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-47011</v>
+        <v>-48033</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>184466.39666666667</v>
+        <v>186805.39666666667</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8091,7 +8109,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>389</v>
+        <v>391</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8115,7 +8133,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8192,15 +8210,15 @@
       </c>
       <c r="B16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A16)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>65078</v>
+        <v>67350</v>
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$995,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$995)=$B$7)*Sales!$C$2:$C$995),0)</f>
-        <v>51746</v>
+        <v>53946</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-13332</v>
+        <v>-13404</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8311,11 +8329,11 @@
       </c>
       <c r="G47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!F:F)</f>
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
@@ -8342,7 +8360,7 @@
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>136591.19666666666</v>
+        <v>138930.19666666666</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9859,16 +9877,32 @@
       </c>
     </row>
     <row r="102" spans="1:4" ht="15" customHeight="1">
-      <c r="A102" s="35"/>
-      <c r="B102" s="36"/>
-      <c r="C102" s="37"/>
-      <c r="D102" s="36"/>
+      <c r="A102" s="35">
+        <v>46225</v>
+      </c>
+      <c r="B102" s="36" t="s">
+        <v>49</v>
+      </c>
+      <c r="C102" s="37">
+        <v>142</v>
+      </c>
+      <c r="D102" s="36" t="s">
+        <v>119</v>
+      </c>
     </row>
     <row r="103" spans="1:4" ht="15" customHeight="1">
-      <c r="A103" s="38"/>
-      <c r="B103" s="39"/>
-      <c r="C103" s="40"/>
-      <c r="D103" s="39"/>
+      <c r="A103" s="38">
+        <v>46228</v>
+      </c>
+      <c r="B103" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="C103" s="40">
+        <v>2130</v>
+      </c>
+      <c r="D103" s="39" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="104" spans="1:4" ht="15" customHeight="1">
       <c r="A104" s="35"/>
@@ -11961,7 +11995,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:I292"/>
+  <dimension ref="A1:I330"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13"/>
   <cols>
     <col min="1" max="1" width="10" style="42" customWidth="1"/>
@@ -18397,7 +18431,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>148</v>
@@ -18904,7 +18938,7 @@
         <v>46220</v>
       </c>
       <c r="B282" s="49" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C282" s="50">
         <v>1500</v>
@@ -18918,7 +18952,7 @@
       <c r="F282" s="49"/>
       <c r="G282" s="49"/>
       <c r="H282" s="51" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="I282" s="49" t="s">
         <v>148</v>
@@ -18929,7 +18963,7 @@
         <v>46221</v>
       </c>
       <c r="B283" s="53" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="C283" s="54">
         <v>1100</v>
@@ -18943,7 +18977,7 @@
       <c r="F283" s="56"/>
       <c r="G283" s="56"/>
       <c r="H283" s="57" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="I283" s="53" t="s">
         <v>148</v>
@@ -18954,7 +18988,7 @@
         <v>46222</v>
       </c>
       <c r="B284" s="49" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="C284" s="50">
         <v>850</v>
@@ -18968,7 +19002,7 @@
       <c r="F284" s="49"/>
       <c r="G284" s="49"/>
       <c r="H284" s="51" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="I284" s="49" t="s">
         <v>148</v>
@@ -18979,7 +19013,7 @@
         <v>46222</v>
       </c>
       <c r="B285" s="53" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="C285" s="54">
         <v>1250</v>
@@ -18993,7 +19027,7 @@
       <c r="F285" s="56"/>
       <c r="G285" s="56"/>
       <c r="H285" s="57" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="I285" s="53" t="s">
         <v>148</v>
@@ -19004,7 +19038,7 @@
         <v>46222</v>
       </c>
       <c r="B286" s="49" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="C286" s="50">
         <v>700</v>
@@ -19029,7 +19063,7 @@
         <v>46222</v>
       </c>
       <c r="B287" s="53" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="C287" s="54">
         <v>699</v>
@@ -19054,7 +19088,7 @@
         <v>46223</v>
       </c>
       <c r="B288" s="49" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="C288" s="50">
         <v>1380</v>
@@ -19068,7 +19102,7 @@
       <c r="F288" s="49"/>
       <c r="G288" s="49"/>
       <c r="H288" s="51" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="I288" s="49" t="s">
         <v>148</v>
@@ -19079,7 +19113,7 @@
         <v>46224</v>
       </c>
       <c r="B289" s="53" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C289" s="54">
         <v>1380</v>
@@ -19093,7 +19127,7 @@
       <c r="F289" s="56"/>
       <c r="G289" s="56"/>
       <c r="H289" s="57" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="I289" s="53" t="s">
         <v>148</v>
@@ -19104,7 +19138,7 @@
         <v>46224</v>
       </c>
       <c r="B290" s="49" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="C290" s="50">
         <v>1380</v>
@@ -19118,33 +19152,475 @@
       <c r="F290" s="49"/>
       <c r="G290" s="49"/>
       <c r="H290" s="51" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="I290" s="49" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="291" spans="1:9">
-      <c r="A291" s="52"/>
-      <c r="B291" s="53"/>
-      <c r="C291" s="54"/>
+    <row r="291" spans="1:9" ht="14">
+      <c r="A291" s="52">
+        <v>46228</v>
+      </c>
+      <c r="B291" s="53" t="s">
+        <v>1109</v>
+      </c>
+      <c r="C291" s="54">
+        <v>950</v>
+      </c>
       <c r="D291" s="53"/>
       <c r="E291" s="53"/>
       <c r="F291" s="56"/>
       <c r="G291" s="56"/>
-      <c r="H291" s="57"/>
-      <c r="I291" s="53"/>
-    </row>
-    <row r="292" spans="1:9">
-      <c r="A292" s="48"/>
-      <c r="B292" s="49"/>
-      <c r="C292" s="50"/>
-      <c r="D292" s="49"/>
-      <c r="E292" s="49"/>
+      <c r="H291" s="57" t="s">
+        <v>1201</v>
+      </c>
+      <c r="I291" s="53" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="292" spans="1:9" ht="14">
+      <c r="A292" s="48">
+        <v>46228</v>
+      </c>
+      <c r="B292" s="49" t="s">
+        <v>186</v>
+      </c>
+      <c r="C292" s="50">
+        <v>1250</v>
+      </c>
+      <c r="D292" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E292" s="49" t="s">
+        <v>49</v>
+      </c>
       <c r="F292" s="49"/>
       <c r="G292" s="49"/>
-      <c r="H292" s="51"/>
-      <c r="I292" s="49"/>
+      <c r="H292" s="51" t="s">
+        <v>1204</v>
+      </c>
+      <c r="I292" s="49" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="293" spans="1:9">
+      <c r="A293" s="52"/>
+      <c r="B293" s="53"/>
+      <c r="C293" s="54"/>
+      <c r="D293" s="53"/>
+      <c r="E293" s="53"/>
+      <c r="F293" s="56"/>
+      <c r="G293" s="56"/>
+      <c r="H293" s="57"/>
+      <c r="I293" s="53"/>
+    </row>
+    <row r="294" spans="1:9">
+      <c r="A294" s="48"/>
+      <c r="B294" s="49"/>
+      <c r="C294" s="50"/>
+      <c r="D294" s="49"/>
+      <c r="E294" s="49"/>
+      <c r="F294" s="49"/>
+      <c r="G294" s="49"/>
+      <c r="H294" s="51"/>
+      <c r="I294" s="49"/>
+    </row>
+    <row r="295" spans="1:9">
+      <c r="A295" s="52"/>
+      <c r="B295" s="53"/>
+      <c r="C295" s="54"/>
+      <c r="D295" s="53"/>
+      <c r="E295" s="53"/>
+      <c r="F295" s="56"/>
+      <c r="G295" s="56"/>
+      <c r="H295" s="57"/>
+      <c r="I295" s="53"/>
+    </row>
+    <row r="296" spans="1:9">
+      <c r="A296" s="48"/>
+      <c r="B296" s="49"/>
+      <c r="C296" s="50"/>
+      <c r="D296" s="49"/>
+      <c r="E296" s="49"/>
+      <c r="F296" s="49"/>
+      <c r="G296" s="49"/>
+      <c r="H296" s="51"/>
+      <c r="I296" s="49"/>
+    </row>
+    <row r="297" spans="1:9">
+      <c r="A297" s="52"/>
+      <c r="B297" s="53"/>
+      <c r="C297" s="54"/>
+      <c r="D297" s="53"/>
+      <c r="E297" s="53"/>
+      <c r="F297" s="56"/>
+      <c r="G297" s="56"/>
+      <c r="H297" s="57"/>
+      <c r="I297" s="53"/>
+    </row>
+    <row r="298" spans="1:9">
+      <c r="A298" s="48"/>
+      <c r="B298" s="49"/>
+      <c r="C298" s="50"/>
+      <c r="D298" s="49"/>
+      <c r="E298" s="49"/>
+      <c r="F298" s="49"/>
+      <c r="G298" s="49"/>
+      <c r="H298" s="51"/>
+      <c r="I298" s="49"/>
+    </row>
+    <row r="299" spans="1:9">
+      <c r="A299" s="52"/>
+      <c r="B299" s="53"/>
+      <c r="C299" s="54"/>
+      <c r="D299" s="53"/>
+      <c r="E299" s="53"/>
+      <c r="F299" s="56"/>
+      <c r="G299" s="56"/>
+      <c r="H299" s="57"/>
+      <c r="I299" s="53"/>
+    </row>
+    <row r="300" spans="1:9">
+      <c r="A300" s="48"/>
+      <c r="B300" s="49"/>
+      <c r="C300" s="50"/>
+      <c r="D300" s="49"/>
+      <c r="E300" s="49"/>
+      <c r="F300" s="49"/>
+      <c r="G300" s="49"/>
+      <c r="H300" s="51"/>
+      <c r="I300" s="49"/>
+    </row>
+    <row r="301" spans="1:9">
+      <c r="A301" s="52"/>
+      <c r="B301" s="53"/>
+      <c r="C301" s="54"/>
+      <c r="D301" s="53"/>
+      <c r="E301" s="53"/>
+      <c r="F301" s="56"/>
+      <c r="G301" s="56"/>
+      <c r="H301" s="57"/>
+      <c r="I301" s="53"/>
+    </row>
+    <row r="302" spans="1:9">
+      <c r="A302" s="48"/>
+      <c r="B302" s="49"/>
+      <c r="C302" s="50"/>
+      <c r="D302" s="49"/>
+      <c r="E302" s="49"/>
+      <c r="F302" s="49"/>
+      <c r="G302" s="49"/>
+      <c r="H302" s="51"/>
+      <c r="I302" s="49"/>
+    </row>
+    <row r="303" spans="1:9">
+      <c r="A303" s="52"/>
+      <c r="B303" s="53"/>
+      <c r="C303" s="54"/>
+      <c r="D303" s="53"/>
+      <c r="E303" s="53"/>
+      <c r="F303" s="56"/>
+      <c r="G303" s="56"/>
+      <c r="H303" s="57"/>
+      <c r="I303" s="53"/>
+    </row>
+    <row r="304" spans="1:9">
+      <c r="A304" s="48"/>
+      <c r="B304" s="49"/>
+      <c r="C304" s="50"/>
+      <c r="D304" s="49"/>
+      <c r="E304" s="49"/>
+      <c r="F304" s="49"/>
+      <c r="G304" s="49"/>
+      <c r="H304" s="51"/>
+      <c r="I304" s="49"/>
+    </row>
+    <row r="305" spans="1:9">
+      <c r="A305" s="52"/>
+      <c r="B305" s="53"/>
+      <c r="C305" s="54"/>
+      <c r="D305" s="53"/>
+      <c r="E305" s="53"/>
+      <c r="F305" s="56"/>
+      <c r="G305" s="56"/>
+      <c r="H305" s="57"/>
+      <c r="I305" s="53"/>
+    </row>
+    <row r="306" spans="1:9">
+      <c r="A306" s="48"/>
+      <c r="B306" s="49"/>
+      <c r="C306" s="50"/>
+      <c r="D306" s="49"/>
+      <c r="E306" s="49"/>
+      <c r="F306" s="49"/>
+      <c r="G306" s="49"/>
+      <c r="H306" s="51"/>
+      <c r="I306" s="49"/>
+    </row>
+    <row r="307" spans="1:9">
+      <c r="A307" s="52"/>
+      <c r="B307" s="53"/>
+      <c r="C307" s="54"/>
+      <c r="D307" s="53"/>
+      <c r="E307" s="53"/>
+      <c r="F307" s="56"/>
+      <c r="G307" s="56"/>
+      <c r="H307" s="57"/>
+      <c r="I307" s="53"/>
+    </row>
+    <row r="308" spans="1:9">
+      <c r="A308" s="48"/>
+      <c r="B308" s="49"/>
+      <c r="C308" s="50"/>
+      <c r="D308" s="49"/>
+      <c r="E308" s="49"/>
+      <c r="F308" s="49"/>
+      <c r="G308" s="49"/>
+      <c r="H308" s="51"/>
+      <c r="I308" s="49"/>
+    </row>
+    <row r="309" spans="1:9">
+      <c r="A309" s="52"/>
+      <c r="B309" s="53"/>
+      <c r="C309" s="54"/>
+      <c r="D309" s="53"/>
+      <c r="E309" s="53"/>
+      <c r="F309" s="56"/>
+      <c r="G309" s="56"/>
+      <c r="H309" s="57"/>
+      <c r="I309" s="53"/>
+    </row>
+    <row r="310" spans="1:9">
+      <c r="A310" s="48"/>
+      <c r="B310" s="49"/>
+      <c r="C310" s="50"/>
+      <c r="D310" s="49"/>
+      <c r="E310" s="49"/>
+      <c r="F310" s="49"/>
+      <c r="G310" s="49"/>
+      <c r="H310" s="51"/>
+      <c r="I310" s="49"/>
+    </row>
+    <row r="311" spans="1:9">
+      <c r="A311" s="52"/>
+      <c r="B311" s="53"/>
+      <c r="C311" s="54"/>
+      <c r="D311" s="53"/>
+      <c r="E311" s="53"/>
+      <c r="F311" s="56"/>
+      <c r="G311" s="56"/>
+      <c r="H311" s="57"/>
+      <c r="I311" s="53"/>
+    </row>
+    <row r="312" spans="1:9">
+      <c r="A312" s="48"/>
+      <c r="B312" s="49"/>
+      <c r="C312" s="50"/>
+      <c r="D312" s="49"/>
+      <c r="E312" s="49"/>
+      <c r="F312" s="49"/>
+      <c r="G312" s="49"/>
+      <c r="H312" s="51"/>
+      <c r="I312" s="49"/>
+    </row>
+    <row r="313" spans="1:9">
+      <c r="A313" s="52"/>
+      <c r="B313" s="53"/>
+      <c r="C313" s="54"/>
+      <c r="D313" s="53"/>
+      <c r="E313" s="53"/>
+      <c r="F313" s="56"/>
+      <c r="G313" s="56"/>
+      <c r="H313" s="57"/>
+      <c r="I313" s="53"/>
+    </row>
+    <row r="314" spans="1:9">
+      <c r="A314" s="48"/>
+      <c r="B314" s="49"/>
+      <c r="C314" s="50"/>
+      <c r="D314" s="49"/>
+      <c r="E314" s="49"/>
+      <c r="F314" s="49"/>
+      <c r="G314" s="49"/>
+      <c r="H314" s="51"/>
+      <c r="I314" s="49"/>
+    </row>
+    <row r="315" spans="1:9">
+      <c r="A315" s="52"/>
+      <c r="B315" s="53"/>
+      <c r="C315" s="54"/>
+      <c r="D315" s="53"/>
+      <c r="E315" s="53"/>
+      <c r="F315" s="56"/>
+      <c r="G315" s="56"/>
+      <c r="H315" s="57"/>
+      <c r="I315" s="53"/>
+    </row>
+    <row r="316" spans="1:9">
+      <c r="A316" s="48"/>
+      <c r="B316" s="49"/>
+      <c r="C316" s="50"/>
+      <c r="D316" s="49"/>
+      <c r="E316" s="49"/>
+      <c r="F316" s="49"/>
+      <c r="G316" s="49"/>
+      <c r="H316" s="51"/>
+      <c r="I316" s="49"/>
+    </row>
+    <row r="317" spans="1:9">
+      <c r="A317" s="52"/>
+      <c r="B317" s="53"/>
+      <c r="C317" s="54"/>
+      <c r="D317" s="53"/>
+      <c r="E317" s="53"/>
+      <c r="F317" s="56"/>
+      <c r="G317" s="56"/>
+      <c r="H317" s="57"/>
+      <c r="I317" s="53"/>
+    </row>
+    <row r="318" spans="1:9">
+      <c r="A318" s="48"/>
+      <c r="B318" s="49"/>
+      <c r="C318" s="50"/>
+      <c r="D318" s="49"/>
+      <c r="E318" s="49"/>
+      <c r="F318" s="49"/>
+      <c r="G318" s="49"/>
+      <c r="H318" s="51"/>
+      <c r="I318" s="49"/>
+    </row>
+    <row r="319" spans="1:9">
+      <c r="A319" s="52"/>
+      <c r="B319" s="53"/>
+      <c r="C319" s="54"/>
+      <c r="D319" s="53"/>
+      <c r="E319" s="53"/>
+      <c r="F319" s="56"/>
+      <c r="G319" s="56"/>
+      <c r="H319" s="57"/>
+      <c r="I319" s="53"/>
+    </row>
+    <row r="320" spans="1:9">
+      <c r="A320" s="48"/>
+      <c r="B320" s="49"/>
+      <c r="C320" s="50"/>
+      <c r="D320" s="49"/>
+      <c r="E320" s="49"/>
+      <c r="F320" s="49"/>
+      <c r="G320" s="49"/>
+      <c r="H320" s="51"/>
+      <c r="I320" s="49"/>
+    </row>
+    <row r="321" spans="1:9">
+      <c r="A321" s="52"/>
+      <c r="B321" s="53"/>
+      <c r="C321" s="54"/>
+      <c r="D321" s="53"/>
+      <c r="E321" s="53"/>
+      <c r="F321" s="56"/>
+      <c r="G321" s="56"/>
+      <c r="H321" s="57"/>
+      <c r="I321" s="53"/>
+    </row>
+    <row r="322" spans="1:9">
+      <c r="A322" s="48"/>
+      <c r="B322" s="49"/>
+      <c r="C322" s="50"/>
+      <c r="D322" s="49"/>
+      <c r="E322" s="49"/>
+      <c r="F322" s="49"/>
+      <c r="G322" s="49"/>
+      <c r="H322" s="51"/>
+      <c r="I322" s="49"/>
+    </row>
+    <row r="323" spans="1:9">
+      <c r="A323" s="52"/>
+      <c r="B323" s="53"/>
+      <c r="C323" s="54"/>
+      <c r="D323" s="53"/>
+      <c r="E323" s="53"/>
+      <c r="F323" s="56"/>
+      <c r="G323" s="56"/>
+      <c r="H323" s="57"/>
+      <c r="I323" s="53"/>
+    </row>
+    <row r="324" spans="1:9">
+      <c r="A324" s="48"/>
+      <c r="B324" s="49"/>
+      <c r="C324" s="50"/>
+      <c r="D324" s="49"/>
+      <c r="E324" s="49"/>
+      <c r="F324" s="49"/>
+      <c r="G324" s="49"/>
+      <c r="H324" s="51"/>
+      <c r="I324" s="49"/>
+    </row>
+    <row r="325" spans="1:9">
+      <c r="A325" s="52"/>
+      <c r="B325" s="53"/>
+      <c r="C325" s="54"/>
+      <c r="D325" s="53"/>
+      <c r="E325" s="53"/>
+      <c r="F325" s="56"/>
+      <c r="G325" s="56"/>
+      <c r="H325" s="57"/>
+      <c r="I325" s="53"/>
+    </row>
+    <row r="326" spans="1:9">
+      <c r="A326" s="48"/>
+      <c r="B326" s="49"/>
+      <c r="C326" s="50"/>
+      <c r="D326" s="49"/>
+      <c r="E326" s="49"/>
+      <c r="F326" s="49"/>
+      <c r="G326" s="49"/>
+      <c r="H326" s="51"/>
+      <c r="I326" s="49"/>
+    </row>
+    <row r="327" spans="1:9">
+      <c r="A327" s="52"/>
+      <c r="B327" s="53"/>
+      <c r="C327" s="54"/>
+      <c r="D327" s="53"/>
+      <c r="E327" s="53"/>
+      <c r="F327" s="56"/>
+      <c r="G327" s="56"/>
+      <c r="H327" s="57"/>
+      <c r="I327" s="53"/>
+    </row>
+    <row r="328" spans="1:9">
+      <c r="A328" s="48"/>
+      <c r="B328" s="49"/>
+      <c r="C328" s="50"/>
+      <c r="D328" s="49"/>
+      <c r="E328" s="49"/>
+      <c r="F328" s="49"/>
+      <c r="G328" s="49"/>
+      <c r="H328" s="51"/>
+      <c r="I328" s="49"/>
+    </row>
+    <row r="329" spans="1:9">
+      <c r="A329" s="52"/>
+      <c r="B329" s="53"/>
+      <c r="C329" s="54"/>
+      <c r="D329" s="53"/>
+      <c r="E329" s="53"/>
+      <c r="F329" s="56"/>
+      <c r="G329" s="56"/>
+      <c r="H329" s="57"/>
+      <c r="I329" s="53"/>
+    </row>
+    <row r="330" spans="1:9">
+      <c r="A330" s="48"/>
+      <c r="B330" s="49"/>
+      <c r="C330" s="50"/>
+      <c r="D330" s="49"/>
+      <c r="E330" s="49"/>
+      <c r="F330" s="49"/>
+      <c r="G330" s="49"/>
+      <c r="H330" s="51"/>
+      <c r="I330" s="49"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I267" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
@@ -27574,7 +28050,7 @@
         <v>472</v>
       </c>
       <c r="L93" s="66" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="M93" s="66"/>
       <c r="N93" s="63" t="s">
@@ -27710,10 +28186,10 @@
         <v>1450</v>
       </c>
       <c r="F96" s="64">
+        <v>1</v>
+      </c>
+      <c r="G96" s="64">
         <v>0</v>
-      </c>
-      <c r="G96" s="64">
-        <v>1</v>
       </c>
       <c r="H96" s="63">
         <f t="shared" si="4"/>
@@ -27725,16 +28201,18 @@
       </c>
       <c r="J96" s="63">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1250</v>
       </c>
       <c r="K96" s="63">
         <f t="shared" si="6"/>
-        <v>1250</v>
-      </c>
-      <c r="L96" s="63"/>
+        <v>0</v>
+      </c>
+      <c r="L96" s="63" t="s">
+        <v>1200</v>
+      </c>
       <c r="M96" s="63"/>
       <c r="N96" s="63" t="s">
-        <v>678</v>
+        <v>504</v>
       </c>
       <c r="O96" s="63"/>
       <c r="P96" s="63"/>
@@ -29010,7 +29488,7 @@
         <v>3351.6266666666638</v>
       </c>
       <c r="L120" s="63" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="M120" s="63" t="s">
         <v>49</v>
@@ -29020,7 +29498,7 @@
       </c>
       <c r="O120" s="63"/>
       <c r="P120" s="63" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="Q120" s="63"/>
       <c r="R120" s="63"/>
@@ -31100,7 +31578,7 @@
         <v>0</v>
       </c>
       <c r="L147" s="66" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="M147" s="66"/>
       <c r="N147" s="66" t="s">
@@ -33373,7 +33851,7 @@
         <v>0</v>
       </c>
       <c r="L190" s="63" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="M190" s="63"/>
       <c r="N190" s="58" t="s">
@@ -33819,14 +34297,14 @@
         <v>1401</v>
       </c>
       <c r="L199" s="66" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="M199" s="66"/>
       <c r="N199" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P199" s="58" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="S199" s="58"/>
       <c r="T199" s="58"/>
@@ -33972,14 +34450,14 @@
         <v>940</v>
       </c>
       <c r="L202" s="63" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="M202" s="63"/>
       <c r="N202" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="58" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="S202" s="58"/>
       <c r="T202" s="58"/>
@@ -34845,10 +35323,10 @@
         <v>1150</v>
       </c>
       <c r="F220" s="78">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G220" s="78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H220" s="77">
         <f t="shared" si="12"/>
@@ -34860,19 +35338,21 @@
       </c>
       <c r="J220" s="77">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>761</v>
       </c>
       <c r="K220" s="77">
         <f t="shared" si="14"/>
-        <v>4566</v>
-      </c>
-      <c r="L220" s="63"/>
+        <v>3805</v>
+      </c>
+      <c r="L220" s="63" t="s">
+        <v>1205</v>
+      </c>
       <c r="M220" s="63"/>
       <c r="N220" s="58" t="s">
-        <v>678</v>
+        <v>589</v>
       </c>
       <c r="P220" s="58" t="s">
-        <v>1174</v>
+        <v>1206</v>
       </c>
       <c r="S220" s="58"/>
       <c r="T220" s="58"/>
@@ -34881,23 +35361,31 @@
       <c r="A221" s="66" t="s">
         <v>1044</v>
       </c>
-      <c r="B221" s="63"/>
-      <c r="C221" s="63"/>
-      <c r="D221" s="64"/>
-      <c r="E221" s="64"/>
+      <c r="B221" s="63" t="s">
+        <v>1202</v>
+      </c>
+      <c r="C221" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="D221" s="64">
+        <v>870</v>
+      </c>
+      <c r="E221" s="64">
+        <v>1380</v>
+      </c>
       <c r="F221" s="76">
         <v>0</v>
       </c>
       <c r="G221" s="76">
-        <v>-36</v>
+        <v>5</v>
       </c>
       <c r="H221" s="75">
         <f t="shared" si="12"/>
-        <v>-36</v>
+        <v>5</v>
       </c>
       <c r="I221" s="75">
         <f>IF(D221&lt;&gt;"",D221,IFERROR(E221/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
-        <v>0</v>
+        <v>870</v>
       </c>
       <c r="J221" s="75">
         <f t="shared" si="13"/>
@@ -34905,10 +35393,16 @@
       </c>
       <c r="K221" s="75">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>4350</v>
       </c>
       <c r="L221" s="66"/>
       <c r="M221" s="66"/>
+      <c r="N221" s="58" t="s">
+        <v>678</v>
+      </c>
+      <c r="P221" s="58" t="s">
+        <v>1203</v>
+      </c>
       <c r="S221" s="58"/>
       <c r="T221" s="58"/>
     </row>
@@ -39037,15 +39531,15 @@
       </c>
       <c r="B8" s="9">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A8,Purchases!$C:$C),0)</f>
-        <v>250158</v>
+        <v>252430</v>
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>173075</v>
+        <v>173832.33333333334</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>77083</v>
+        <v>78597.666666666657</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -39053,7 +39547,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>77083</v>
+        <v>78597.666666666657</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -39061,7 +39555,7 @@
       </c>
       <c r="H8" s="85">
         <f>F8-G8</f>
-        <v>58779.66</v>
+        <v>60294.32666666666</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -39074,11 +39568,11 @@
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>173075</v>
+        <v>173832.33333333334</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>63392</v>
+        <v>62634.666666666657</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -39086,7 +39580,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>63392</v>
+        <v>62634.666666666657</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -39094,7 +39588,7 @@
       </c>
       <c r="H9" s="86">
         <f>F9-G9</f>
-        <v>21752.67</v>
+        <v>20995.336666666655</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -39107,11 +39601,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>173075</v>
+        <v>173832.33333333334</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-140475</v>
+        <v>-141232.33333333334</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -39119,7 +39613,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-140475</v>
+        <v>-141232.33333333334</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -39127,7 +39621,7 @@
       </c>
       <c r="H10" s="85">
         <f>F10-G10</f>
-        <v>-80532.33</v>
+        <v>-81289.663333333345</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">
@@ -39544,7 +40038,7 @@
       </c>
       <c r="B4" s="9">
         <f>IFERROR(SUMIFS(Sales!$C:$C,Sales!$E:$E,$A4,Sales!$I:$I,"Completed"),0)</f>
-        <v>405060</v>
+        <v>406310</v>
       </c>
       <c r="C4" s="9">
         <f>VLOOKUP($A4,PartnerShares!$A$3:$B$5,2,FALSE())</f>
@@ -39552,11 +40046,11 @@
       </c>
       <c r="D4" s="9">
         <f>Summary!$B$4*C4</f>
-        <v>157436.1476</v>
+        <v>157852.8976</v>
       </c>
       <c r="E4" s="9">
         <f>B4-D4</f>
-        <v>247623.8524</v>
+        <v>248457.1024</v>
       </c>
       <c r="F4" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A4,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39564,7 +40058,7 @@
       </c>
       <c r="G4" s="85">
         <f>E4+F4</f>
-        <v>110313.82639999999</v>
+        <v>111147.07639999999</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="13.5" customHeight="1">
@@ -39581,11 +40075,11 @@
       </c>
       <c r="D5" s="11">
         <f>Summary!$B$4*C5</f>
-        <v>157341.70480000001</v>
+        <v>157758.20480000001</v>
       </c>
       <c r="E5" s="11">
         <f>B5-D5</f>
-        <v>-102717.70480000001</v>
+        <v>-103134.20480000001</v>
       </c>
       <c r="F5" s="11">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A5,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39593,7 +40087,7 @@
       </c>
       <c r="G5" s="86">
         <f>E5+F5</f>
-        <v>-31130.662800000006</v>
+        <v>-31547.162800000006</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="13.5" customHeight="1">
@@ -39610,11 +40104,11 @@
       </c>
       <c r="D6" s="9">
         <f>Summary!$B$4*C6</f>
-        <v>157436.1476</v>
+        <v>157852.8976</v>
       </c>
       <c r="E6" s="9">
         <f>B6-D6</f>
-        <v>-144906.1476</v>
+        <v>-145322.8976</v>
       </c>
       <c r="F6" s="9">
         <f>IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$D$13:$D$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)-IFERROR(SUMIFS(PartnerShares!$E$13:$E$499,PartnerShares!$C$13:$C$499,$A6,PartnerShares!$B$13:$B$499,"Cash"),0)</f>
@@ -39622,7 +40116,7 @@
       </c>
       <c r="G6" s="85">
         <f>E6+F6</f>
-        <v>-79183.163599999985</v>
+        <v>-79599.913599999985</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="13.5" customHeight="1">

</xml_diff>

<commit_message>
7/27 - Purchases, Sales & Returns
</commit_message>
<xml_diff>
--- a/docs/Chiraath-Summary-Jul26.xlsx
+++ b/docs/Chiraath-Summary-Jul26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anooppremachandran/Desktop/CHIRAATH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35D40928-5299-BD44-8298-5D073C89AE0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75A03562-8B86-724C-9AAF-E8969D1DA0F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Notes" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">INVENTORY!$A$1:$T$188</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Purchases!$A$1:$D$32</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$267</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Sales!$A$1:$I$294</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3086" uniqueCount="1211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3094" uniqueCount="1214">
   <si>
     <t>Notes:</t>
   </si>
@@ -3565,9 +3565,6 @@
     <t>Soft Mul Tissue saree Collection</t>
   </si>
   <si>
-    <t>Rust, Purple, Dark Grey, Olive Green</t>
-  </si>
-  <si>
     <t>Mul Tissue saree Collection</t>
   </si>
   <si>
@@ -3633,9 +3630,6 @@
     <t>Sourabhya (XL - 580), Lakshmi - L</t>
   </si>
   <si>
-    <t>CHR-157 2 piece cotton salwar, Banarasi golden yellow blue</t>
-  </si>
-  <si>
     <t>Violet - Ambika, Navy Blue - Simi Upanesh, Light Green - Saraladevi</t>
   </si>
   <si>
@@ -3660,9 +3654,6 @@
     <t>Rose pink, dusty lavender, champagne, chocolate brown, magenta</t>
   </si>
   <si>
-    <t>CHR-182 (Yellow Linen Saree with Lotus, CHR-217 cream/gold with stars and paisley</t>
-  </si>
-  <si>
     <t>Ranju Bank Staff</t>
   </si>
   <si>
@@ -3675,17 +3666,6 @@
     <t>Cream/gold with leaves, cream/gold with flowers</t>
   </si>
   <si>
-    <t xml:space="preserve"> - CHR-212 - Purple
- - CHR-215 - green and maroon with golden design
- - CHR-198 - light blue</t>
-  </si>
-  <si>
-    <t>Teena mathew - Paeach, Shylaja - light blue</t>
-  </si>
-  <si>
-    <t>pink, light green</t>
-  </si>
-  <si>
     <t>Shylaja - Green and maroon with golden design</t>
   </si>
   <si>
@@ -3698,8 +3678,34 @@
     <t>Yellow/Orange(4), Green, Blue</t>
   </si>
   <si>
-    <t xml:space="preserve"> - CHR-212 - Red
- - CHR-214 - Yellow/Blue Chanderi Silk</t>
+    <t>CHR-111 white cotton salwar, Banarasi golden yellow blue</t>
+  </si>
+  <si>
+    <t>CHR-212 - Red, CHR-214 - Yellow/Blue Chanderi Silk, CHR-95 Chinon Silk</t>
+  </si>
+  <si>
+    <t>CHR-182 (Yellow Linen Saree with Lotus, CHR-217 cream/gold with stars and paisley &amp; cream/gold with flowers</t>
+  </si>
+  <si>
+    <t>Teena mathew - Paeach</t>
+  </si>
+  <si>
+    <t>pink, light green, light blue</t>
+  </si>
+  <si>
+    <t>CHR-212 - Purple, CHR-215 - Green and Maroon with golden design, CHR-172 - Kathakali</t>
+  </si>
+  <si>
+    <t>Niroop</t>
+  </si>
+  <si>
+    <t>CHR-192 Small temple design</t>
+  </si>
+  <si>
+    <t>Rust, Purple, Olive Green</t>
+  </si>
+  <si>
+    <t>Dark Grey - returned</t>
   </si>
 </sst>
 </file>
@@ -4582,7 +4588,7 @@
                   <c:v>297</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>95</c:v>
+                  <c:v>96</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>5</c:v>
@@ -4682,10 +4688,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>178</c:v>
+                  <c:v>176</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>53</c:v>
+                  <c:v>52</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>3</c:v>
@@ -5012,10 +5018,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>56434</c:v>
+                  <c:v>55458</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>136202.19666666666</c:v>
+                  <c:v>133666.19666666666</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>1062</c:v>
@@ -5348,7 +5354,7 @@
                   <c:v>99043</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>67350</c:v>
+                  <c:v>102200</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5508,7 +5514,7 @@
                   <c:v>72885</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>59195</c:v>
+                  <c:v>62696</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -5948,7 +5954,7 @@
                   <c:v>-26158</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-8155</c:v>
+                  <c:v>-39504</c:v>
                 </c:pt>
                 <c:pt idx="7">
                   <c:v>0</c:v>
@@ -6412,10 +6418,10 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="2"/>
                 <c:pt idx="0">
-                  <c:v>397</c:v>
+                  <c:v>398</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>39</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7587,7 +7593,7 @@
       </c>
       <c r="B3" s="8">
         <f>SUM(Purchases!C:C)</f>
-        <v>521497</v>
+        <v>556347</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>42</v>
@@ -7619,7 +7625,7 @@
       </c>
       <c r="B5" s="12">
         <f>SUM(Sales!C:C)</f>
-        <v>487693</v>
+        <v>491194</v>
       </c>
       <c r="E5" s="11" t="str">
         <f>PartnerShares!A4</f>
@@ -7636,7 +7642,7 @@
       </c>
       <c r="B6" s="10">
         <f>B4-B3</f>
-        <v>-48033</v>
+        <v>-82883</v>
       </c>
       <c r="E6" s="9" t="str">
         <f>PartnerShares!A5</f>
@@ -7671,7 +7677,7 @@
       </c>
       <c r="B10" s="13">
         <f>PartnerShares!H8</f>
-        <v>60294.32666666666</v>
+        <v>48677.66</v>
       </c>
       <c r="C10" s="9"/>
     </row>
@@ -7681,7 +7687,7 @@
       </c>
       <c r="B11" s="14">
         <f>PartnerShares!H9</f>
-        <v>20995.336666666655</v>
+        <v>44228.67</v>
       </c>
       <c r="C11" s="11"/>
     </row>
@@ -7691,7 +7697,7 @@
       </c>
       <c r="B12" s="13">
         <f>PartnerShares!H10</f>
-        <v>-81289.663333333345</v>
+        <v>-92906.33</v>
       </c>
       <c r="C12" s="9"/>
     </row>
@@ -7734,11 +7740,11 @@
       </c>
       <c r="C18" s="10">
         <f>PartnerShares!C8</f>
-        <v>173832.33333333334</v>
+        <v>185449</v>
       </c>
       <c r="D18" s="10">
         <f>PartnerShares!D8</f>
-        <v>78597.666666666657</v>
+        <v>66981</v>
       </c>
       <c r="E18" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A18,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7746,11 +7752,11 @@
       </c>
       <c r="F18" s="13">
         <f>D18-E18</f>
-        <v>60294.32666666666</v>
+        <v>48677.66</v>
       </c>
       <c r="G18" s="16" t="str">
         <f>IF(ROUND(F18,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F18),"#,##0"),IF(ROUND(F18,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F18),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹60,294</v>
+        <v>Receive ₹48,678</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="13.5" customHeight="1">
@@ -7760,15 +7766,15 @@
       </c>
       <c r="B19" s="12">
         <f>PartnerShares!B9</f>
-        <v>236467</v>
+        <v>271317</v>
       </c>
       <c r="C19" s="12">
         <f>PartnerShares!C9</f>
-        <v>173832.33333333334</v>
+        <v>185449</v>
       </c>
       <c r="D19" s="12">
         <f>PartnerShares!D9</f>
-        <v>62634.666666666657</v>
+        <v>85868</v>
       </c>
       <c r="E19" s="12">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A19,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7776,11 +7782,11 @@
       </c>
       <c r="F19" s="14">
         <f>D19-E19</f>
-        <v>20995.336666666655</v>
+        <v>44228.67</v>
       </c>
       <c r="G19" s="17" t="str">
         <f>IF(ROUND(F19,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F19),"#,##0"),IF(ROUND(F19,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F19),"#,##0"),"✓ Settled"))</f>
-        <v>Receive ₹20,995</v>
+        <v>Receive ₹44,229</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="13.5" customHeight="1">
@@ -7794,11 +7800,11 @@
       </c>
       <c r="C20" s="10">
         <f>PartnerShares!C10</f>
-        <v>173832.33333333334</v>
+        <v>185449</v>
       </c>
       <c r="D20" s="10">
         <f>PartnerShares!D10</f>
-        <v>-141232.33333333334</v>
+        <v>-152849</v>
       </c>
       <c r="E20" s="10">
         <f>IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$D$14:$D$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)-IFERROR(SUMIFS(PartnerShares!$E$14:$E$500,PartnerShares!$C$14:$C$500,$A20,PartnerShares!$B$14:$B$500,"Contribution"),0)</f>
@@ -7806,11 +7812,11 @@
       </c>
       <c r="F20" s="13">
         <f>D20-E20</f>
-        <v>-81289.663333333345</v>
+        <v>-92906.33</v>
       </c>
       <c r="G20" s="17" t="str">
         <f>IF(ROUND(F20,0)&gt;0,"Receive ₹"&amp;TEXT(ABS(F20),"#,##0"),IF(ROUND(F20,0)&lt;0,"Pay ₹"&amp;TEXT(ABS(F20),"#,##0"),"✓ Settled"))</f>
-        <v>Pay ₹81,290</v>
+        <v>Pay ₹92,906</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="15.75" customHeight="1">
@@ -8049,7 +8055,7 @@
       </c>
       <c r="B5" s="21">
         <f>Summary!B3</f>
-        <v>521497</v>
+        <v>556347</v>
       </c>
       <c r="D5" s="19" t="s">
         <v>69</v>
@@ -8065,14 +8071,14 @@
       </c>
       <c r="B6" s="21">
         <f>Summary!B6</f>
-        <v>-48033</v>
+        <v>-82883</v>
       </c>
       <c r="D6" s="19" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="21">
         <f>SUMIFS(INVENTORY!K:K, INVENTORY!N:N, "&lt;&gt;Sold Out")</f>
-        <v>184077.39666666667</v>
+        <v>180565.39666666667</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1">
@@ -8124,7 +8130,7 @@
       </c>
       <c r="G10" s="21">
         <f>SUM(INVENTORY!F:F)</f>
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="15" customHeight="1">
@@ -8148,7 +8154,7 @@
       </c>
       <c r="G11" s="27">
         <f>SUM(INVENTORY!G:G)</f>
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="15" customHeight="1">
@@ -8225,15 +8231,15 @@
       </c>
       <c r="B16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Purchases!$A$2:$A$998,"MMM")=$A16)*(YEAR(Purchases!$A$2:$A$998)=$B$7)*Purchases!$C$2:$C$998),0)</f>
-        <v>67350</v>
+        <v>102200</v>
       </c>
       <c r="C16" s="21">
         <f>IFERROR(SUMPRODUCT((TEXT(Sales!$A$2:$A$994,"MMM")=$A16)*(YEAR(Sales!$A$2:$A$994)=$B$7)*Sales!$C$2:$C$994),0)</f>
-        <v>59195</v>
+        <v>62696</v>
       </c>
       <c r="D16" s="21">
         <f t="shared" si="0"/>
-        <v>-8155</v>
+        <v>-39504</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="15" customHeight="1">
@@ -8348,14 +8354,14 @@
       </c>
       <c r="H47" s="30">
         <f>SUMIF(INVENTORY!C:C, F47, INVENTORY!G:G)</f>
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="J47" s="30" t="s">
         <v>96</v>
       </c>
       <c r="K47" s="31">
         <f t="array" ref="K47">SUMPRODUCT((INVENTORY!$C$2:$C$477=J47)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>56434</v>
+        <v>55458</v>
       </c>
     </row>
     <row r="48" spans="6:11" ht="15" customHeight="1">
@@ -8364,18 +8370,18 @@
       </c>
       <c r="G48" s="30">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!F:F)</f>
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H48" s="30">
         <f>SUMIF(INVENTORY!C:C, F48, INVENTORY!G:G)</f>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J48" s="30" t="s">
         <v>95</v>
       </c>
       <c r="K48" s="31">
         <f t="array" ref="K48">SUMPRODUCT((INVENTORY!$C$2:$C$477=J48)*(INVENTORY!$D$2:$D$477)*(INVENTORY!$G$2:$G$477))</f>
-        <v>136202.19666666666</v>
+        <v>133666.19666666666</v>
       </c>
     </row>
     <row r="49" spans="5:12" ht="15" customHeight="1">
@@ -9920,10 +9926,18 @@
       </c>
     </row>
     <row r="104" spans="1:4" ht="15" customHeight="1">
-      <c r="A104" s="35"/>
-      <c r="B104" s="36"/>
-      <c r="C104" s="37"/>
-      <c r="D104" s="36"/>
+      <c r="A104" s="35">
+        <v>46231</v>
+      </c>
+      <c r="B104" s="36" t="s">
+        <v>50</v>
+      </c>
+      <c r="C104" s="37">
+        <v>34850</v>
+      </c>
+      <c r="D104" s="36" t="s">
+        <v>118</v>
+      </c>
     </row>
     <row r="105" spans="1:4" ht="15" customHeight="1">
       <c r="A105" s="38"/>
@@ -18446,7 +18460,7 @@
       <c r="F261" s="56"/>
       <c r="G261" s="56"/>
       <c r="H261" s="57" t="s">
-        <v>1189</v>
+        <v>1204</v>
       </c>
       <c r="I261" s="53" t="s">
         <v>148</v>
@@ -18953,7 +18967,7 @@
         <v>46220</v>
       </c>
       <c r="B282" s="49" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="C282" s="50">
         <v>1500</v>
@@ -18967,7 +18981,7 @@
       <c r="F282" s="49"/>
       <c r="G282" s="49"/>
       <c r="H282" s="51" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="I282" s="49" t="s">
         <v>148</v>
@@ -18978,7 +18992,7 @@
         <v>46221</v>
       </c>
       <c r="B283" s="53" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C283" s="54">
         <v>1100</v>
@@ -18992,7 +19006,7 @@
       <c r="F283" s="56"/>
       <c r="G283" s="56"/>
       <c r="H283" s="57" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="I283" s="53" t="s">
         <v>148</v>
@@ -19003,7 +19017,7 @@
         <v>46222</v>
       </c>
       <c r="B284" s="49" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C284" s="50">
         <v>850</v>
@@ -19017,7 +19031,7 @@
       <c r="F284" s="49"/>
       <c r="G284" s="49"/>
       <c r="H284" s="51" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="I284" s="49" t="s">
         <v>148</v>
@@ -19028,7 +19042,7 @@
         <v>46222</v>
       </c>
       <c r="B285" s="53" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="C285" s="54">
         <v>1250</v>
@@ -19042,7 +19056,7 @@
       <c r="F285" s="56"/>
       <c r="G285" s="56"/>
       <c r="H285" s="57" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="I285" s="53" t="s">
         <v>148</v>
@@ -19053,7 +19067,7 @@
         <v>46222</v>
       </c>
       <c r="B286" s="49" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="C286" s="50">
         <v>700</v>
@@ -19078,7 +19092,7 @@
         <v>46222</v>
       </c>
       <c r="B287" s="53" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="C287" s="54">
         <v>699</v>
@@ -19103,7 +19117,7 @@
         <v>46223</v>
       </c>
       <c r="B288" s="49" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="C288" s="50">
         <v>1380</v>
@@ -19117,7 +19131,7 @@
       <c r="F288" s="49"/>
       <c r="G288" s="49"/>
       <c r="H288" s="51" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="I288" s="49" t="s">
         <v>148</v>
@@ -19128,7 +19142,7 @@
         <v>46224</v>
       </c>
       <c r="B289" s="53" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C289" s="54">
         <v>1380</v>
@@ -19142,7 +19156,7 @@
       <c r="F289" s="56"/>
       <c r="G289" s="56"/>
       <c r="H289" s="57" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="I289" s="53" t="s">
         <v>148</v>
@@ -19153,7 +19167,7 @@
         <v>46224</v>
       </c>
       <c r="B290" s="49" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="C290" s="50">
         <v>1380</v>
@@ -19167,7 +19181,7 @@
       <c r="F290" s="49"/>
       <c r="G290" s="49"/>
       <c r="H290" s="51" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="I290" s="49" t="s">
         <v>148</v>
@@ -19192,7 +19206,7 @@
       <c r="F291" s="49"/>
       <c r="G291" s="49"/>
       <c r="H291" s="51" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="I291" s="49" t="s">
         <v>148</v>
@@ -19203,23 +19217,23 @@
         <v>46229</v>
       </c>
       <c r="B292" s="53" t="s">
-        <v>1199</v>
+        <v>1196</v>
       </c>
       <c r="C292" s="54">
-        <v>1300</v>
+        <v>1900</v>
       </c>
       <c r="D292" s="53"/>
       <c r="E292" s="53"/>
       <c r="F292" s="56"/>
       <c r="G292" s="56"/>
       <c r="H292" s="57" t="s">
-        <v>1198</v>
+        <v>1206</v>
       </c>
       <c r="I292" s="53" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="42">
+    <row r="293" spans="1:9" ht="28">
       <c r="A293" s="48">
         <v>46229</v>
       </c>
@@ -19227,14 +19241,14 @@
         <v>293</v>
       </c>
       <c r="C293" s="50">
-        <v>2599</v>
+        <v>3000</v>
       </c>
       <c r="D293" s="49"/>
       <c r="E293" s="49"/>
       <c r="F293" s="49"/>
       <c r="G293" s="49"/>
       <c r="H293" s="51" t="s">
-        <v>1203</v>
+        <v>1209</v>
       </c>
       <c r="I293" s="49" t="s">
         <v>356</v>
@@ -19248,29 +19262,39 @@
         <v>1109</v>
       </c>
       <c r="C294" s="54">
-        <v>2300</v>
+        <v>3250</v>
       </c>
       <c r="D294" s="53"/>
       <c r="E294" s="53"/>
       <c r="F294" s="56"/>
       <c r="G294" s="56"/>
       <c r="H294" s="57" t="s">
-        <v>1210</v>
+        <v>1205</v>
       </c>
       <c r="I294" s="53" t="s">
         <v>356</v>
       </c>
     </row>
-    <row r="295" spans="1:9">
-      <c r="A295" s="48"/>
-      <c r="B295" s="49"/>
-      <c r="C295" s="50"/>
+    <row r="295" spans="1:9" ht="14">
+      <c r="A295" s="48">
+        <v>46229</v>
+      </c>
+      <c r="B295" s="49" t="s">
+        <v>1210</v>
+      </c>
+      <c r="C295" s="50">
+        <v>1550</v>
+      </c>
       <c r="D295" s="49"/>
       <c r="E295" s="49"/>
       <c r="F295" s="49"/>
       <c r="G295" s="49"/>
-      <c r="H295" s="51"/>
-      <c r="I295" s="49"/>
+      <c r="H295" s="51" t="s">
+        <v>1211</v>
+      </c>
+      <c r="I295" s="49" t="s">
+        <v>356</v>
+      </c>
     </row>
     <row r="296" spans="1:9">
       <c r="A296" s="52"/>
@@ -19647,7 +19671,7 @@
       <c r="I329" s="49"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I267" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:I294" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G1258" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"Ordered,Pending,Completed,Cancelled"</formula1>
@@ -28074,7 +28098,7 @@
         <v>472</v>
       </c>
       <c r="L93" s="66" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="M93" s="66"/>
       <c r="N93" s="63" t="s">
@@ -28210,10 +28234,10 @@
         <v>1450</v>
       </c>
       <c r="F96" s="64">
+        <v>1</v>
+      </c>
+      <c r="G96" s="64">
         <v>0</v>
-      </c>
-      <c r="G96" s="64">
-        <v>1</v>
       </c>
       <c r="H96" s="63">
         <f t="shared" si="4"/>
@@ -28225,16 +28249,18 @@
       </c>
       <c r="J96" s="63">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1250</v>
       </c>
       <c r="K96" s="63">
         <f t="shared" si="6"/>
-        <v>1250</v>
-      </c>
-      <c r="L96" s="63"/>
+        <v>0</v>
+      </c>
+      <c r="L96" s="63" t="s">
+        <v>1109</v>
+      </c>
       <c r="M96" s="63"/>
       <c r="N96" s="63" t="s">
-        <v>678</v>
+        <v>504</v>
       </c>
       <c r="O96" s="63"/>
       <c r="P96" s="63"/>
@@ -29068,10 +29094,10 @@
         <v>1600</v>
       </c>
       <c r="F112" s="64">
+        <v>1</v>
+      </c>
+      <c r="G112" s="64">
         <v>0</v>
-      </c>
-      <c r="G112" s="64">
-        <v>1</v>
       </c>
       <c r="H112" s="63">
         <f t="shared" si="7"/>
@@ -29083,16 +29109,18 @@
       </c>
       <c r="J112" s="63">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>976</v>
       </c>
       <c r="K112" s="63">
         <f t="shared" si="6"/>
-        <v>976</v>
-      </c>
-      <c r="L112" s="63"/>
+        <v>0</v>
+      </c>
+      <c r="L112" s="63" t="s">
+        <v>1109</v>
+      </c>
       <c r="M112" s="63"/>
       <c r="N112" s="63" t="s">
-        <v>678</v>
+        <v>504</v>
       </c>
       <c r="O112" s="63" t="s">
         <v>207</v>
@@ -29510,7 +29538,7 @@
         <v>3351.6266666666638</v>
       </c>
       <c r="L120" s="63" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="M120" s="63" t="s">
         <v>49</v>
@@ -29520,7 +29548,7 @@
       </c>
       <c r="O120" s="63"/>
       <c r="P120" s="63" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="Q120" s="63"/>
       <c r="R120" s="63"/>
@@ -31600,7 +31628,7 @@
         <v>0</v>
       </c>
       <c r="L147" s="66" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="M147" s="66"/>
       <c r="N147" s="66" t="s">
@@ -33511,7 +33539,7 @@
         <v>1676</v>
       </c>
       <c r="L183" s="66" t="s">
-        <v>1200</v>
+        <v>1197</v>
       </c>
       <c r="M183" s="66"/>
       <c r="N183" s="66" t="s">
@@ -33873,7 +33901,7 @@
         <v>0</v>
       </c>
       <c r="L190" s="63" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="M190" s="63"/>
       <c r="N190" s="58" t="s">
@@ -34297,10 +34325,10 @@
         <v>850</v>
       </c>
       <c r="F199" s="76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G199" s="76">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H199" s="75">
         <f t="shared" si="12"/>
@@ -34312,21 +34340,21 @@
       </c>
       <c r="J199" s="75">
         <f t="shared" si="13"/>
-        <v>934</v>
+        <v>467</v>
       </c>
       <c r="K199" s="75">
         <f t="shared" si="14"/>
-        <v>934</v>
+        <v>1401</v>
       </c>
       <c r="L199" s="66" t="s">
-        <v>1204</v>
+        <v>1207</v>
       </c>
       <c r="M199" s="66"/>
       <c r="N199" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P199" s="58" t="s">
-        <v>1205</v>
+        <v>1208</v>
       </c>
       <c r="S199" s="58"/>
       <c r="T199" s="58"/>
@@ -34472,14 +34500,14 @@
         <v>940</v>
       </c>
       <c r="L202" s="63" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="M202" s="63"/>
       <c r="N202" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P202" s="58" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="S202" s="58"/>
       <c r="T202" s="58"/>
@@ -35022,14 +35050,14 @@
         <v>3330</v>
       </c>
       <c r="L213" s="66" t="s">
-        <v>1208</v>
+        <v>1202</v>
       </c>
       <c r="M213" s="66"/>
       <c r="N213" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P213" s="58" t="s">
-        <v>1209</v>
+        <v>1203</v>
       </c>
       <c r="S213" s="58"/>
       <c r="T213" s="58"/>
@@ -35103,11 +35131,11 @@
         <v>1</v>
       </c>
       <c r="G215" s="76">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H215" s="75">
         <f t="shared" si="12"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I215" s="75">
         <f>IF(D215&lt;&gt;"",D215,IFERROR(E215/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -35119,7 +35147,7 @@
       </c>
       <c r="K215" s="75">
         <f t="shared" si="14"/>
-        <v>4960</v>
+        <v>3968</v>
       </c>
       <c r="L215" s="66" t="s">
         <v>1109</v>
@@ -35173,14 +35201,14 @@
         <v>2880</v>
       </c>
       <c r="L216" s="63" t="s">
-        <v>1206</v>
+        <v>1200</v>
       </c>
       <c r="M216" s="63"/>
       <c r="N216" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P216" s="58" t="s">
-        <v>1207</v>
+        <v>1201</v>
       </c>
       <c r="S216" s="58"/>
       <c r="T216" s="58"/>
@@ -35273,14 +35301,14 @@
         <v>828</v>
       </c>
       <c r="L218" s="63" t="s">
-        <v>1201</v>
+        <v>1198</v>
       </c>
       <c r="M218" s="63"/>
       <c r="N218" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P218" s="58" t="s">
-        <v>1202</v>
+        <v>1199</v>
       </c>
       <c r="S218" s="58"/>
       <c r="T218" s="58"/>
@@ -35305,11 +35333,11 @@
         <v>0</v>
       </c>
       <c r="G219" s="76">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H219" s="75">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I219" s="75">
         <f>IF(D219&lt;&gt;"",D219,IFERROR(E219/(IFERROR(SUM(Sales!C:C),0))*(IFERROR(SUM(Purchases!C:C),0)),0))</f>
@@ -35321,15 +35349,17 @@
       </c>
       <c r="K219" s="75">
         <f t="shared" si="14"/>
-        <v>3044</v>
-      </c>
-      <c r="L219" s="66"/>
+        <v>2283</v>
+      </c>
+      <c r="L219" s="66" t="s">
+        <v>1213</v>
+      </c>
       <c r="M219" s="66"/>
       <c r="N219" s="58" t="s">
         <v>678</v>
       </c>
       <c r="P219" s="58" t="s">
-        <v>1167</v>
+        <v>1212</v>
       </c>
       <c r="S219" s="58"/>
       <c r="T219" s="58"/>
@@ -35339,7 +35369,7 @@
         <v>1043</v>
       </c>
       <c r="B220" s="66" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="C220" s="66" t="s">
         <v>95</v>
@@ -35373,14 +35403,14 @@
         <v>3805</v>
       </c>
       <c r="L220" s="63" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="M220" s="63"/>
       <c r="N220" s="58" t="s">
         <v>589</v>
       </c>
       <c r="P220" s="58" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="S220" s="58"/>
       <c r="T220" s="58"/>
@@ -35390,7 +35420,7 @@
         <v>1044</v>
       </c>
       <c r="B221" s="63" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="C221" s="63" t="s">
         <v>95</v>
@@ -35429,7 +35459,7 @@
         <v>678</v>
       </c>
       <c r="P221" s="58" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="S221" s="58"/>
       <c r="T221" s="58"/>
@@ -39563,11 +39593,11 @@
       </c>
       <c r="C8" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>173832.33333333334</v>
+        <v>185449</v>
       </c>
       <c r="D8" s="9">
         <f>B8-C8</f>
-        <v>78597.666666666657</v>
+        <v>66981</v>
       </c>
       <c r="E8" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A8,$A$3:$B$5,2,FALSE()),0)</f>
@@ -39575,7 +39605,7 @@
       </c>
       <c r="F8" s="9">
         <f>D8+E8</f>
-        <v>78597.666666666657</v>
+        <v>66981</v>
       </c>
       <c r="G8" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A8,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A8,$B$13:$B$499,"Profit"),0)</f>
@@ -39583,7 +39613,7 @@
       </c>
       <c r="H8" s="85">
         <f>F8-G8</f>
-        <v>60294.32666666666</v>
+        <v>48677.66</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="13.5" customHeight="1">
@@ -39592,15 +39622,15 @@
       </c>
       <c r="B9" s="11">
         <f>IFERROR(SUMIF(Purchases!$B:$B,$A9,Purchases!$C:$C),0)</f>
-        <v>236467</v>
+        <v>271317</v>
       </c>
       <c r="C9" s="11">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>173832.33333333334</v>
+        <v>185449</v>
       </c>
       <c r="D9" s="11">
         <f>B9-C9</f>
-        <v>62634.666666666657</v>
+        <v>85868</v>
       </c>
       <c r="E9" s="11">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A9,$A$3:$B$5,2,FALSE()),0)</f>
@@ -39608,7 +39638,7 @@
       </c>
       <c r="F9" s="11">
         <f>D9+E9</f>
-        <v>62634.666666666657</v>
+        <v>85868</v>
       </c>
       <c r="G9" s="11">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A9,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A9,$B$13:$B$499,"Profit"),0)</f>
@@ -39616,7 +39646,7 @@
       </c>
       <c r="H9" s="86">
         <f>F9-G9</f>
-        <v>20995.336666666655</v>
+        <v>44228.67</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="13.5" customHeight="1">
@@ -39629,11 +39659,11 @@
       </c>
       <c r="C10" s="9">
         <f>SUM($B$8:$B$10)/3</f>
-        <v>173832.33333333334</v>
+        <v>185449</v>
       </c>
       <c r="D10" s="9">
         <f>B10-C10</f>
-        <v>-141232.33333333334</v>
+        <v>-152849</v>
       </c>
       <c r="E10" s="9">
         <f>IF(Summary!$B$6&gt;0, Summary!$B$6*VLOOKUP($A10,$A$3:$B$5,2,FALSE()),0)</f>
@@ -39641,7 +39671,7 @@
       </c>
       <c r="F10" s="9">
         <f>D10+E10</f>
-        <v>-141232.33333333334</v>
+        <v>-152849</v>
       </c>
       <c r="G10" s="9">
         <f>IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Contribution"),0)+IFERROR(SUMIFS($E$13:$E$499,$D$13:$D$499,$A10,$B$13:$B$499,"Profit"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Contribution"),0)-IFERROR(SUMIFS($E$13:$E$499,$C$13:$C$499,$A10,$B$13:$B$499,"Profit"),0)</f>
@@ -39649,7 +39679,7 @@
       </c>
       <c r="H10" s="85">
         <f>F10-G10</f>
-        <v>-81289.663333333345</v>
+        <v>-92906.33</v>
       </c>
     </row>
     <row r="12" spans="1:8" s="87" customFormat="1" ht="15.75" customHeight="1">

</xml_diff>